<commit_message>
📊 Daily Chinese DB update: 2026-05-29 | 131/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5492,6 +5492,1134 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>CHI-20260529-001</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>家长群炸了</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>jiāzhǎng qún zhà le</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>학부모 단체 채팅방이 난리가 났다 (폭발했다)</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>家长群炸了！毕业生100%进世界前50！就读这所学...</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>老师一宣布放假通知，家长群里立刻就炸了，大家都在讨论出行计划。</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>CHI-20260529-002</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>社保</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Noun (Colloquialism/Abbreviation)</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>shèbǎo</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>사회 보험</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>无社保、无合同，工亡赔偿找谁要？</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>新入职的员工，公司都会帮忙办理社保和公积金。</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>CHI-20260529-003</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>维权</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Separable Verb</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>wéiquán</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>권리를 옹호하다; 권리를 지키다</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>在工亡赔偿维权中，最让家属绝望的，莫过于“无社保、无合同”...</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>消费者在购买商品时，如果遇到质量问题，一定要学会维权。</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>CHI-20260529-004</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>失联跑路</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Colloquialism (Verb Phrase)</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>shīlián pǎolù</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>연락이 끊기고 도주하다 (책임을 회피하기 위해)</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>...单位直接否认劳动关系，拒绝支付任何赔偿，甚至失联跑路。</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>那家健身房突然关门，老板也失联跑路了，很多会员的钱都打了水漂。</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>CHI-20260529-005</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>大咖</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Colloquialism (Noun)</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>dàkā</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>거물; 전문가; 유명 인사</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>大咖说丨尹后庆：在教育家精神指引下，办好学校的价值...</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>这次行业峰会邀请了很多国内外的大咖来分享经验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>CHI-20260529-006</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>狂妄自大</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Idiom</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>kuáng wàng zì dà</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>오만방자하다; 거만하다</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>班主任怒斥狂妄自大...</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>他总是觉得自己比别人强，有点狂妄自大。</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>CHI-20260529-007</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>贯彻落实</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Verb phrase</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>guàn chè luò shí</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>철저히 이행하다; 관철시키다</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>要深入贯彻落实习近平总书记在雄安新区考察时的重要讲话精神...</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>会议强调，要将新政策精神贯彻落实到每个部门。</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>CHI-20260529-008</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>提速提质</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>tí sù tí zhì</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>속도를 높이고 품질을 향상시키다</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>推动北京地区高校向雄安疏解和承接工作提速提质...</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>为了应对市场变化，我们必须在产品研发上提速提质。</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>CHI-20260529-009</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>成绩出炉</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>chéng jì chū lú</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>성적이 발표되다; 결과가 나오다</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>高考成绩出炉，普通大学都没有他的名字...</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>经过一个月的等待，项目最终评估成绩终于出炉了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>CHI-20260529-010</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>一眼识破</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>yī yǎn shí pò</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>한눈에 간파하다, 한눈에 알아채다</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>法官一眼识破：假的！</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>经理一眼识破了他的谎言，让他非常尴尬。</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>CHI-20260529-011</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>拖欠</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>tuō qiàn</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>체납하다, 밀리다 (빚, 요금 등)</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>要求支付拖欠半年的租金</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>如果你继续拖欠房租，房东可能会采取法律行动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>CHI-20260529-012</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>刷屏</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Separable Verb / Colloquialism</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>shuā píng</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>(SNS 등에서) 화면을 도배하다, (정보가) 쇄도하다, (인터넷에서) 화제가 되다</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>留学圈被一所“年轻”的美高刷屏了</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>昨晚那部电影太火了，我的朋友圈都被刷屏了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>CHI-20260529-013</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>小升初</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Colloquialism (Abbreviation)</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>xiǎo shēng chū</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>초등학교에서 중학교로 진학</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>小升初5月22日报名！</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>很多家长为了孩子的小升初，提前几年就开始准备了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>CHI-20260529-014</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>全员开挂</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>quán yuán kāi guà</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>전원 (게임에서) 치트키를 쓰다; 전원이 엄청난 실력을 발휘하다</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>全员开挂：100%获得美国前30大学录取</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>我们团队这次项目表现太出色了，简直是全员开挂！</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>CHI-20260529-015</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>十年磨一剑</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Idiom</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>shí nián mó yī jiàn</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>끈기 있는 노력으로 실력을 연마하다; 오랜 시간 공들여 준비하다</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>十年磨一剑！神仙学校给你稳稳的幸福.</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>我们的团队为了这个项目十年磨一剑，终于取得了突破性进展。</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>CHI-20260529-016</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>变废为宝</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Idiom</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>biànfèiwéibǎo</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>폐품을 보물로 만들다; 재활용하다</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>它就藏在变废为宝的巧思里</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>公司鼓励员工将旧文件变废为宝，制作成创意办公用品。</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>CHI-20260529-017</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>打卡</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>dǎkǎ</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>출근/퇴근 기록을 남기다; (장소에) 방문 인증하다</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>旅客纷纷来打卡.</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>每天早上九点前，我都要在公司系统上打卡。</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>CHI-20260529-018</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>告别</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Separable Verb</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>gàobié</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>작별하다; 떠나다</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>老列车在逐渐“告别”</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>他决定告别大城市的生活，回到家乡发展。</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>CHI-20260529-019</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>解锁</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>jiěsuǒ</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>잠금을 해제하다; (새로운 가능성 등을) 발견하다/드러내다</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>解锁亲子环保新场景</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>这款新软件可以帮助我们解锁更多工作效率的潜力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>CHI-20260529-020</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>融入</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>róngrù</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>~에 녹아들다, ~에 융합되다, ~에 스며들다</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>通讯｜融入街区的“环保时尚场”</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>我们公司正在努力让新员工尽快融入团队。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>CHI-20260529-021</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>转发</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Separable Verb</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>zhuǎnfā</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>(메시지, 게시물 등을) 전달하다, 공유하다, 포워딩하다</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>获外交部发言人转发</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>请大家把这个通知转发到各个部门群里。</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>CHI-20260529-022</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>吐槽</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>tǔcáo</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>불평하다, 투덜거리다, 하소연하다 (속어)</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>网友吐槽</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>昨天会议太长了，好多同事都在私下吐槽。</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>CHI-20260529-023</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>没有印象</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Verb Phrase</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>méiyǒu yìngxiàng</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>인상이 없다, 기억나지 않다</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>却始终没有印象</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>我对那个新来的实习生没什么印象，他好像不太爱说话。</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>CHI-20260529-024</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>扫码</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Separable Verb</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>sǎomǎ</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>(QR 코드를) 스캔하다</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>为获取密码“扫码添加</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>吃饭前记得扫码点餐，方便又快捷。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-05-29 | 136/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I132"/>
+  <dimension ref="A1:I137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6620,6 +6620,241 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>CHI-20260529-025</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>召开</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>zhàokāi</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>(회의 등을) 개최하다, 열다</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>江华工商业联合会（总商会）第十四次会员代表大会召开.</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>经理决定下周一召开一次全体员工会议。</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>CHI-20260529-026</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>初心</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Noun</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>chūxīn</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>초심, 처음의 마음</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>致敬劳动者｜出租车司机刘自立：用行动诠释劳模初心.</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>无论遇到什么困难，我们都不能忘记自己的初心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>CHI-20260529-027</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>冲刺</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Verb/Noun</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>chōngcì</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>(결승점을 향해) 전력 질주하다; (목표 달성을 위해) 마지막 박차를 가하다</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>后来到了高考冲刺前100天，他又“突然消失”不来参加。</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>离项目截止日期还有一周，我们必须冲刺了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>CHI-20260529-028</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>开挂</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>kāi guà</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>(게임에서) 치트키를 쓰다; (비유적으로) 비정상적으로 뛰어나다, 엄청나게 잘하다</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>成绩单一出，全员开挂：100%获得美国前30大学录取，75%斩获全美前20大学offer。</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>他学习能力太强了，感觉像开了挂一样，什么知识点都能很快掌握。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>CHI-20260529-029</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>研发</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Noun/Verb</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>yán fā</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>연구 개발 (R&amp;D); 연구 개발하다</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>公司主营高品质卫浴全系产品、建筑陶瓷及环保新材料（亚克力）的研发、生产与销售。</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>我们公司每年都会投入大量资金进行新产品的研发。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-05-31 | 145/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I137"/>
+  <dimension ref="A1:I146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6855,6 +6855,429 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>CHI-20260531-001</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>失联</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Separable Verb</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>shīlián</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>연락이 끊기다, 실종되다.</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>...拒绝支付任何赔偿，甚至失联跑路。</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>他已经好几天没来上班了，电话也打不通，好像失联了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>CHI-20260531-002</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>跑路</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>pǎolù</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>도망가다, (책임을 회피하고) 잠적하다.</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>...拒绝支付任何赔偿，甚至失联跑路。</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>那家小公司老板欠了员工工资就跑路了，真是太不负责任了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>CHI-20260531-003</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>凭借</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>píngjiè</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>~에 의지하여, ~을 바탕으로.</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>肖战、马丽分别凭借电影《得闲谨制》与《水饺皇后》，...</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>他凭借自己的努力和才华，终于在公司里获得了晋升。</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>CHI-20260531-004</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>融合</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Verb / Noun</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>rónghé</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>융합하다, 통합하다, 융합.</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>当百年遗产“邂逅”文旅潮流 工商文旅融合解锁跨界“...</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>现代科技与传统文化如何更好地融合，是我们需要思考的问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>CHI-20260531-005</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>出炉</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>chū lú</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>(결과, 제품 등이) 나오다, 발표되다</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>高考成绩出炉</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>经过几个月的紧张筹备，我们公司的新产品终于出炉了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>CHI-20260531-006</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>致敬</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>zhì jìng</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>경의를 표하다, 존경을 표하다</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>致敬劳动者</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>在这个特殊的日子里，我们向所有医护人员致敬。</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>CHI-20260531-007</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>聚焦</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>jù jiāo</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>초점을 맞추다, 집중하다</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>聚焦赣江流域水生...</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>下周的会议将聚焦如何提高市场份额的问题，请大家提前做好准备。</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>CHI-20260531-008</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>服役</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Separable Verb</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>fúyì</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>복무하다, 근무하다, (기계 등이) 운행되다</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>北京地铁一号线“服役”20多年的老列车在逐渐“告别...</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>这台服务器已经服役五年了，是时候考虑更新换代了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>CHI-20260531-009</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>咨询</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>zīxún</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>상담하다, 문의하다</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>我曾直接参与学校的心理健康咨询工作。</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>如果你对新政策有疑问，可以去人事部咨询。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-05-31 | 148/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I146"/>
+  <dimension ref="A1:I149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7278,6 +7278,147 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>CHI-20260531-010</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>签订合同</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Verb-Noun phrase</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>qiāndìng hétong</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>계약을 체결하다</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>...用人单位未签订劳动合同、未缴纳工伤保险...</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>我们公司今天和新客户签订了一份重要的合作合同。</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>CHI-20260531-011</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>缴纳</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>jiǎonà</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>납부하다 (세금, 비용 등을 내다)</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>...用人单位未签订劳动合同、未缴纳工伤保险...</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>每个月公司都会按时为员工缴纳社会保险。</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>CHI-20260531-012</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>启动</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>qǐdòng</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>시작하다, 가동하다, 발동하다</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>贝德美正式启动“旧物新生自然有续”环保计划...</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>公司下周将启动一个新的市场推广项目。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-01 | 150/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I149"/>
+  <dimension ref="A1:I151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7419,6 +7419,100 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>CHI-20260601-001</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>邂逅</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>xièhòu</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>우연히 만나다; 뜻밖에 만나다</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>当百年遗产“邂逅”文旅潮流 工商文旅融合解锁跨界“...</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>在这次国际会议上，我意外邂逅了一位多年未见的老同学。</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>CHI-20260601-002</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>志愿服务</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Separable Verb Phrase</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>zhì yuàn fú wù</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>자원봉사하다</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>践行志愿服务...</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>周末我们一起去养老院志愿服务吧。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-02 | 153/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I151"/>
+  <dimension ref="A1:I154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7513,6 +7513,147 @@
         </is>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>CHI-20260602-001</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>炸了</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>zhà le</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>(그룹 채팅방 등이) 난리가 났다, 폭발했다</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>家长群炸了！毕业生100%进世界前50！就读这所学...</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>今天老板突然宣布要加班，我们部门的微信群都炸了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>CHI-20260602-002</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>莫过于</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Fixed Phrase</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>mòguòyú</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>~보다 더한 것은 없다, ~만한 것이 없다</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>最让家属绝望的，莫过于“无社保、无合同”——用人单位未签订劳动合同、未缴纳工伤保险，员工因工死亡后，单位直接否认劳动关系，拒绝支付任何赔偿，甚至失联跑路。</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>对我们公司来说，最重要的莫过于客户的信任。</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>CHI-20260602-003</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>暖心</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>nuǎnxīn</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>마음을 따뜻하게 하는, 감동적인</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>张家界宠游客｜张家界环保客运 “宠客服务” 暖心护...</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>同事在我生病时送来了汤，这个举动真暖心。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-03 | 157/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I154"/>
+  <dimension ref="A1:I158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7654,6 +7654,194 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>CHI-20260603-001</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>深耕</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>shēn gēng</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>깊이 경작하다, 심층적으로 파고들다 (비유적으로)</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>北京多所学校深耕健...</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>这家公司在人工智能领域深耕多年，积累了丰富的经验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>CHI-20260603-002</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>践行</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>jiàn xíng</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>실천하다; 이행하다</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>践行志愿服务...</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>我们应该在日常工作中践行公司的核心价值观。</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>CHI-20260603-003</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>抱团</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>bàotuán</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>뭉치다, 단결하다 (서로 돕기 위해)</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>麻江教育“抱团记”.</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>面对激烈的市场竞争，小公司更需要抱团取暖，共同发展。</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>CHI-20260603-004</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>扫码添加</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Verb phrase</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>sǎomǎ tiānjiā</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>QR 코드를 스캔하여 추가하다</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>为获取密码“扫码添加...</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>你可以扫码添加我的微信，方便以后联系。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-03 | 158/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I158"/>
+  <dimension ref="A1:I159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7842,6 +7842,53 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>CHI-20260603-005</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>用人单位</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Noun</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>yòngrén dānwèi</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>고용주, 사용자 (회사, 기관 등)</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>用人单位未签订劳动合同、未缴纳工伤保险，员工因工死亡后，单位直接否认劳动关系，拒绝支付任何赔偿，甚至失联跑路。</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>在入职前，一定要仔细了解用人单位的规章制度。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-03 | 160/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I159"/>
+  <dimension ref="A1:I161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7889,6 +7889,100 @@
         </is>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>CHI-20260603-006</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>签订劳动合同</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Separable Verb Phrase</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>qiāndìng láodòng hétong</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>근로 계약을 체결하다</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>用人单位未签订劳动合同、未缴纳工伤保险...</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>新员工入职前，必须先签订劳动合同，明确双方的权利义务。</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>CHI-20260603-007</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>作证据</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Verb phrase</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>zuò zhèng jù</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>증거로 삼다, 증거가 되다</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>“AI生成照片”作证据？</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>你的证词可以作证据提交给警方。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-04 | 161/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I161"/>
+  <dimension ref="A1:I162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7983,6 +7983,53 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>CHI-20260604-001</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>亮了</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>liàng le</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>(성과 등이) 빛나다, 대단하다</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>成绩单，亮了.</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>他这次的提案非常精彩，直接让老板的眼睛都亮了。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-05 | 162/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I162"/>
+  <dimension ref="A1:I163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8030,6 +8030,53 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>CHI-20260605-001</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>提交</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>tí jiāo</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>제출하다</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>向法庭提交了两张电表照</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>请大家务必在周五下班前提交报告。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-09 | 165/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I163"/>
+  <dimension ref="A1:I166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8077,6 +8077,147 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>CHI-20260609-001</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>提醒</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>tí xǐng</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>상기시키다, 주의를 주다</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>车尾流行挂“毛绒尾巴”？律师提醒！</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>请你提醒会议室的同事，下午两点有重要会议。</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>CHI-20260609-002</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>流行</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Verb/Adjective</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>liú xíng</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>유행하다, 유행하는</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>车尾流行挂“毛绒尾巴”？律师提醒！</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>最近，线上学习在年轻人中越来越流行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>CHI-20260609-003</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>报名</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Separable Verb</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>bào míng</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>등록하다, 신청하다</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>小升初5月22日报名！</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>公司组织了一个羽毛球比赛，你想报名参加吗？</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-11 | 166/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I166"/>
+  <dimension ref="A1:I167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8218,6 +8218,53 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>CHI-20260611-001</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>保送</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Separable Verb</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>bǎo sòng</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>(시험 없이) 추천 입학시키다, 추천하다</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>拒绝清北的保送</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>他学习很好，被保送进了重点大学。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-12 | 167/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I167"/>
+  <dimension ref="A1:I168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8265,6 +8265,53 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>CHI-20260612-001</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>签订</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>qiāndìng</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>(계약, 협정 등을) 체결하다, 서명하다</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>用人单位未签订劳动合同、未缴纳工伤保险...</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>我们公司昨天和一家大客户签订了新的合作协议。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-14 | 171/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I168"/>
+  <dimension ref="A1:I172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8312,6 +8312,194 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>CHI-20260614-001</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>获悉</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>huòxī</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>알게 되다, 접수하다</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>4月29日，记者从北京市发改委获悉，自2024</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>我们刚刚获悉，公司下个月将推出新产品。</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>CHI-20260614-002</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>稳稳的幸福</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>wěnwěn de xìngfú</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>안정적인 행복</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>十年磨一剑！神仙学校给你稳稳的幸福.</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>对很多人来说，一份稳定的工作和健康的家庭就是稳稳的幸福。</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>CHI-20260614-003</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>受到关注</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Verb phrase</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>shòudào guānzhù</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>주목받다, 관심을 받다</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>这次受到关注的是在成都高新区双塔双集举办的“胡安·米罗：艺述真言”艺术展。</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>他的新书一上市就受到了广泛关注，销量非常好。</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>CHI-20260614-004</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>印象</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Noun</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>yìnxiàng</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>인상</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>却始终没有印象。</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>他给我的第一印象非常好，看起来很专业。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-14 | 173/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I172"/>
+  <dimension ref="A1:I174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8500,6 +8500,100 @@
         </is>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>CHI-20260614-005</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>座谈会</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Noun</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>zuò tán huì</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>좌담회, 간담회</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>雄安新区高校建设发展座谈会在河北雄安新区召开。</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>公司每个季度都会组织一次员工座谈会，听取大家的意见。</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>CHI-20260614-006</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>刷屏了</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Colloquialism</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>shuā píng le</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>(인터넷에서) 화면을 도배하다, 화제가 되다</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>留学圈被一所“年轻”的美高刷屏了</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>昨晚那部电影的预告片在朋友圈刷屏了，大家都想去看。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-15 | 194/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I174"/>
+  <dimension ref="A1:I195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8594,6 +8594,993 @@
         </is>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>CHI-20260615-001</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>跳槽</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>tiàocáo</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>이직하다, 직장을 옮기다</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>경쟁이 치열한 요즘, 더 나은 기회를 찾아 이직하는 사람들이 늘고 있다.</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>他在这家公司干了五年，最近决定跳槽去一家新公司。</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>CHI-20260615-002</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>考研</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>kǎoyán</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>대학원 입학시험을 치르다, 대학원 진학을 준비하다</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>많은 학생들이 학부 졸업 후 취업 대신 더 깊이 공부하기 위해 대학원 진학을 선택한다.</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>她打算毕业后考研，继续深造经济学。</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>CHI-20260615-003</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>开小差</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>kāi xiǎochāi</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>딴생각하다, 정신을 팔다, 게으름 피우다</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>수업 시간이나 회의 중에 집중하지 못하고 딴생각을 하는 경우가 있다.</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>开会的时候，他总是开小差，不知道在想什么。</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>CHI-20260615-004</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>脑洞</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>nǎodòng</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>기발한 상상력, 엉뚱한 아이디어</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>창의적인 사람들은 보통 예측 불가능하고 기발한 아이디어를 많이 생각해낸다.</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>他的脑洞真大，想出来的点子总是与众不同。</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>CHI-20260615-005</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>吃香</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>chīxiāng</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>(직업, 사람 등이) 인기 있다, 대우가 좋다</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>어떤 직업은 수요가 많거나 전망이 좋아서 사람들이 선호한다.</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>现在懂人工智能的技术人才非常吃香。</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>CHI-20260615-006</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>学霸</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>xuébà</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>모범생, 학업 성취가 매우 우수한 학생</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>어떤 학생은 항상 좋은 성적을 받고 모든 시험에서 뛰어나다.</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>我们班的学霸不仅学习好，体育也特别棒。</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>CHI-20260615-007</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>学渣</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>xuézhā</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>(자조적 표현) 공부 못하는 사람, 학업 성취가 낮은 학생</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>어떤 학생은 공부에 흥미가 없거나 성적이 좋지 않아 자책하기도 한다.</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>我以前一直是个学渣，直到高中才开始努力学习。</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>CHI-20260615-008</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>甩锅</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>shuǎi guō</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>(책임 등을) 남에게 떠넘기다, 전가하다</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>문제가 발생했을 때 자신의 책임을 회피하고 다른 사람에게 떠넘기는 경우가 있다.</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>项目失败后，他总是想方设法甩锅给别人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>CHI-20260615-009</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>内卷</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>nèijuǎn</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>과도한 내부 경쟁, 치열한 경쟁 심화 (인벌루션)</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>학업, 취업 등 다양한 분야에서 지나치게 치열한 경쟁이 사회적 문제로 대두되고 있다.</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>教育领域的内卷越来越严重，家长和学生压力都很大。</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>CHI-20260615-010</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>躺平</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>tǎngpíng</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>드러눕다; (사회적 경쟁에서) 포기하고 최소한의 노력만 하며 살아가다</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>치열한 경쟁에 지쳐 적극적인 삶을 포기하고 최소한의 노력으로 만족하는 태도를 보이기도 한다.</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>工作太累了，有时候真想直接躺平，什么都不干。</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>CHI-20260615-011</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>放鸽子</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>fàng gēzi</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>(약속을) 바람맞히다, 펑크 내다</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>친구와의 약속을 갑자기 취소하거나 나타나지 않아 상대를 기다리게 하는 상황.</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>他昨天又放我鸽子了，说好的电影票都浪费了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>CHI-20260615-012</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>接地气</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>jiē dìqì</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>서민적이다, 현실적이다, 대중과 친숙하다</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>어떤 사람이나 작품이 대중의 삶과 정서에 가까워 공감을 얻을 때 사용한다.</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>这位演员的表演很接地气，让人感觉很真实。</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>CHI-20260615-013</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>吃瓜</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>chī guā</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>(온라인에서) 흥미로운 가십이나 논쟁을 구경하다, 관망하다</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>인터넷에서 화제가 되는 사건이나 연예계 소식을 그저 지켜보는 행위.</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>网上又爆出大新闻了，快来一起吃瓜！</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>CHI-20260615-014</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>摸鱼</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>mōyú</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>땡땡이치다, 근무 중에 농땡이 피우다</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>직장에서 근무 시간에 몰래 다른 일을 하거나 시간을 낭비하는 행동.</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>老板不在，大家都开始摸鱼了，没人认真工作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>CHI-20260615-015</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>有戏</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>yǒuxì</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>가망 있다, 가능성 있다, 될 것 같다</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>어떤 일이 잘 될 가능성이 보이거나 희망이 있을 때 사용한다.</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>面试官对你印象很好，这事儿有戏！</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>CHI-20260615-016</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>莫名其妙</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>mòmíng qímiào</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>영문을 모르겠다, 어리둥절하다, 어이없다</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>예상치 못한 상황이나 행동에 대해 이해할 수 없을 때 쓰는 표현이다.</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>他突然生气，真是让我莫名其妙。</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>CHI-20260615-017</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>一干二净</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>yī gān èr jìng</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>말끔하게, 흔적도 없이, 깨끗이</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>무언가를 완전히 처리하거나 사라지게 만들었을 때 사용하는 표현이다.</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>他把桌上的文件整理得一干二净。</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>CHI-20260615-018</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>乱糟糟</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>luànzāozāo</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>엉망진창이다, 뒤죽박죽이다, 매우 지저분하다</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>정돈되지 않고 어지러운 상태나 복잡하고 혼란스러운 상황을 묘사할 때 쓴다.</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>我的房间已经乱糟糟的了，周末得好好收拾一下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>CHI-20260615-019</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>不负韶华</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>bù fù sháohuá</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>청춘을 헛되이 보내지 않다, 젊음을 소중히 하다</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>젊은 시절의 소중함과 그 시기를 의미 있게 보내야 한다는 격려의 메시지로 사용된다.</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>作为新时代的青年，我们应该努力学习，不负韶华。</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>CHI-20260615-020</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>得闲</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>déxián</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>틈이 나다, 한가해지다</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>肖战、马丽分别凭借电影《得闲谨制》...</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>你最近得闲了吗？我想约你一起去喝咖啡。</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>CHI-20260615-021</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>揭晓</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>jiēxiǎo</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>(결과, 정답 등이) 발표되다, 공개되다</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>全国大学生参与评选的各项荣誉正式揭晓。</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>比赛结果将于下周一正式揭晓，大家都非常期待。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-16 | 216/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I195"/>
+  <dimension ref="A1:I217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9581,6 +9581,1040 @@
         </is>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>CHI-20260616-001</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>炸锅</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>zhà guō</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>발칵 뒤집히다 (사람들이 흥분하거나 소동이 나다)</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>听到这所学校毕业生100%进世界前50的消息，家长群里瞬间炸锅了。</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>公司突然宣布要取消年终奖，整个办公室顿时炸锅了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>CHI-20260616-002</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>有一套</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>yǒu yī tào</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>자기만의 특별한 노하우가 있다, 솜씨가 보통이 아니다</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>这支青年团队在解决复杂技术问题方面，确实非常有一套。</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>李老师在调动学生积极性这方面真的很有一套，大家都爱上他的课。</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>CHI-20260616-003</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>不靠谱</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>bù kào pǔ</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>믿을 수 없다, 신뢰성이 떨어지다, 어설프다</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>原以为提交AI生成的照片当证据能瞒过去，结果这种不靠谱的做法被法官一眼识破了。</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>找合作伙伴千万不能找那种满嘴大话、办事不靠谱的人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>CHI-20260616-004</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>露馅儿</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>lòu xiànr</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>비밀이나 거짓말이 탄로나다, 들통나다</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>李某试图用修改过的假照片来蒙混过关，结果法官一核对细节就露馅儿了。</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>他本来想假装懂法语，结果一开口跟法国人说话就露馅儿了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>CHI-20260616-005</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>一技之长</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>yī jì zhī cháng</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>한 가지 전문적인 기술이나 특기</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>高职院校的学生通过各种技能大赛，练就了足以立足社会的一技之长。</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>不管时代怎么变，只要拥有一技之长，走到哪里都不怕找不到工作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>CHI-20260616-006</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>眼高手低</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>yǎn gāo shǒu dǐ</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>눈만 높고 실력은 형편없다</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>有些考生盲目拒绝名校保送，老师担心他眼高手低，在高考中吃亏。</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>年轻人找工作不能眼高手低，要先从基层做起积累经验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>CHI-20260616-007</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>打退堂鼓</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>dǎ tuì táng gǔ</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>도중에 포기하다, 꽁무니를 빼다</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>高考冲刺虽然辛苦，但已经走到了这一步，绝对不能半途打退堂鼓。</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>刚开始学游泳觉得特别难，我甚至想过打退堂鼓，但最后还是坚持下来了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>CHI-20260616-008</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>一清二楚</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>yī qīng èr chǔ</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>아주 명명백백하다, 또렷하다</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>专业团队提交了完备的证据链，把用人单位的各种违规操作扒得一清二楚。</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>合同条款已经写得一清二楚了，双方都必须按规定执行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>CHI-20260616-009</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>凑热闹</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>còu rè nao</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>구경거리에 합세하다, 유행에 편승하다</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>看到车站里举办精美的国画展，过往的旅客纷纷围上去凑热闹拍照打卡。</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>听说那家新开的奶茶店在打折，走，我们也去凑个热闹。</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>CHI-20260616-010</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>挑大梁</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>tiāo dà liáng</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>중요한 기둥 역할을 하다, 메인 책임을 지다</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>在这项国家级的青年科研项目中，有很多年轻的技术骨干开始挑大梁。</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>这次的大型晚会，导演决定让新来的主持人来挑大梁。</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>CHI-20260616-011</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>留一手</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>liú yī shǒu</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>만약을 대비해 한 수 숨겨두다, 노하우를 다 가르쳐주지 않다</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>那名工程师在离职前不仅没有留一手，反而偷偷带走了核心的技术资产。</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>师傅教徒弟手艺的时候，多多少少都会自己留一手。</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>CHI-20260616-012</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>钻空子</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>zuān kòng zi</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>허점을 노리다, 틈새를 이용하다</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>一些不法企业企图不签劳动合同来钻法律空子，以此逃避工伤赔偿责任。</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>规则制定得不够严密，就会给不法分子留下钻空子的机会。</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>CHI-20260616-013</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>唱反调</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>chàng fǎn diào</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>딴지를 걸다, 반대로 행동하여 엇나가다</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>处于青春叛逆期的孩子，常常喜欢和父母及学校的规定唱反调。</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>开会时大家都同意这个方案，只有他一个人故意和经理唱反调。</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>CHI-20260616-014</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>出风头</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>chū fēng tou</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>튀고 싶어 하다, 주목받으려 나서다</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>有些车主为了在马路上出风头，故意在车尾挂上夸张的毛绒尾巴饰品。</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>他在社交媒体上发布那些炫富的视频，无非就是想出风头罢了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>CHI-20260616-015</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>走弯路</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>zǒu wān lù</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>시행착오를 겪다, 비효율적인 길을 돌아가다</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>有名师在前方指引，青年教师们在办学实践中就能少走许多弯路。</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>多听听过来人的建议，可以让你在创业的过程中少走弯路。</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>CHI-20260616-016</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>泼冷水</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>pō lěng shuǐ</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>찬물을 끼얹다, 초를 치다</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>当学生提出具有创意的想法时，老师不应该一味地批评指责，更不能直接泼冷水。</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>大家都对这个新项目兴致勃勃，你先别急着给大家泼冷水。</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>CHI-20260616-017</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>打主意</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>dǎ zhǔ yi</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>딴마음을 품다, (나쁜 목적으로) 잔머리를 굴리다</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>有些心怀不轨的员工，利用职务便利对公司的高纯度原材料打起了主意。</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>你别想打那笔公款的主意，财务审计查得很严的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>CHI-20260616-018</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>有两下子</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>yǒu liǎng xià zi</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>제법 실력이 있다, 보통이 아니다</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>这些小朋友能用废弃矿泉水瓶做成精致的绿植花盆，动手能力确实有两下子。</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>看他写代码的速度和质量，就知道这个新来的程序员确实有两下子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>CHI-20260616-019</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>套近乎</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>tào jìn hū</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>친한 척 굴다, 사근사근하게 굴며 환심을 사다</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>网络诈骗犯往往会先通过各种方式跟受害人套近乎，骗取信任后再实施诈骗。</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>那个人一见面就跟我套近乎，肯定是有什么事情想求我帮忙。</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>CHI-20260616-020</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>走后门</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>zǒu hòu mén</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>빽을 쓰다, 부정한 방법으로 청탁하다</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>这所重点高中的招生政策十分公平公正，绝不允许任何人通过走后门入学。</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>我们公司招聘一向公开透明，绝不接受任何走后门的关系户。</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>CHI-20260616-021</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>吃闭门羹</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>chī bì mén gēng</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>문전박대당하다, 거절당하다</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>家属去涉事单位讨要工伤赔偿，结果不仅吃了闭门羹，连老板的电话也打不通了。</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>他好几次想约见那位投资人，结果都吃了闭门羹，连面都没见上。</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>CHI-20260616-022</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>开绿灯</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>kāi lǜ dēng</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>승인해 주다, 편의를 봐주다</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>为了吸引并留住优秀的文旅商户，当地相关部门在审批手续上为其特意开了绿灯。</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>为了支持这个环保项目的快速落地，市政府各部门决定特事特办，一路开绿灯。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-17 | 231/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I217"/>
+  <dimension ref="A1:I232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10615,6 +10615,711 @@
         </is>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>CHI-20260617-001</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>不负青春</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>búfù qīngchūn</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>청춘을 헛되이 보내지 않다, 청춘에 걸맞게 살다</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>致青春，向未来，要不负青春，努力拼搏。</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>我们应该珍惜时间，不负青春，去追求自己的梦想。</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>CHI-20260617-002</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>拼搏</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>동사 / 구어</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>pīnbó</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>있는 힘을 다해 싸우다, 분투하다</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>奋战环保一线15年，他用实际行动诠释着拼搏精神。</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>为了实现自己的目标，他一直在努力拼搏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>CHI-20260617-003</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>荣获</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>동사 / 오피스</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>rónghuò</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>영예롭게 획득하다, 수상하다</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>爱写诗的“理工男”荣获全国五一劳动奖章。</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>这家公司在国际大赛中荣获多项大奖，为国争光。</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>CHI-20260617-004</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>提质增效</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>관용구 / 오피스</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>tízhì zēngxiào</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>품질을 높이고 효율을 증대하다</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>推动高校向雄安疏解和承接工作提速提质。</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>我们今年的主要任务是提质增效，优化产品和服务。</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>CHI-20260617-005</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>宠客</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>동사 / 구어</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>chǒngkè</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>손님을 극진히 대하다, (과도하게) 챙겨주다</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>张家界环保客运的“宠客服务”暖心护航。</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>这家酒店的服务非常好，真是把客人宠到家了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>CHI-20260617-006</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>逞勇斗狠</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>chěngyǒng dòuhěn</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>용맹을 과시하고 난폭하게 싸우다</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>校务纠纷不容逞勇斗狠，要理性解决问题。</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>在公共场合逞勇斗狠只会让事情变得更糟。</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>CHI-20260617-007</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>以案促改</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>관용구 / 오피스</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>yǐ àn cù gǎi</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>사례(사건)를 통해 개혁을 촉진하다</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>零陵区柳子街小学召开“镜鉴”以案促改专项活动。</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>通过以案促改，我们吸取教训，完善了公司的管理制度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>CHI-20260617-008</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>不盲目</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>bù mángmù</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>맹목적이지 않다, 분별력 있게 행동하다</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>高考进补不盲目，选对食材是关键。</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>投资要理性，不盲目跟风，才能降低风险。</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>CHI-20260617-009</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>职务便利</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>명사 / 오피스</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>zhíwù biànlì</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>직무상의 편의 (주로 권한 남용을 의미)</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>工程师利用职务便利，将高纯度金线藏于无尘服口袋。</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>他因利用职务便利谋取私利而被公司开除。</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>CHI-20260617-010</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>加紧</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>동사 / 오피스</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>jiājǐn</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>더욱 서두르다, 바짝 옥죄다</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>宜昌长江公铁大桥加紧建设，确保工程进度。</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>时间紧迫，我们必须加紧工作，按时完成任务。</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>CHI-20260617-011</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>交出成绩单</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>구어 / 오피스</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>jiāochū chéngjìdān</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>성적표를 제출하다; (비유적으로) 성과를 보여주다</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>缺少重高生源，却能交出重高成绩。</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>面对股东，CEO必须在年终会议上交出满意的成绩单。</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>CHI-20260617-012</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>跨界</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>kuàjiè</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>분야를 넘나들다, 크로스오버하다</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>工商文旅融合解锁跨界“...”</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>越来越多的艺人开始尝试跨界合作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>CHI-20260617-013</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>开拓</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>kāituò</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>개척하다, 개발하다 (시장, 영역 등을 새롭게 열다)</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>高新区第一实验学校开拓校...</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>公司计划开拓新的国际市场。</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>CHI-20260617-014</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>奋战</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>fènzhàn</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>분투하다, 역전하다 (어려운 환경에서 열심히 싸우거나 노력하다)</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>奋战环保一线15年！</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>为了按时完成项目，我们团队奋战了几个通宵。</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>CHI-20260617-015</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>识破</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>shípò</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>(음모, 거짓말 등을) 간파하다, 꿰뚫어보다</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>法官一眼识破：假的！</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>他的谎言很快就被识破了。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-18 | 245/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I232"/>
+  <dimension ref="A1:I246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11320,6 +11320,664 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>CHI-20260618-001</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>致青春</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>zhì qīng chūn</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>청춘에게 바치는, 청춘을 기념하는</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>致青春 向未来丨这支“丝路青锋”青年团队的超能力是...</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>我们的毕业典礼主题就是致青春，希望大家永远保持年轻的心态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>CHI-20260618-002</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>提速</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>tí sù</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>속도를 높이다, 가속하다</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>推动北京地区高校向雄安疏解和承接工作提速提质...</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>为了赶上项目进度，我们必须提速了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>CHI-20260618-003</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>提质</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>tí zhì</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>품질을 향상시키다</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>推动北京地区高校向雄安疏解和承接工作提速提质...</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>公司今年的目标是产品提质增效。</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>CHI-20260618-004</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>盲目</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>형용사</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>máng mù</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>맹목적인, 무턱대고</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>高考进补不盲目，选对食材是关键。</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>做任何决定都不能盲目跟风，要有自己的判断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>CHI-20260618-005</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>心甘情愿</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>xīn gān qíng yuàn</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>기꺼이 바라다, 자진해서 하다, 달갑게 여기다</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>致敬劳动者｜出租车司机刘自立：用行动诠释劳模初心.</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>他为了自己的梦想，心甘情愿地付出了所有。</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>CHI-20260618-006</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>筑梦</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>zhù mèng</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>꿈을 이루다, 꿈을 만들어가다</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>以技筑梦 以农启航 湘潭生物机电学校农林牧渔技能竞...</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>年轻人要勇敢追逐，为自己的人生筑梦。</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>CHI-20260618-007</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>启航</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>qǐ háng</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>출항하다 (본래 의미), (새로운 여정을) 시작하다</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>以技筑梦 以农启航 湘潭生物机电学校农林牧渔技能竞...</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>新的一年，我们的公司将开启新的征程，再度启航。</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>CHI-20260618-008</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>消失</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>xiāo shī</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>사라지다, 없어지다</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>高考冲刺前100天，他又“突然消失”不来参加。</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>魔术师变了一个戏法，硬币就消失了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>CHI-20260618-009</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>理工男</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>lǐ gōng nán</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>이공계 남자 (학생/출신)</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>爱写诗的“理工男”荣获全国五一...</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>他虽然是个典型的理工男，但思维非常活跃。</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>CHI-20260618-010</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>参与评选</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>cān yù píng xuǎn</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>참여하여 심사하다, 평가에 참여하다</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>由全国大学生参与评选的各项荣誉正式揭晓。</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>今年的最佳影片将由观众投票参与评选。</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>CHI-20260618-011</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>传承</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>chuán chéng</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>계승하다, 전승하다</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>“传承教育家精神 潜心办学育新人”研讨会...</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>我们有责任传承中华民族的优秀文化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>CHI-20260618-012</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>潜心</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>qián xīn</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>마음을 다하다, 몰두하다</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>“传承教育家精神 潜心办学育新人”研讨会...</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>这位科学家潜心研究多年，终于取得了突破性进展。</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>CHI-20260618-013</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>诠释</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>quán shì</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>해석하다, 설명하다, 잘 보여주다</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>出租车司机刘自立：用行动诠释劳模初心。</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>这部电影完美诠释了友情的力量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>CHI-20260618-014</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>疏解</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>shū jiě</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>해소하다, 완화하다 (주로 인구, 기능 등)</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>推动北京地区高校向雄安疏解和承接工作提速提质...</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>政府正在采取措施疏解大城市的交通压力。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-19 | 269/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I246"/>
+  <dimension ref="A1:I270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11978,6 +11978,1134 @@
         </is>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>CHI-20260619-001</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>点亮</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>diǎn liàng</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>(등불을) 켜다; (비유) 밝히다, 빛나게 하다, 활성화하다</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>设计师들은 창의적인 활동으로 아비장 커뮤니티의 새로운 이미지를 **点亮**했다.</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>这部电影**点亮**了我对生活的热情。</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>CHI-20260619-002</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>对接</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>duì jiē</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>(업무나 시스템을) 연결하다, 접목하다, 연계하다</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>雄安新区와 베이징 지역 대학 간의 **对接** 작업을 가속화하여 질을 높여야 한다.</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>我们正在和客户**对接**项目细节，争取尽快签订合同。</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>CHI-20260619-003</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>拍板</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>pāi bǎn</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>최종 결정을 내리다, (협상을) 타결하다</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>这个项目的最终方案，还需要等老板来**拍板**。</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>会议上大家讨论了很久，最后还是由经理**拍板**决定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>CHI-20260619-004</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>搞定</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>gǎo dìng</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>일을 해내다, 문제를 해결하다, 상황을 마무리하다</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>这个复杂的客户需求，他居然一个人就**搞定**了。</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>别担心，这点小事我很快就能**搞定**。</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>CHI-20260619-005</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>划水</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>huá shuǐ</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>(비유) 대충대충 일하다, 게으름을 피우다 (원래는 수영에서 물을 젓는 동작)</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>现在很多人在工作中都喜欢**划水**，能少做就少做。</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>团队里总有人**划水**，导致其他人工作量增加。</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>CHI-20260619-006</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>一举两得</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>yī jǔ liǎng dé</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>일거양득, 한 가지 행동으로 두 가지 이득을 얻다</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>开展空瓶回收과 清山行动은 환경 보호와 공익 활동 **一举两得**다.</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>骑自行车上班，既能锻炼身体又能省钱，真是**一举两得**。</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>CHI-20260619-007</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>应付</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>yìng fù</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>대응하다, 처리하다; (건성으로) 대처하다, 얼버무리다</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>他工作总是敷衍了事，每次都是在**应付**领导和客户。</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>我今天有很多工作要**应付**，估计要加班了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>CHI-20260619-008</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>砥砺前行</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>dǐ lì qián xíng</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>어려움을 겪으며 노력하여 앞으로 나아가다, 역경을 딛고 정진하다</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>在挑战与机遇并存的时代，我们更要坚定信念，砥砺前行。</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>面对激烈的市场竞争，这家公司始终坚持创新，砥砺前行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>CHI-20260619-009</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>顺应潮流</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>shùn yìng cháo liú</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>흐름에 따르다, 시대의 조류에 부응하다</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>百年遗产要“邂逅”文旅潮流，就要学会顺应潮流，实现创新发展。</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>随着科技的进步，教育方式也要顺应潮流，利用新技术提升教学质量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>CHI-20260619-010</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>突破瓶颈</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>tū pò píng jìng</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>병목 현상을 돌파하다, 난관을 극복하다</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>工商文旅融合解锁跨界发展，旨在突破瓶颈，开创新的增长点。</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>公司目前面临技术瓶颈，急需引进人才来突破瓶颈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>CHI-20260619-011</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>赞不绝口</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>zàn bù jué kǒu</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>칭찬을 아끼지 않다, 입이 마르도록 칭찬하다</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>童声颂祖国，诗韵赞春天，现场观众听后都赞不绝口。</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>他做的菜太好吃了，大家都赞不绝口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>CHI-20260619-012</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>名列前茅</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>míng liè qián máo</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>선두에 서다, 상위권에 들다</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>毕业生100%进世界前50！这所学校的成绩一直名列前茅。</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>经过努力，他的学习成绩在班级中名列前茅。</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>CHI-20260619-013</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>脱颖而出</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>tuō yǐng ér chū</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>재능이 뛰어나 두각을 나타내다, 발군하다</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>在众多优秀学子中，他凭借卓越的表现脱颖而出，获得了保送资格。</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>她在这次选拔赛中脱颖而出，成功入选国家队。</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>CHI-20260619-014</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>兢兢业业</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>jīng jīng yè yè</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>조심스럽고 성실하게 일하다, 근면성실하다</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>奋战环保一线15年，他始终兢兢业业，为环保事业默默奉献。</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>他对待工作总是兢兢业业，从不马虎。</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>CHI-20260619-015</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>任劳任怨</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>rèn láo rèn yuàn</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>힘든 일도 마다하지 않고 불평하지 않다, 불평 없이 묵묵히 일하다</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>出租车司机刘自立用行动诠释劳模初心，他总是任劳任怨，服务乘客。</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>这位护士长对待病人总是任劳任怨，得到了大家的尊敬。</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>CHI-20260619-016</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>推卸责任</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>tuī xiè zé rèn</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>책임을 회피하다, 핑계를 대다</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>用人单位否认劳动关系，拒绝支付任何赔偿，企图推卸责任。</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>在团队合作中，每个人都应该承担自己的责任，不能互相推卸责任。</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>CHI-20260619-017</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>置之不理</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>zhì zhī bù lǐ</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>개의치 않다, 내버려 두다, 거들떠보지도 않다</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>有些单位失联跑路，对员工的合理诉求置之不理。</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>面对谣言，最好的办法就是置之不理，让它不攻自破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>CHI-20260619-018</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>攻坚克难</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>gōng jiān kè nán</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>난관을 극복하다, 굳게 버텨 어려움을 이겨내다</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>教育部长强调要全力以赴打好首批疏解高校雄安校区建设这场攻坚战，攻坚克难。</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>在科研项目中，我们常常需要团结协作，攻坚克难。</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>CHI-20260619-019</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>深耕细作</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>shēn gēng xì zuò</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>깊게 경작하고 섬세하게 재배하다 (비유적으로 정성껏 노력하다)</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>北京多所学校深耕健康教育，对学生进行深耕细作的引导。</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>在这个行业，只有深耕细作，才能建立自己的核心竞争力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>CHI-20260619-020</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>不负众望</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>bù fù zhòng wàng</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>기대에 부응하다, 기대에 어긋나지 않다</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>美国世外首届毕业生交出亮眼成绩单，不负众望，取得了优异的录取结果。</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>他以优异的成绩考上了理想的大学，不负众望。</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>CHI-20260619-021</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>出人意料</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>chū rén yì liào</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>예상 밖이다, 뜻밖이다</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>高考冲刺前他“突然消失”，但最终结果却出人意料，全福建为他骄傲！</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>比赛结果出人意料，原本不被看好的队伍竟然赢得了冠军。</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>CHI-20260619-022</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>以权谋私</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>yǐ quán móu sī</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>권력을 이용하여 사사로운 이익을 꾀하다</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>工程师利用职务便利，监守自盗，这是典型的以权谋私行为。</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>任何公职人员都不能以权谋私，必须廉洁奉公。</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>CHI-20260619-023</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>抱团取暖</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>bào tuán qǔ nuǎn</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>서로 의지하며 어려움을 극복하다 (추울 때 서로 끌어안고 체온을 나누듯)</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>麻江教育“抱团记”讲述了大家共同努力，抱团取暖的故事。</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>经济不景气，小企业之间更应该抱团取暖，共同应对挑战。</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>CHI-20260619-024</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>保驾护航</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>bǎo jià hù háng</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>호위하다, 안전을 지키다, 순조롭게 진행되도록 돕다</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>“四位一体”模式为学生心灵成长保驾护航，让他们健康快乐地成长。</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>专业律师团队为这次的并购案保驾护航，确保一切顺利进行。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-22 | 283/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I270"/>
+  <dimension ref="A1:I284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13106,6 +13106,664 @@
         </is>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>CHI-20260622-001</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>人间蒸发</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>rén jiān zhēng fā</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>흔적도 없이 사라지다, 종적을 감추다</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>高三考生拒绝清北保送，高考冲刺前100天他又突然不来参加，整个人就像人间蒸发了一样。</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>自从他借了钱以后，就整个人间蒸发了，电话也不接。</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>CHI-20260622-002</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>套路</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>tào lù</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>상투적인 수법, 꼼수, 낚시 (속임수)</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>购买化妆品后收到密码箱，为了获取密码需要扫码添加客服，这其实是新型的网络诈骗套路。</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>现在商家的促销活动全是套路，根本省不了多少钱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>CHI-20260622-003</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>拔尖</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>bá jiān</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>특출나다, 남보다 훨씬 뛰어나다</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>尽管缺少重点高中的生源，但这所学校在高考中依然取得了拔尖的成绩。</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>他在我们班里是成绩最拔尖的孩子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>CHI-20260622-004</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>放狠话</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>fàng hěn huà</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>엄포를 놓다, 독설을 퍼붓다, 악담하다</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>厦门一高三考生拒绝了保送，班主任气得放狠话，怒斥他狂妄自大。</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>他虽然嘴上经常放狠话，但其实心肠特别软。</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>CHI-20260622-005</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>硬撑</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>yìng chēng</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>억지로 버티다, 허세를 부리며 견디다</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>有些企业在没有合同和社保的情况下，面对工亡赔偿一味硬撑，拒不支付合理补偿。</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>生病了就赶紧去医院，别自己硬撑着。</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>CHI-20260622-006</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>吃独食</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>chī dú shí</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>독식하다, 혼자서 이득을 다 취하다</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>工程师利用职务便利，想把高纯度的金线偷偷藏进无尘服口袋里，这种吃独食的行为终究会败露。</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>团队合作最重要的就是利益共享，千万不能吃独食。</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>CHI-20260622-007</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>大手大脚</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>dà shǒu dà jiǎo</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>씀씀이가 헤프다, 돈을 펑펑 쓰다</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>虽然我们要提升生活质量，但环保低碳的生活要求我们不能再大手大脚地浪费资源。</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>他花钱总是大手大脚的，月底经常要向朋友借钱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>CHI-20260622-008</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>眼熟</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>yǎn shú</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>눈에 익다, 낯이 익다</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>校长在餐厅里努力搜寻着女孩的面孔，觉得她很眼熟，却一时想不起名字。</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>这个人我好像在哪里见过，看着特别眼熟。</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>CHI-20260622-009</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>玩失踪</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>wán shī zōng</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>잠수를 타다, 행방을 감추다, 연락을 끊다</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>无良的老板在发生工伤事故后，不仅不承担赔偿责任，甚至直接关门玩失踪。</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>有什么问题就当面解决，天天玩失踪算什么本事？</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>CHI-20260622-010</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>露一手</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>lòu yī shǒu</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>솜씨를 한 번 보여주다, 기량을 뽐내다</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>以技筑梦，农林牧渔技能竞赛提供了一个让同学们露一手的舞台。</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>今天家里请客，我爸特意下厨准备露一手他的拿手好菜。</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>CHI-20260622-011</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>对簿公堂</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>duì bù gōng táng</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>법정에서 시시비비를 가리다, 맞고소하다</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>房东与租客因为租金纠纷，最终只能选择对簿公堂。</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>既然双方无法达成和解，那就只能对簿公堂，让法律来裁判了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>CHI-20260622-012</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>对症下药</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>duì zhèng xià yào</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>상황이나 문제에 맞는 적절한 대책을 세우다</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>做心理咨询工作，最重要的一步就是了解情况后对症下药。</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>我们要分析客户流失的原因，对症下药，才能挽回损失。</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>CHI-20260622-013</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>迎难而上</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>yíng nán ér shàng</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>어려움을 마주하고 용감하게 나아가다</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>奋战环保一线15年，正是凭着这种迎难而上的精神，他才克服了重重阻碍。</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>面对市场的低迷，我们更要迎难而上，积极开拓新的业务领域。</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>CHI-20260622-014</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>煞费苦心</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>shà fèi kǔ xīn</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>몹시 고심하다, 무던히 애를 쓰다</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>为了让考生们在备考期间吃得有营养，妈妈每天都在菜单上煞费苦心。</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>老师为了纠正学生的错误习惯，可以说是煞费苦心。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-23 | 301/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I284"/>
+  <dimension ref="A1:I302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13764,6 +13764,852 @@
         </is>
       </c>
     </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>CHI-20260623-001</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>走心</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>zǒu xīn</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>마음을 쓰다, 진심을 담다, 정성을 들이다</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>不管是教学还是做公益，只要足够走心，就能赢得大家的支持。</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>这次的活动策划确实很走心，大家都很满意。</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>CHI-20260623-002</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>出圈</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>chū quān</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>유행을 타다, 팬덤을 넘어 대중적인 인기를 얻다</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>这部电影凭借口碑实现逆袭，成功在朋友圈出圈。</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>这部网剧刚上线就迅速出圈，成了社交媒体上的热门话题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>CHI-20260623-003</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>拿手</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>ná shǒu</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>능숙하다, 가장 자신 있는 분야이다</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>这几位工程师最拿手的就是精密设备的组装。</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>做红烧肉是妈妈的拿手好戏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>CHI-20260623-004</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>动刀子</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>dòng dāo zi</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>흉기를 휘두르다, 무력을 쓰다</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>学校里绝对不允许学生逞勇斗狠，甚至动刀子。</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>有话好好说，千万别冲动动刀子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>CHI-20260623-005</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>散步</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>sàn bù</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>산책하다</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>夕阳西下，居民们在河边悠闲地散步。</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>吃完饭去附近的公园散步对身体有好处。</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>CHI-20260623-006</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>稳扎稳打</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>wěn zhā wěn dǎ</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>착실하게 일을 처리하다, 신중하게 접근하다</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>高考拼营养｜三餐巧搭配 营养稳状态。</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>学习要稳扎稳打，不能急于求成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>CHI-20260623-007</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>顺水推舟</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>shùn shuǐ tuī zhōu</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>상황에 맞춰 대응하다, 기회를 이용해 일을 처리하다</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>工商业联合会（总商会）第十四次会员代表大会召开。</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>既然大家都同意这个方案，我就顺水推舟把它定下来了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>CHI-20260623-008</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>误打误撞</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>wù dǎ wù zhuàng</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>우연히 ~하게 되다</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>离奇的租赁纠纷，房东李某起诉租客。</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>我当初误打误撞进了这家公司，没想到发展得这么好。</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>CHI-20260623-009</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>碰瓷</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>pèng cí</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>고의적으로 사고를 내어 합의금을 뜯어내다</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>女子买99元化妆品收到密码箱，为了获取密码添加微信。</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>开车时遇到碰瓷的，一定要报警。</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>CHI-20260623-010</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>走马观花</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>zǒu mǎ guān huā</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>겉핥기식으로 대충 보다</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>成都高新这场艺术展，胡安·米罗展览吸引观众。</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>这次参观太匆忙，只能走马观花地看了一下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>CHI-20260623-011</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>解铃还须系铃人</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>jiě líng hái xū xì líng rén</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>문제를 일으킨 사람이 해결해야 한다</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>员工因工死亡后，单位直接否认劳动关系。</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>这件事谁引起的谁解决，真是解铃还须系铃人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>CHI-20260623-012</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>力不从心</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>lì bù cóng xóng xīn</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>마음은 원하나 능력이 따르지 않다</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>最让家属绝望的，莫过于“无社保、无合同”。</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>我也想多帮帮你，但是最近工作太忙，实在力不从心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>CHI-20260623-013</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>吃力不讨好</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>chī lì bù tǎo hǎo</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>수고는 많이 하지만 인정받지 못하다</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>校务纠纷处理不当，往往引发争议。</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>这种吃力不讨好的工作，没人愿意做。</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>CHI-20260623-014</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>不言而喻</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>bù yán ér yù</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>말하지 않아도 자명하다</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>办好学校的价值追求，潜心育人。</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>健康对每个人的重要性，是不言而喻的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>CHI-20260623-015</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>未雨绸缪</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>wèi yǔ chóu móu</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>미리 대비하다</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>高考拼营养，三餐巧搭配。</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>我们要未雨绸缪，提前做好项目的风险预案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>CHI-20260623-016</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>敷衍了事</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>fū yǎn liǎo liǎo shì</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>대충 얼렁뚱땅 일을 끝내다</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>单位直接否认劳动关系，拒绝支付赔偿。</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>对待工作绝不能敷衍了事，要认真负责。</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>CHI-20260623-017</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>如出一辙</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>rú chū yī zhé</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>똑같다, 판박이다</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>离奇的租赁纠纷，多起诈骗案手法相似。</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>这两个案例的处理方式几乎如出一辙。</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>CHI-20260623-018</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>自告奋勇</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>zì gào fèn yǒng</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>자진해서 나서다</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>学生积极参与志愿服务活动。</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>这次志愿者活动，他第一个自告奋勇去报名。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-24 | 318/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I302"/>
+  <dimension ref="A1:I319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14610,6 +14610,805 @@
         </is>
       </c>
     </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>CHI-20260624-001</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>打拼</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>동사 / 구어</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>dǎ pīn</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>고생하며 노력하다, 분투하다 (주로 타향에서)</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>젊은이들이 미래를 위해 도시에서 열심히 일하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>独自在外打拼几年，她终于有了自己的事业。</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>CHI-20260624-002</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>搭档</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>이합사 / 명사</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>dā dàng</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>짝을 이루다, 파트너; 동반자</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>협력 프로젝트에서 좋은 파트너를 찾는 것이 중요합니다.</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>我很喜欢和他一起工作，我们是最佳搭档。</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>CHI-20260624-003</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>创新</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>이합사 / 명사</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>chuàng xīn</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>혁신하다, 창조하다; 혁신, 창조</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>기업들은 끊임없이 새로운 아이디어를 내고 혁신해야 합니다.</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>这个产品在技术上有很多创新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>CHI-20260624-004</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>大跌眼镜</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>dà diē yǎn jìng</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>매우 놀라다, 깜짝 놀라다 (예상 밖의 일에)</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>예상치 못한 결과나 상황에 사람들이 놀라움을 표현합니다.</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>他竟然辞职了，真是让所有人大跌眼镜。</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>CHI-20260624-005</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>出人头地</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>chū rén tóu dì</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>출세하다, 남들보다 뛰어나다, 두각을 나타내다</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>많은 사람들이 성공해서 남들보다 돋보이기를 바랍니다.</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>父母都希望自己的孩子能出人头地。</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>CHI-20260624-006</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>望子成龙</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>wàng zǐ chéng lóng</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>자식이 용처럼 훌륭하게 되기를 바라다 (자식의 성공을 바람)</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>학부모들이 자녀의 성공에 대한 높은 기대를 가집니다.</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>天下父母心，谁不望子成龙、望女成凤呢？</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>CHI-20260624-007</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>一言难尽</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>yī yán nán jìn</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>한마디로 다 말하기 어렵다, 사정이 복잡하다</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>복잡하거나 설명하기 어려운 상황에 대해 이야기할 때 사용합니다.</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>他最近的遭遇真是一言难尽，你就别问了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>CHI-20260624-008</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>吃亏</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>chī kuī</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>손해를 보다, 불이익을 당하다</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>계약 관계나 거래에서 손해를 보는 상황을 말합니다.</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>做生意不能总是怕吃亏，有时候要懂得付出。</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>CHI-20260624-009</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>身体力行</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>shēn tǐ lì xíng</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>몸소 실천하다, 솔선수범하다</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>말로만 하는 것이 아니라 직접 행동으로 보여주는 것을 강조합니다.</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>作为领导，他总是身体力行，给员工树立榜样。</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>CHI-20260624-010</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>言传身教</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>yán chuán shēn jiào</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>말로 가르치고 행동으로 본보기를 보이다 (가르침의 방식)</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>교사나 부모가 말과 행동으로 자녀나 학생을 지도하는 방식입니다.</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>父母的言传身教对孩子的成长至关重要。</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>CHI-20260624-011</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>弄虚作假</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>nòng xū zuò jiǎ</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>허위 사실을 조작하다, 사기 치다, 속임수를 쓰다</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>가짜 증거나 정보를 만들어내어 사람들을 속이는 행위를 말합니다.</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>考试作弊就是弄虚作假的行为，后果很严重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>CHI-20260624-012</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>花言巧语</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>huā yán qiǎo yǔ</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>교활한 말솜씨, 감언이설 (진심이 담기지 않은 듣기 좋은 말)</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>겉으로 듣기에는 좋지만 사실은 진실되지 않은 말을 의미합니다.</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>别相信他的花言巧语，他只是想利用你。</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>CHI-20260624-013</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>化解</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>huà jiě</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>해결하다, 완화하다 (갈등, 위기 등)</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>분쟁이나 어려운 상황을 풀고 해결하는 과정을 말합니다.</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>通过沟通，他们终于化解了误会。</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>CHI-20260624-014</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>和解</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>hé jiě</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>화해하다, 합의하다</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>갈등이 있던 양측이 서로 타협하여 평화를 되찾는 것입니다.</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>经过调解，双方最终达成了和解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>CHI-20260624-015</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>撕破脸</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>sī pò liǎn</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>체면을 구기다, 공개적으로 다투다 (관계가 악화되어)</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>더 이상 서로의 체면을 봐주지 않고 관계를 단절할 정도로 싸우는 상황입니다.</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>为了这点小事，犯不着撕破脸。</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>CHI-20260624-016</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>脑洞大开</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>구어 / 관용구</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>nǎo dòng dà kāi</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>기발한 아이디어가 넘치다, 상상력이 풍부하다 (새롭고 엉뚱한 생각)</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>창의적인 생각이나 기발한 아이디어가 샘솟는 상태를 묘사합니다.</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>看这部电影的时候，真是让我脑洞大开，想象力无限。</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>CHI-20260624-017</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>就读</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>jiù dú</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>학교에 다니다, 재학하다</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>毕业生100%进世界前50！就读这所学...</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>他大学毕业后选择继续就读研究生，希望能深造专业知识。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-25 | 326/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I319"/>
+  <dimension ref="A1:I327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15409,6 +15409,382 @@
         </is>
       </c>
     </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>CHI-20260625-001</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>一线</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>yīxiàn</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>최전선, 현장 (업무의 핵심이나 위험한 곳)</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>환경보호 一线에서 15년간 분투하다! 시 쓰는 '이공남'이 전국 5.1노동절 상을 수상했다.</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>医护人员一直奋战在抗疫一线，非常辛苦。</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>CHI-20260625-002</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>亮点</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>liàngdiǎn</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>하이라이트, 돋보이는 점, 매력 포인트</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>미국 월드아웃 첫 졸업생들의 성적표가 눈에 띄었다 (亮了).</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>这个方案的亮点在于它兼顾了效率和环保。</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>CHI-20260625-003</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>播出</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>bō chū</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>방송하다, 방영하다</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>荣誉盛典播出</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>这部电视剧每晚八点准时播出。</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>CHI-20260625-004</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>评选</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>píng xuǎn</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>평가하여 선정하다, 심사 선발하다</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>由全国大学生参与评选的各项荣誉正式揭晓。</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>公司每年都会评选出优秀的团队和个人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>CHI-20260625-005</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>绝望</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>jué wàng</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>절망하다, 희망을 잃다</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>最让家属绝望的，莫过于“无社保、无合同”</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>面对如此困境，她几乎要绝望了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>CHI-20260625-006</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>否认</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>fǒu rèn</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>부인하다, 부정하다</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>单位直接否认劳动关系</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>他否认了所有指控，坚称自己无罪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>CHI-20260625-007</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>指引</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>zhǐ yǐn</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>안내하다, 이끌다, 지시하다</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>在教育家精神指引下</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>在老师的指引下，我找到了学习的方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>CHI-20260625-008</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>宠爱</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>chǒng ài</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>(아랫사람을) 매우 아끼고 사랑하다, 응석을 받아주다</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>张家界宠游客</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>爷爷奶奶特别宠爱小孙子，几乎有求必应。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-26 | 339/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I327"/>
+  <dimension ref="A1:I340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15785,6 +15785,617 @@
         </is>
       </c>
     </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>CHI-20260626-001</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>扯皮</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>chěpí</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>서로 책임 전가하며 다투다, 지루하게 실랑이하다, 핑계를 대다</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>这项工作谁来负责，他们已经扯皮好几天了，还没个结果。</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>别再扯皮了，我们得尽快解决这个问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>CHI-20260626-002</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>踏实</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>형용사</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>tāshi</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>착실하다, 성실하다, 마음이 편안하고 안정되다, 견실하다</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>神仙学校给你稳稳的幸福，让学生学得踏实，活得自在。</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>他工作一直很踏实，深得领导信任。</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>CHI-20260626-003</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>护航</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>hùháng</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>(안전하게) 호위하다, 보호하다, (성장을) 지원하다</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>“四位一体”护航学生心灵成长，保障心理健康。</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>父母的爱为孩子的健康成长保驾护航。</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>CHI-20260626-004</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>上当受骗</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>shàng dàng shòu piàn</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>속아서 피해를 입다, 사기를 당하다</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>女子买99元化妆品收到密码箱，不慎扫码后上当受骗。</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>提醒大家，不要轻易相信网络上的陌生信息，以免上当受骗。</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>CHI-20260626-005</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>出差</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>chūchāi</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>출장 가다</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>最近部门业务繁忙，很多同事都经常出差。</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>他下周要去上海出差三天。</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>CHI-20260626-006</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>磨合</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>móhé</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>(사람, 팀, 기계 등이) 길들다, 조화를 이루다, 마찰을 통해 조정하다</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>新来的团队成员需要一段时间的磨合才能配合默契。</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>新组建的团队还需要时间磨合才能达到最佳状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>CHI-20260626-007</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>拉黑</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>lāhēi</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>(SNS 등에서) 차단하다, 블랙리스트에 올리다</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>那个一直发广告骚扰我的人，我把他拉黑了。</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>他总是发一些不实信息，我决定把他拉黑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>CHI-20260626-008</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>点赞</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>diǎnzàn</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>(SNS에서) '좋아요'를 누르다, 칭찬하다, 엄지 척하다</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>看到朋友分享的美食照片，忍不住给他点了个赞。</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>你的演讲非常精彩，我给你点赞！</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>CHI-20260626-009</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>蹭饭</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>cèngfàn</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>(남에게) 얻어먹다, 염치없이 밥을 얻어먹다</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>我今天没带饭，能去你家蹭饭吗？</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>他脸皮厚，经常去朋友家蹭饭。</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>CHI-20260626-010</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>一帆风顺</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>yī fān fēng shùn</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>순조롭다, 만사형통하다, 순풍에 돛 단 듯하다</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>希望你的学业和事业都能一帆风顺。</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>祝你新的一年工作顺利，一帆风顺！</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>CHI-20260626-011</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>马马虎虎</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>mǎmǎhǔhǔ</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>그럭저럭, 대충대충, 그저 그렇다 (보통 부정적인 뉘앙스)</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>这篇文章他写得马马虎虎，还有很多需要修改的地方。</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>你做事情总是马马虎虎，怎么能保证质量呢？</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>CHI-20260626-012</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>临时抱佛脚</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>línshí bào fójiǎo</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>급해져서야 발등에 불 떨어진 듯 행동하다, 벼락치기하다</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>马上要考试了，他才开始临时抱佛脚，希望能及格。</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>学习不能临时抱佛脚，平时积累很重要。</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>CHI-20260626-013</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>一拍即合</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>yī pāi jí hé</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>(의견, 의기투합하여) 즉시 잘 맞다, 의기투합하다</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>他们两个人的想法一拍即合，很快就达成了合作。</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>我们对这个项目的看法一拍即合，合作非常顺利。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-29 | 351/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I340"/>
+  <dimension ref="A1:I352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16396,6 +16396,570 @@
         </is>
       </c>
     </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>CHI-20260629-001</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>有两把刷子</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>yǒu liǎng bǎ shuā zi</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>실력이 좋다, 솜씨가 뛰어나다</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>그는 고생해서 15년 동안 환경 보호 일선에서 일했는데, 정말 실력이 뛰어난 사람이다.</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>别看他年纪轻，工作起来可是有两把刷子的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>CHI-20260629-002</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>逆袭</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>nì xí</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>역전하다, (약자가 강자를) 제압하다, 반격하여 성공하다</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>고등학교 3학년 학생이 청화대, 북경대 추천을 거절하고 사라졌다가 20일 후 모두를 놀라게 하는 역전 드라마를 썼다.</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>那支弱队在最后几分钟成功逆袭，赢得了比赛。</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>CHI-20260629-003</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>脚踏实地</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>jiǎo tà shí dì</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>성실하고 착실하다, 현실에 발붙이다</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>꿈을 이루려면 하늘에 닿는 구름만 쫓지 말고, 성실하게 한 걸음 한 걸음 나아가야 한다.</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>成功没有捷径，只有脚踏实地，一步一个脚印才能实现。</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>CHI-20260629-004</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>精益求精</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>jīng yì qiú jīng</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>더욱 더 완벽을 기하다, 끊임없이 발전시키다</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>우리는 제품의 품질을 더욱 더 완벽하게 만들고, 더 높은 환경 보호 등급의 재료를 사용해야 한다.</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>对待工作，我们应该抱着精益求精的态度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>CHI-20260629-005</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>与时俱进</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>yǔ shí jù jìn</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>시대와 더불어 발전하다, 시대의 흐름에 발맞추다</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>백년의 유산이 문화 관광 트렌드와 만나 시대의 흐름에 발맞춰 융합을 이뤄내다.</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>教育理念要与时俱进，才能培养出适应社会发展的人才。</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>CHI-20260629-006</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>哭笑不得</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>kū xiào bù dé</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>울지도 웃지도 못하다, 어이가 없다</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>그 상황을 보고 나는 정말 울지도 웃지도 못했다.</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>听到这个荒唐的理由，我真是哭笑不得。</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>CHI-20260629-007</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>碰壁</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>pèng bì</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>장애에 부딪히다, 거절당하다, 좌절을 겪다</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>그는 이번 일에서 여러 번 좌절을 겪었지만, 포기하지 않았다.</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>求职之路屡次碰壁，但他从没放弃。</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>CHI-20260629-008</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>画大饼</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>huà dà bǐng</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>허황된 약속을 하다, 헛된 희망을 주다 (주로 부정적)</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>일부 고용주들은 직원들에게 사회 보험이나 계약 없이 말로만 허황된 약속을 한다.</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>老板总是在会议上给大家画大饼，但实际行动却很少。</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>CHI-20260629-009</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>打水漂</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>dǎ shuǐ piāo</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>돈이나 노력이 허사가 되다, 헛수고하다</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>이 프로젝트에 투자한 모든 노력이 허사가 될까 봐 걱정된다.</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>这笔钱要是投资失败，可就全部打水漂了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>CHI-20260629-010</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>一刀切</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>yī dāo qiē</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>일률적으로 적용하다, 획일적으로 처리하다 (종종 부정적 뉘앙스)</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>정책을 제정할 때는 지역 상황을 고려해야지, 일률적으로 적용해서는 안 된다.</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>这种一刀切的管理方式，不适合我们公司的多元化发展。</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>CHI-20260629-011</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>无功而返</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>wú gōng ér fǎn</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>수확 없이 돌아오다, 헛수고만 하고 돌아오다</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>그는 이번 출장에서 아무런 성과 없이 돌아왔다.</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>我们找了一天，最后还是无功而返。</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>CHI-20260629-012</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>水深火热</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>shuǐ shēn huǒ rè</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>매우 고통스러운 상황, 극심한 곤경에 처하다</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>사회 보험도 계약도 없는 근로자는 사고가 났을 때 극심한 곤경에 처하게 된다.</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>战争让那里的人民生活在水深火热之中。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-06-30 | 370/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I352"/>
+  <dimension ref="A1:I371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16960,6 +16960,899 @@
         </is>
       </c>
     </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>CHI-20260630-001</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>有出息</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>yǒu chū xi</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>출세하다, 장래가 촉망되다</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>退休的老教师看着当年的学生如今在各行各业发光发热，心里觉得他们真有出息。</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>只要你肯脚踏实地努力工作，以后一定会有出息的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>CHI-20260630-002</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>开眼界</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>kāi yǎn jiè</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>시야를 넓히다, 안목을 틔우다</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>学校安排高考生走进能源一线去实地参观，真的让大家开了眼界。</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>这次去国外参加行业博览会，真是让我大开眼界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>CHI-20260630-003</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>下功夫</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>xià gōng fu</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>공을 들이다, 노력과 시간을 쏟다</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>要想考入理想的高校，不下一番苦功夫是不可能的。</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>为了准备这次的汇报，他在演讲稿上着实下了一番功夫。</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>CHI-20260630-004</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>半路出家</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>bàn lù chū jiā</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>비전공자로 시작하다, 중간에 전업하다</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>有些学生在大学期间跨专业学习，虽然是半路出家，但凭借热爱也学得很好。</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>他虽然是半路出家当的程序员，但技术水平不亚于科班出身的人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>CHI-20260630-005</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>说得过去</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>shuō de guò qù</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>그럭저럭 말이 되다, 봐줄 만하다</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>只要这次的高考成绩还说得过去，我们就能报个不错的本地大学。</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>虽然没有拿到第一名，但这个成绩在家里人面前也算说得过去了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>CHI-20260630-006</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>合得来</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>hé de lái</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>성격이 맞다, 마음이 잘 맞다</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>能和同宿舍的朋友们合得来，大学四年的生活质量会提高很多。</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>新来的同事性格开朗，跟大家都挺合得来的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>CHI-20260630-007</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>吃苦耐劳</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>chī kǔ nài láo</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>고생을 참고 견디며 성실히 일하다</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>国企招聘时，非常看重毕业生是否具备吃苦耐劳的精神和实干作风。</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>那个新员工不仅聪明，而且吃苦耐劳，深得老板的赏识。</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>CHI-20260630-008</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>心血来潮</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>xīn xuè lái cháo</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>갑자기 생각이 떠오르다, 충동적으로 결정하다</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>家长把家里的鸵鸟送给学校当谢师礼，绝对不是心血来潮，而是充满诚意的感恩之举。</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>他昨晚心血来潮，买了一张今天一早去海边的机票。</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>CHI-20260630-009</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>干脆利落</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>gān cuì lì luò</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>시원시원하고 군더더기 없다, 매끄럽다</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>这次的退役军人荣休典礼办得干脆利落，每一个流程都恰到好处。</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>他做事情向来干脆利落，最讨厌拖泥带水了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>CHI-20260630-010</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>铁饭碗</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>tiě fàn wǎn</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>안정적인 직장, 철밥통</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>现在的年轻人虽然追求自由，但在长辈眼里，国企依然是个稳当的铁饭碗。</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>在这个瞬息万变的时代，已经没有绝对一成不变的铁饭碗了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>CHI-20260630-011</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>干劲儿</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>gàn jìn r</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>의욕, 열정, 일할 맛</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>大家刚拿到心仪企业的offer，对待接下来的实操培训都充满了干劲儿。</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>听到项目奖金翻倍的消息，大家的干劲儿一下子就上来了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>CHI-20260630-012</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>顺风顺水</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>shùn fēng shùn shuǐ</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>모든 일이 순조롭게 잘 풀리다</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>校长祝愿毕业生们在新的人生下一程中，顺风顺水，前程似锦。</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>希望你换了新工作之后能够顺风顺水，步步高升。</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>CHI-20260630-013</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>打破砂锅问到底</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>dǎ pò shā guō wèn dào dǐ</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>집요하게 끝까지 캐묻다</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>在学术研讨和名师对话中，我们应该保持那种打破砂锅问到底的求知欲。</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>这个小孩子好奇心特别强，遇到不懂的总是喜欢打破砂锅问到底。</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>CHI-20260630-014</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>摸不着头脑</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>mō bù zháo tóu nǎo</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>갈피를 잡지 못하다, 영문을 모르다</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>突然宣布的招生考试新规则让很多考生和家长摸不着头脑。</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>他今天莫名其妙地对我发火，真是让我摸不着头脑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>CHI-20260630-015</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>不景气</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>bù jǐng qì</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>(경제나 사업 등이) 불황이다, 침체하다</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>近年来环保产业面临一些挑战，但在行业不景气的时候，绿创江南依然坚持技术升级。</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>虽然今年整体市场不景气，但只要我们能保证产品质量，依然能赢得客户。</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>CHI-20260630-016</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>急于求成</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>jí yú qiú chéng</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>서둘러 성공을 거두려 하다, 성급하게 서두르다</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>刘校长寄语毕业生，在未来的事业中要循序渐进，切勿急于求成。</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>创业需要长期的积累，急于求成往往会导致失败。</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>CHI-20260630-017</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>耳目一新</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>ěr mù yī xīn</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>눈과 귀가 새로워지다, 완전히 새로운 느낌을 주다</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>北碚区状元小学校越剧节目让观众耳目一新，斩获了多项大奖。</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>这次林氏整家定制发布的新产品，从设计到功能都让人耳目一新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>CHI-20260630-018</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>人不可貌相</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>rén bù kě mào xiàng</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>사람을 겉모습으로만 평가해서는 안 된다</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>中职学校的学生同样展现出了蓬勃的生命力，真是人不可貌相。</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>别看他穿得很朴素，其实他是个深藏不露的计算机天才，真是人不可貌相。</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>CHI-20260630-019</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>见世面</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>jiàn shì miàn</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>세상 경험을 쌓다, 넓은 세상을 보고 배우다</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>60余名高考生走进能源一线，正是为了多见见世面，了解真正的产业现状。</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>年轻人应该多去大城市或先进企业见世面，提升自己的综合素质。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-01 | 398/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I371"/>
+  <dimension ref="A1:I399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17853,6 +17853,1322 @@
         </is>
       </c>
     </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>CHI-20260701-001</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>备考</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>bèi kǎo</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>시험을 준비하다</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>高考结束了，走出了早起晚睡的备考模式。</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>为了考研，我最近一直在紧张地备考。</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>CHI-20260701-002</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>开会</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>kāi huì</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>회의하다</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>今天下午有一个重要的客户会议，请大家准时参加。</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>我们的团队每周一早上都会开会讨论工作计划。</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>CHI-20260701-003</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>奉献</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>fèng xiàn</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>헌신하다, 기여하다</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>感谢他为公司做出的巨大奉献。</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>老师们默默耕耘，把青春都奉献给了教育事业。</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>CHI-20260701-004</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>退休</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>tuì xiū</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>퇴직하다, 은퇴하다</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>株洲市第七中学举办退休教师座谈会。</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>父母退休后终于有时间去环游世界了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>CHI-20260701-005</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>就职</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>jiù zhí</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>취임하다, 직위에 오르다</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>李常官已任民政部党组书记。</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>新任校长将于下周举行就职典礼。</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>CHI-20260701-006</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>入职</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>rù zhí</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>입사하다</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>全员入职央国企这间大学宿舍“电力”全开。</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>我下个月就正式入职新公司了，有点紧张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>CHI-20260701-007</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>填报</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>tián bào</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>(양식 등을) 작성하여 제출하다</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>为帮助考生更科学地填报志愿。</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>截止日期前请务必完成个人信息的填报。</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>CHI-20260701-008</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>爆单</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>bào dān</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>주문이 폭주하다, 주문량이 엄청나게 늘다</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>爆单的“高考志愿填报指导”服务。</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>双十一期间，我们店铺的销量直接爆单了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>CHI-20260701-009</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>赋能</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>fù néng</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>역량을 부여하다, 능력을 활성화하다 (empower)</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>康森饰家FOSB欧松板：结构突破环保先行，赋能家居。</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>这项新技术将赋能我们的产品，使其更具竞争力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>CHI-20260701-010</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>布局</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>bù jú</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>(전략적으로) 배치하다, 구도를 짜다, 계획하다</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>山东龙山产发：深耕主业布局新赛道。</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>公司正在积极布局海外市场，寻求新的增长点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>CHI-20260701-011</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>新赛道</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>xīn sàidào</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>새로운 사업 분야/시장 (비즈니스 용어)</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>深耕主业布局新赛道。</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>很多传统企业都在积极探索转型，寻找新的赛道。</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>CHI-20260701-012</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>助力</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>zhù lì</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>힘을 보태다, 도움을 주다, 촉진하다</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>助力区域高质量发展。</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>感谢各方力量助力本次活动的成功举办。</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>CHI-20260701-013</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>上线</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>shàng xiàn</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>(서비스, 앱 등이) 출시되다, 시작되다, (컴퓨터) 온라인 상태가 되다</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>“官方带娃”上线 湖州所有义务段学校将开启暑期托管。</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>我们的新产品预计下个月正式上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>CHI-20260701-014</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>零门槛</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>líng mén kǎn</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>진입 장벽이 없다, 아무나 할 수 있다 (어떤 활동이나 서비스에 대해)</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>零门槛3天速成。</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>这项兼职工作零门槛，非常适合学生党。</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>CHI-20260701-015</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>拾级而上</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>shí jí ér shàng</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>계단을 밟고 오르다, 점진적으로 발전하다/향상하다</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>校长刘昌胜院士以《拾级而上弘深致远》为题，为同学们带来了“最后一课”。</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>学习是一个拾级而上的过程，需要耐心和坚持。</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>CHI-20260701-016</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>初心不改</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>chū xīn bù gǎi</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>초심을 잃지 않다, 처음의 뜻을 변치 않다</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>青丝染霜初心不改。</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>无论未来遇到什么困难，希望我们都能初心不改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>CHI-20260701-017</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>薪火相传</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>xīn huǒ xiāng chuán</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>(학문, 기술, 정신적 유산 등을) 대대로 전하다, 계승하다</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>芳华岁月薪火相传。</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>传统文化的精髓需要一代代人薪火相传。</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>CHI-20260701-018</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>水到渠成</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>shuǐ dào qú chéng</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>때가 되면 자연스럽게 이루어지다, 순리대로 되다</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>（인생 조언） 很多事情只要努力了，水到渠成是早晚的事。</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>只要功夫深，铁杵磨成针，成功自然会水到渠成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>CHI-20260701-019</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>来之不易</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>lái zhī bù yì</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>어렵게 얻은, 쉽지 않게 얻은, 소중한</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>（격려의 말） 珍惜这来之不易的幸福生活。</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>今天的成就来之不易，我们更应该加倍努力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>CHI-20260701-020</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>早起晚睡</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>zǎo qǐ wǎn shuì</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>일찍 일어나고 늦게 자다 (열심히 일하거나 공부함을 비유)</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>走出了早起晚睡的备考模式。</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>为了完成这个项目，大家最近都早起晚睡，非常辛苦。</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>CHI-20260701-021</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>带娃</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>dài wá</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>아이를 돌보다, 아이를 키우다</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>“官方带娃”上线 湖州所有义务段学校将开启暑期托管。</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>她辞职在家全职带娃，压力确实不小。</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>CHI-20260701-022</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>收官</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>오피스</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>shōu guān</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>(사업, 행사 등을) 마무리하다, 종결하다</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>信达生物公益行在苏州收官。</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>经过大家的努力，这个月的销售任务终于完美收官。</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>CHI-20260701-023</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>投用</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>tóu yòng</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>투입하여 사용하다, 가동하다</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>宁波：两所新学校9月投用。</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>新的生产线下个月就能正式投用了，这将大大提高效率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>CHI-20260701-024</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>施救</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>shī jiù</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>구조하다, 구원하다</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>30分钟跪地“教科书式”施救！</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>医生们及时施救，才保住了他的生命。</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>CHI-20260701-025</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>寄语</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>jì yǔ</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>(격려, 축하, 당부 등의) 말을 전하다, 메시지를 보내다</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>西政校长林维寄语毕业生：做一个让社会变得更好的人。</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>在毕业典礼上，校长向全体毕业生寄语了美好的祝愿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>CHI-20260701-026</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>戳中</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>chuō zhòng</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>(핵심을) 찌르다, (아픈 곳을) 건드리다, (공감대를) 형성하다</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>“你只是高考完了，不是家里发财了”，戳中了谁？</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>他的话语直接戳中了问题的核心，让大家陷入了沉思。</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>CHI-20260701-027</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>凭空而起</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>píng kōng ér qǐ</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>아무런 근거 없이 생겨나다/일어나다, 갑자기 나타나다</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>没有凭空而起的高地。</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>谣言往往凭空而起，但对社会造成的危害却不容小觑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>CHI-20260701-028</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>查家底</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>chá jiā dǐ</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>(어떤 사람의) 가정 배경이나 재산 상황을 조사하다</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>新生入学查家长职务和车型，打探家底是对教育公...</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>在合作前，我们需要彻底查清对方的家底，确保没有风险。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-02 | 421/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I399"/>
+  <dimension ref="A1:I422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19169,6 +19169,1087 @@
         </is>
       </c>
     </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>CHI-20260702-001</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>打不起精神</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>dǎ bù qǐ jīngshen</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>기운이 나지 않다, 의욕이 없다, 축 처지다</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>고등학교 3학년 때 친구가 중요한 시험에서 실리한 후, "요즘 계속 打不起精神, 아무것도 하고 싶지 않아"라고 말했다.</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>昨天通宵加班，今天早上我一直打不起精神。</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>CHI-20260702-002</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>排期</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>páiqī</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>(일정/계획을) 잡다, 스케줄을 짜다, 일정을 배정하다</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>민박집의 주문이 너무 많아서 6개월 후까지 '排期'되었다.</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>下个月的会议排期已经确定了吗？</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>CHI-20260702-003</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>涌入</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>yǒngrù</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>(사람/물자/감정 등이) 물밀듯이 밀려들다, 쇄도하다</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>수능 고득점 소녀에게 사방에서 사랑과 관심이 '涌入'했다.</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>旅游旺季，大量游客涌入这座小城。</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>CHI-20260702-004</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>回归</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>huíguī</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>(원래의 상태/위치로) 돌아가다, 복귀하다, 회귀하다</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>소녀와 그 가족이 '回归'하여 평온한 삶을 살 수 있기를 희망한다.</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>经历了多年的漂泊，他终于决定回归故里。</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>CHI-20260702-005</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>盘活</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>pánhuó</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>(죽은 자산/자원 등을) 활용하다, 활성화시키다</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>226.9억 위안의 자산 '盘活'의 배경에 충칭이 있다.</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>如何盘活闲置资产，是公司当前面临的重要课题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>CHI-20260702-006</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>响应</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>xiǎngyìng</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>(요청/호소에) 응답하다, 호응하다, 따르다</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>린스정장맞춤 린징판 울트라가 공식 출시되어 시장의 요구에 '响应'했다.</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>公司积极响应国家号召，支持环保事业。</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>CHI-20260702-007</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>违规</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>wéiguī</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>규정을 위반하다, 규칙을 어기다</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>친양시 직업교육센터가 '违规' 학생에게 요금을 부과하여 벌금을 받았다.</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>任何违规操作都将受到严厉处罚。</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>CHI-20260702-008</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>罚款</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>fákuǎn</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>벌금을 부과하다, 벌금을 내다</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>광저우 도시직업기술학교가 '违规毁绿'으로 9.8만 위안의 '罚款'을 받았다.</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>他因为超速驾驶被交警罚款了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>CHI-20260702-009</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>砍伐</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>kǎnfá</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>(나무를) 베다, 벌채하다</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>광저우 도시직업기술학교가 22그루의 나무를 '擅自砍伐'하여 벌금을 받았다.</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>保护森林资源，禁止随意砍伐树木。</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>CHI-20260702-010</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>争先恐后</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>zhēngxiān kǒnghòu</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>앞을 다투다, 서로 먼저 하려고 경쟁하다</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>수능 고득점 소식에 학생들이 경쟁적으로 성적을 확인하려고 '争先恐后'로 몰려들었다.</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>演唱会门票一开售，粉丝们便争先恐后地抢购。</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>CHI-20260702-011</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>精打细算</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>jīngdǎ xìsuàn</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>꼼꼼하게 계산하다, 절약하다, 알뜰하다</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>넉넉하지 못한 가정에서 가족들이 '精打细算'하며 생활비를 아꼈다.</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>过日子要精打细算，才能把钱花在刀刃上。</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>CHI-20260702-012</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>人山人海</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>rénshān rénhǎi</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>인산인해, 사람들로 붐비다</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>'出圈'한 민박집에는 주말마다 '人山人海'의 관광객이 몰렸다.</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>节假日期间，热门景点总是人山人海。</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>CHI-20260702-013</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>一鸣惊人</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>yīmíng jīngrén</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>한 번에 세상 사람들을 놀라게 하다, 일약 유명해지다</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>수능 고득점 소녀는 '一鸣惊人'하여 전국적인 화제가 되었다.</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>他平时默默无闻，没想到在这次比赛中一鸣惊人，获得了冠军。</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>CHI-20260702-014</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>不虚此行</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>bù xū cǐ xíng</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>헛걸음하지 않았다, 온 보람이 있다, 기대 이상이었다</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>아름다운 시골 민박집에 방문한 모든 손님들이 '不虚此行'이라고 칭찬했다.</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>这次旅行不仅欣赏了美景，还体验了当地文化，真是不虚此行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>CHI-20260702-015</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>爱不释手</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>ài bù shì shǒu</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>너무 좋아서 손에서 놓을 수 없다, 애지중지하다</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>'순환 상점'의 독특한 분위기와 상품에 젊은이들이 '爱不释手'했다.</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>这本小说太精彩了，我拿到手里就爱不释手。</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>CHI-20260702-016</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>独当一面</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>dú dāng yī miàn</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>한 가지 일을 책임지고 처리하다, 독자적으로 맡아서 하다</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>이 대학 졸업생들은 빠르게 성장하여 사회에서 '独当一面'할 수 있는 인재가 되었다.</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>经过几年的锻炼，他已经能够独当一面，负责整个项目了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>CHI-20260702-017</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>擦肩而过</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>cājiān'érgùo</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>스쳐 지나가다, 아깝게 놓치다, 인연이 닿지 않다</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>그녀는 고득점 기회를 아깝게 '擦肩而过'했지만, 다른 길을 찾아 성공했다.</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>我本来有机会出国留学，可惜因为一些原因和那个机会擦肩而过了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>CHI-20260702-018</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>四面八方</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>sì miàn bā fāng</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>사방팔방, 모든 곳에서, 여기저기서</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>四面八方的爱心涌向这个拮据的小家。</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>世界各地的游客从四面八方赶来，只为一睹这座古城的风采。</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>CHI-20260702-019</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>拮据</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>형용사</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>jié jū</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>경제적으로 곤궁하다, 빠듯하다</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>四面八方的爱心涌向这个拮据的小家。</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>因为失业，他们家的经济状况一直很拮据，生活压力很大。</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>CHI-20260702-020</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>万家灯火</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>wàn jiā dēng huǒ</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>만가의 불빛, 도시의 휘황찬란한 야경 (가정의 평화로운 모습 비유)</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>亮化工程点亮迪庆高原村寨万家灯火。</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>站在山顶俯瞰，城市里万家灯火，一片温馨祥和的景象。</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>CHI-20260702-021</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>填报志愿</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>tián bào zhì yuàn</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>(진학) 지원서를 작성하다, 지원 학교/학과를 기입하다</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>为帮助考生更科学地填报志愿，小编整理了中南林业科技大学...</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>高考结束后，如何科学合理地填报志愿成了考生和家长最关心的问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>CHI-20260702-022</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>急需</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>jí xū</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>급히 필요하다, 절실히 요구되다</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>近三年学校深耕国家战略急需领域，仅材料科学与工程学院...</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>灾区目前急需医疗物资和干净的饮用水。</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>CHI-20260702-023</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>登攀</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>dēng pān</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>등반하다, 높은 곳을 오르다 (목표 달성, 발전 등을 비유)</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>十年德润，三度登攀：一所高中的“阶梯成长”育人样本。</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>他一生都在科学的高峰上不断登攀，为人类进步做出了巨大贡献。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-03 | 443/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I422"/>
+  <dimension ref="A1:I444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20250,6 +20250,1040 @@
         </is>
       </c>
     </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>CHI-20260703-001</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>不堪纷扰</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>bù kān fēn rǎo</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>번거로움/소란을 견딜 수 없다, 시달림을 감당하기 어렵다</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>高考 699점 소녀는四面八方的爱心에不堪纷扰，평온한 생활을 원한다고 밝혔습니다.</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>媒体的过度关注让他的家人不堪纷扰，不得不搬家。</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>CHI-20260703-002</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>回归平静</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>huí guī píng jìng</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>평온함을 되찾다, 조용한 일상으로 돌아가다</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>이 소녀와 가족이 다시回归平静生活하기를 바랍니다.</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>经历了一段混乱后，他终于回归平静，开始新的生活。</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>CHI-20260703-003</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>志愿填报</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>zhì yuàn tián bào</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>(대학, 학과) 지원서를 작성하다, 원서 접수를 하다</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>길림성에서高考志愿填报에 관한 중요 공지가 발표되었습니다.</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>今年的志愿填报规则有些变化，得仔细研究一下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>CHI-20260703-004</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>辞职</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>cí zhí</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>사직하다, 퇴직하다, 그만두다</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>그는 새로운 도전을 위해 갑자기 회사에 辞职을 통보했다.</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>我正在考虑辞职，寻找一个更适合自己的工作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>CHI-20260703-005</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>打招呼</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>dǎ zhāo hu</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>인사하다, 안부를 묻다, 미리 언질을 주다</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>아침에 옆집 사람과 마주쳐서 가볍게 打招呼했어요.</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>你见到李经理的时候，记得替我跟他打个招呼。</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>CHI-20260703-006</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>蹭热度</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>cèng rè dù</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>인기에 편승하다, 화제에 묻어가다, 이슈에 편승해 홍보하다</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>어떤 브랜드들은 유명인사의 스캔들을 이용해 蹭热度를 시도하기도 한다.</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>这家公司总喜欢蹭热度，发布一些跟风的产品。</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>CHI-20260703-007</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>扎心</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>zhā xīn</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>마음을 찌르다, 가슴 아프다, 뼈 때리다 (직역: 심장을 찌르다)</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>그가 무심코 던진 한마디가 나에게 정말 扎心하게 다가왔어.</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>老板说我工作效率低，这句话真是太扎心了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>CHI-20260703-008</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>发财</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>fā cái</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>돈을 벌다, 부자가 되다</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>“你只是高考完了，不是家里发财了”，戳中了谁？</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>新年快乐，恭喜发财！希望你今年事业顺利，财源广进。</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>CHI-20260703-009</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>登记</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>dēng jì</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>등록하다, 등기하다</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>振芯科技完成工商变更登记 法定代表人变更为董事长梁...</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>参观前请您在入口处进行登记。</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>CHI-20260703-010</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>亮相</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>liàng xiàng</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>(공개적으로) 모습을 드러내다, 등장하다</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>建发集团亮相2026年APEC工商领导人中国论坛，...</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>新产品将在下个月的发布会上正式亮相。</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>CHI-20260703-011</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>正能量</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>zhèng néng liàng</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>긍정적인 에너지, 좋은 기운</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>高考606分的脑瘫男孩 获1万元天天正能量...</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>他总是给身边的人带来正能量，大家都很喜欢他。</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>CHI-20260703-012</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>对外表示</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>duì wài biǎo shì</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>대외적으로 표명하다, 외부에 밝히다</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>女孩和家长已通过大象新闻记者对外表示，感谢大家善意、爱心，目前不再接受探视、采访...</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>公司对外表示，将加大对环保项目的投入，履行企业社会责任。</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>CHI-20260703-013</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>访华</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>fǎng Huá</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>중국을 방문하다</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>纳米比亚总统恩代特瓦将访华，外交部介绍有关安排.</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>美国总统明年将访华，两国关系有望改善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>CHI-20260703-014</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>回应</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>huí yìng</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>응답하다, 회신하다</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>档案可以本人转递吗？人社部回应.</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>面对媒体的质疑，公司迅速做出了回应。</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>CHI-20260703-015</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>披露</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>pī lù</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>(비밀 등을) 폭로하다, 공표하다</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>胜百携智控发布2025 ESG报告，披露双项碳核查...</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>公司定期披露财务报表以增加透明度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>CHI-20260703-016</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>失利</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>shī lì</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>실패하다, 패배하다</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>高考失利后，她用民宿“考”出千万营收：人生不必被分...</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>尽管在比赛中失利了，但他并没有放弃，决定继续努力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>CHI-20260703-017</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>涌向</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>yǒng xiàng</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>쇄도하다, (어딘가로) 밀려들다</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>四面八方的爱心涌向这个拮据的小家。</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>灾情发生后，无数志愿者和物资涌向灾区。</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>CHI-20260703-018</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>引领</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>yǐn lǐng</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>선도하다, 이끌다</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>“环保铁军”以党建“红”引领生态“绿”.</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>科技创新引领着社会发展，改变着人们的生活方式。</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>CHI-20260703-019</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>突破</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>tū pò</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>돌파하다, (난관을) 극복하다</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>低品位钛铁尾矿资源化获新突破 恒誉环保原创技术达国...</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>科学家们在癌症治疗方面取得了重大突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>CHI-20260703-020</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>出台</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>chū tái</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>(정책, 법안 등이) 발표되다, 나오다</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>中方最近出台的民族法案是否有涉外权限，外交部：敦促...</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>新的经济政策即将出台，预计会对市场产生积极影响。</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>CHI-20260703-021</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>敦促</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>dūn cù</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>촉구하다, 재촉하다</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>外交部：敦促...</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>国际社会敦促有关各方保持克制，通过对话解决争端。</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>CHI-20260703-022</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>诋毁</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>dǐ huǐ</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>훼손하다, 비방하다</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>外交部：坚决反对有关国家恶意诋毁中国民族政策.</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>这些毫无根据的报道都是对公司声誉的恶意诋毁。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-06 | 468/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I444"/>
+  <dimension ref="A1:I469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21284,6 +21284,1181 @@
         </is>
       </c>
     </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>CHI-20260706-001</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>面试</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>miàn shì</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>면접을 보다</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>明天有一个很重要的面试。</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>我面试了三家公司，终于拿到offer了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>CHI-20260706-002</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>升职</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>shēng zhí</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>승진하다</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>恭喜你升职加薪！</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>他工作表现很好，很快就升职了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>CHI-20260706-003</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>充电</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>이합사 / 구어</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>chōng diàn</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>충전하다 (물리적/비유적), (지식·기술 등을) 배우다, 재충전하다</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>我准备利用周末时间多充电，学习新技能。</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>最近太累了，需要好好休息充电。</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>CHI-20260706-004</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>人脉</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>rén mài</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>인맥</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>在商业领域，人脉非常重要。</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>他通过广泛的人脉找到了很多合作机会。</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>CHI-20260706-005</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>情商</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>qíng shāng</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>정서 지능 (EQ)</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>高情商的人更懂得如何与人沟通。</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>情商比智商在某些时候更重要。</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>CHI-20260706-006</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>金榜题名</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>jīn bǎng tí míng</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>과거에 급제하다, 시험에 합격하다 (특히 높은 성적으로)</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>祝愿所有考生金榜题名，前程似锦！</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>他高考金榜题名，考上了理想的大学。</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>CHI-20260706-007</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>名落孙山</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>míng luò sūn shān</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>시험에 떨어지다, 낙방하다</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>虽然这次名落孙山，但他没有放弃。</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>他担心自己高考会名落孙山。</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>CHI-20260706-008</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>啃老</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>kěn lǎo</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>부모에게 기대어 살다, 부모 등골 빼먹다</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>大学毕业后他一直啃老，不找工作。</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>现代社会啃老族越来越多，引发了社会讨论。</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>CHI-20260706-009</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>弹眼落睛</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>tán yǎn luò jīng</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>매우 눈길을 끈다, 시선을 사로잡는다 (주로 시각적으로)</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>她的简历上，一长串技能资格证书可谓弹眼落睛。</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>那件衣服设计独特，真是弹眼落睛。</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>CHI-20260706-010</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>背锅</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>bēi guō</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>책임을 뒤집어쓰다, 덤터기 쓰다</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>这次的失误不是我的错，我不想背锅。</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>为了团队利益，他只能选择背锅。</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>CHI-20260706-011</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>破防</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>pò fáng</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>(감정적으로) 무너지다, 멘탈이 나가다, 방어선이 뚫리다</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>看到那个感人的视频，我瞬间破防了。</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>他被批评后，心里有点破防了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>CHI-20260706-012</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>风雨兼程</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>fēng yǔ jiān chéng</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>비바람을 무릅쓰고 (목표를 향해) 나아가다; 어려운 역경을 이겨내고 꾸준히 노력하다</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>“共和国长子们”一路风雨兼程，才有了今天的成就。</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>创业初期，我们团队风雨兼程，终于把公司做起来了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>CHI-20260706-013</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>校正方向</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>jiào zhèng fāng xiàng</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>방향을 바로잡다, 방향을 수정하다</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>不是再来一年，是校正方向！我们需要从根本上解决问题。</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>市场变化太快，公司战略需要及时校正方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>CHI-20260706-014</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>落下帷幕</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>luò xià wéi mù</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>막을 내리다, 끝나다, 종결되다</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>2026年高考落幕，新的人生篇章即将开启。</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>经过几天的激烈角逐，本次国际会议也终于落下帷幕。</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>CHI-20260706-015</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>思维惯性</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>sī wéi guàn xìng</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>사고 관성, 생각하는 습관</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>失分不是因为知识储备不够，而是思维惯性导致审题偏差。</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>有时候，思维惯性会让我们错过新的机会和视角。</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>CHI-20260706-016</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>错位</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>cuò wèi</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>어긋남, 착오; (제자리에서) 벗어나다, 어긋나다</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>思维惯性与新命题导向之间的错位，导致了答题失误。</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>部门之间的职责错位经常导致工作效率低下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>CHI-20260706-017</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>审议通过</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>shěn yì tōng guò</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>심의하여 통과시키다, 검토 후 가결하다</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>董事会审议通过了修订公司章程的议案。</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>提案在全体员工大会上经过充分讨论，最终被审议通过。</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>CHI-20260706-018</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>印发</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>yìn fā</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>인쇄하여 배포하다, 인쇄하여 발송하다</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>国家发改委印发了《循环经济发展“十五五”规划》。</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>会议结束后，秘书处将会议纪要印发给了所有与会者。</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>CHI-20260706-019</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>上车</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>shàng chē</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>(버스나 차에) 타다; (사업, 기회 등에) 합류하다, 참여하다</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>38个机会，5家国企等你“上车”！</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>这个项目前景很好，现在“上车”还来得及。</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>CHI-20260706-020</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>公示</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>gōng shì</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>공시하다, 공포하다, 대중에게 알리다</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>人社部公示了12个新职业及多个新工种。</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>公司的招聘结果将在下周一进行公示。</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>CHI-20260706-021</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>常态化</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>cháng tài huà</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>상시화하다, 정상화하다, 일상적인 것으로 만들다</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>济南常态化调研市属国企，精准画像选良将。</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>疫情后，远程办公逐渐成为公司的一种常态化工作模式。</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>CHI-20260706-022</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>精准画像</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>jīng zhǔn huà xiàng</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>정밀 분석/묘사, (데이터 기반의) 정확한 프로파일링</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>通过精准画像，可以为人才选拔提供更好的依据。</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>为了提高营销效果，公司需要对目标客户进行精准画像。</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>CHI-20260706-023</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>叫停</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>jiào tíng</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>중지시키다, 중단 명령을 내리다</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>叫停奢华录取通知书，是高校重建定力的一部分。</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>政府部门及时叫停了未经审批的建设项目。</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>CHI-20260706-024</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>含金量</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>hán jīn liàng</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>금 함량; (비유적으로) 가치, 실질적인 내용</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>这所高校含金量拉满，非常值得报考。</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>这份证书的含金量很高，对找工作非常有帮助。</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>CHI-20260706-025</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>加码</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>jiā mǎ</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>(도박에서) 판돈을 올리다; (비유적으로) 강도를 높이다, 투자를 늘리다</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>稳投资持续加码，促进经济发展。</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>为了尽快完成项目，团队决定加班加码。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-07 | 489/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I469"/>
+  <dimension ref="A1:I490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22459,6 +22459,993 @@
         </is>
       </c>
     </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>CHI-20260707-001</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>说话</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>shuō huà</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>말하다, 이야기하다</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>회의 중에 크게 말하는 것을 조심해야 해요. (开会时要注意，不要大声说话。)</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>你有什么话想说就直接说吧，别憋着。</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>CHI-20260707-002</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>水土不服</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>shuǐ tǔ bù fú</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>새로운 환경에 적응하지 못하다, 풍토병에 걸리다</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>그는 새로운 도시에 온 후 계속 水土不服해서 좀 힘들어해요. (他来到新城市后一直水土不服，有点难受。)</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>我刚到这个城市的时候，因为水土不服生了一场病。</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>CHI-20260707-003</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>卷</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>juǎn</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>과도한 경쟁에 시달리다, 치열하게 경쟁하다</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>요즘 대입 경쟁이 너무 卷이라 학생들이 스트레스를 많이 받아요. (现在高考竞争太卷了，学生们压力很大。)</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>我们这个行业太卷了，大家都在拼命加班。</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>CHI-20260707-004</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>拉满</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>lā mǎn</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>최대한으로 하다, 꽉 채우다, 극대화하다</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>이 학교는 교육의 含金量을 拉满해서 학생들이 아주 만족해요. (这所高校含金量拉满，学生们都很满意。)</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>这次活动的热情度直接拉满，大家都玩得很开心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>CHI-20260707-005</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>释放潜力</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>shì fàng qián lì</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>잠재력을 발휘하다, 잠재력을 끌어내다</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>暑期释放消费潜力！</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>公司鼓励员工释放潜力，积极创新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>CHI-20260707-006</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>打探家底</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>dǎ tàn jiā dǐ</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>(주로 몰래) 집안 배경/재력/속내를 알아보다</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>新生入学查家长职务和车型，打探家底是对教育公...</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>他总是喜欢打探别人的家底，让人很不舒服。</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>CHI-20260707-007</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>梳理</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>shū lǐ</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>(정리되지 않은 것을) 정리하다, 검토하다, 분류하다</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>网警梳理了4个“高考查分陷阱”，家有考生的速看！</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>请你把最近的工作内容梳理一下，明天会上汇报。</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>CHI-20260707-008</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>肄业</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>yì yè</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>(학업을 마치지 못하고) 수료하다, 학업을 중단하다 (졸업은 못함)</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>人大博士肄业宅家六年靠父母供养，曾进入职场难以适应...</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>他因为家庭原因，大学本科肄业了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>CHI-20260707-009</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>宅家</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>zhái jiā</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>집에서 지내다, 방콕하다</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>人大博士肄业宅家六年靠父母供养...</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>周末我只想宅家，看看电影，放松一下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>CHI-20260707-010</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>被看见</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>bèi kàn jiàn</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>(노력이나 가치가) 인정받다, 주목받다</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>城市如何被看见？</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>很多年轻设计师渴望自己的作品能被更多人看见。</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>CHI-20260707-011</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>辨别</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>biàn bié</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>식별하다, 분별하다, 구별하다</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>怎么辨别板材环保等级？</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>消费者应该学会辨别产品的真伪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>CHI-20260707-012</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>奉行</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>fèng xíng</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>(정책, 원칙 등을) 견지하다, 고수하다, 받들어 행하다</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>4国明确坚定奉行一个...</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>我国一贯奉行和平共处五项原则的外交政策。</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>CHI-20260707-013</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>聚力</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>jù lì</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>(힘, 역량을) 한데 모으다, 결집하다</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>青春聚力反诈护航...</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>团队成员们聚力攻坚，终于克服了技术难题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>CHI-20260707-014</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>汇总</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>huì zǒng</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>종합하다, 총괄하다, 취합하다</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>21个投档录取问题汇总。</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>请你把各部门的意见汇总一下，形成一份报告。</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>CHI-20260707-015</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>录取</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>lù qǔ</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>(학교, 회사 등에) 합격시키다, 뽑다</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>21个投档录取问题汇总。</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>他凭借优异的成绩被北京大学录取了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>CHI-20260707-016</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>开展</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>kāi zhǎn</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>(활동, 사업 등을) 전개하다, 벌이다, 진행하다</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>聊城市特殊教育学校开展防溺水安全教育系列活动。</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>学校将开展一系列丰富多彩的课外活动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>CHI-20260707-017</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>预防</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>yù fáng</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>예방하다, 막다</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>聊城市特殊教育学校开展防溺水安全教育系列活动。</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>冬季要特别注意预防感冒。</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>CHI-20260707-018</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>转型</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>zhuǎn xíng</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>(구조, 업종 등을) 전환하다, 변모하다</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>从“军营绿”到“生态绿” 宜昌这位环保尖兵获国家级...</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>随着科技发展，许多传统产业都在积极转型。</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>CHI-20260707-019</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>带头</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>dài tóu</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>앞장서다, 솔선수범하다, 선두에 서다</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>从“军营绿”到“生态绿” 宜昌这位环保尖兵获国家级...</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>经理总是带头加班，给员工树立了榜样。</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>CHI-20260707-020</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>供养</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>gōng yǎng</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>부양하다, 봉양하다, (음식 등으로) 공급하다</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>人大博士肄业宅家六年靠父母供养...</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>父母辛辛苦苦把我们供养长大，我们应该孝顺他们。</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>CHI-20260707-021</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>留下印象</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>liú xià yìn xiàng</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>인상을 남기다, 인상 깊게 하다</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>城市如何被看见？——评《中国当代城市电影与城市印象》</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>第一次见面，他给我留下了深刻的印象。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-08 | 506/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I490"/>
+  <dimension ref="A1:I507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23446,6 +23446,805 @@
         </is>
       </c>
     </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>CHI-20260708-001</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>闹乌龙</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>nào wū lóng</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>어처구니없는 실수를 하다, 해프닝을 벌이다</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>那个女孩本以为高考估分有715分，结果查出来才299分，原来是自己对错答案闹了场乌龙。</t>
+        </is>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>昨天开会我把新产品方案发错群了，真是闹了个大乌龙。</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>CHI-20260708-002</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>嚼舌根</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>jiáo shé gēn</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>뒷공론을 하다, 쓸데없는 험담을 하다</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>那些躲在屏幕背后的键盘侠，天天在网上嚼舌根、网暴高分女学生，真是令人气愤。</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>别在背后嚼舌根，有什么不满意的直接当面跟他说清楚。</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>CHI-20260708-003</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>拍脑门</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>pāi nǎo mén</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>충동적으로 판단하다, 주먹구구식으로 결정하다</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>暑假规划不能靠家长拍脑门决定，那种精确到分钟的日程表往往会让孩子产生逆反心理。</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>做市场决定不能只凭拍脑门，必须有真实可靠的数据支持才行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>CHI-20260708-004</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>连轴转</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>lián zhóu zhuàn</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>쉴 틈 없이 일하다, 쉬지 않고 (바쁘게) 돌아가다</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>高考刚结束，许多自媒体为了抢流量连轴转地做直播、写文章，制造了不少焦虑。</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>为了能在节前完成这批环保建材的交付，工厂的工人们已经连轴转了三天。</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>CHI-20260708-005</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>走过场</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>zǒu guò chǎng</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>형식적으로만 하다, 겉치레로 때우다</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>有些高考志愿填报培训班只是为了圈钱，发的一些所谓“官方证书”完全是在走过场，没有含金量。</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>这次的安全大检查必须严格落实，绝对不能敷衍了事、走过场。</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>CHI-20260708-006</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>挡箭牌</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>dǎng jiàn pái</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>핑계거리, 구실, 방패막이</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>那些网暴考生的自媒体，不能把“言论自由”当做伤害别人的挡箭牌。</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>每次迟到你都拿堵车当挡箭牌，大家早就听腻了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>CHI-20260708-007</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>挑刺</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>tiāo cì</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>꼬투리를 잡다, 트집을 잡다, 딴지를 걸다</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>女孩高考取得高分，却有一些自媒体在人家的志愿选择上挑刺，不断带节奏制造舆论。</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>他这个方案已经写得很完美了，你没必要为了挑刺而故意去挑刺。</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>CHI-20260708-008</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>帮倒忙</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>bāng dào máng</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>도우려다 오히려 해를 끼치다, 긁어 부스럼을 만들다</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>家长本来想帮孩子规划暑假，但如果盲目制定高强度作息表，反而是帮倒忙，让孩子更厌学。</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>我本来是想帮他洗碗的，结果把盘子打碎了，真是帮倒忙。</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>CHI-20260708-009</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>砸锅</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>zá guō</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>일을 그르치다, 망치다, 실패하다</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>高考志愿填报是一件大事，千万不能粗心大意导致砸锅，否则后悔莫及。</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>放心吧，这次的签约仪式我已经排练过很多次了，绝对不会砸锅的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>CHI-20260708-010</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>睁眼瞎</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>zhēng yǎn xiā</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>까막눈, 보고도 모르는 척하는 사람, 무지한 사람</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>网上很多网民不看客观事实，只跟着自媒体起哄，简直是睁眼瞎，跟风黑别人。</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>现在的智能设备虽然方便，但对不识字的老人来说，他们面对这些屏幕就像是睁眼瞎。</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>CHI-20260708-011</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>看热闹</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>kàn rè nao</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>구경꾼 노릇을 하다, 제삼자로서 불 구경하듯 구경하다</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>网上很多键盘侠并不是真的关心这件事，只是在看热闹。</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>遇到别人发生争执，我们不应该围在一起看热闹，而应该主动调解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>CHI-20260708-012</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>吃定心丸</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>chī dìng xīn wán</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>안심하다, 마음을 놓다</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>看到录取通知书的那一刻，焦虑了一整周的家长终于吃了定心丸。</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>医生的权威解释给焦急等待的患者家属吃了一颗定心丸。</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>CHI-20260708-013</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>避重就轻</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>bì zhòng jiù qīng</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>중요한 일(책임)은 피하고 가벼운 일만 다루다, 핵심을 회피하다</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>面对媒体关于环保超标的质问，该企业避重就轻，只谈公益捐款。</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>面对家长的投诉，培训机构负责人避重就轻，不肯正面回答问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>CHI-20260708-014</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>打马虎眼</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>dǎ mǎ hu yǎn</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>얼렁뚱땅 넘어가다, 눈가림하다, 시치미 떼다</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>别想在我面前打马虎眼，合同细节里的这些问题我看得清清楚楚。</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>环保督察非常严格，任何化工企业都别想在排污数据上打马虎眼。</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>CHI-20260708-015</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>干瞪眼</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>gān dèng yǎn</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>뻔히 보면서도 손을 쓰지 못하다, 안타까워하며 발만 동동 구르다</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>查分系统因为人数过多崩溃了，家长和考生在电脑前干瞪眼，毫无办法。</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>车子在半路没电了，附近又没有充电桩，我们只能坐在车里干瞪眼。</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>CHI-20260708-016</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>爆冷门</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>bào lěng mén</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>이변을 낳다, 예상 밖의 대성공(또는 실패)을 거두다</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>谁也没想到，今年高考全省第一名竟然是一所普通中学的学生，真是爆了冷门。</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>在昨晚的世界杯比赛中，名不见经传的小队击败了上届冠军，爆了大冷门。</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>CHI-20260708-017</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>出洋相</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>chū yáng xiàng</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>웃음거리가 되다, 망신살이 뻗치다, 실수를 저질러 창피를 당하다</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>出发前不做好防暑准备，到了海滩中暑晕倒，那可就要出洋相了。</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>填报志愿一定要反复核对学校代码，千万别因为一时粗心出了洋相。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-09 | 523/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I507"/>
+  <dimension ref="A1:I524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24245,6 +24245,805 @@
         </is>
       </c>
     </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>CHI-20260709-001</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>破局</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>구어 / 동사</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>pò jú</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>난국을 타개하다, 국면을 전환하다, 돌파구를 찾다</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>新疆兵团破局打造跨境物流枢纽新支点。</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>公司需要新的策略来破局，否则市场份额会继续下滑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>CHI-20260709-002</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>网暴</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>구어 / 동사</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>wǎng bào</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>(인터넷) 사이버 폭력을 가하다, 악성 댓글을 달다</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>高考699分女孩报清华却被网暴，到底是谁在替她“不...</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>这种行为属于网暴，我们应该抵制并保护受害者。</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>CHI-20260709-003</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>放飞自我</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>구어 / 관용구</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>fàngfēi zìwǒ</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>자신을 해방하다, 마음껏 자유롭게 하다, 거리낌 없이 행동하다</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>另一种是彻底放飞，作息全凭“随缘”。</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>暑假到了，孩子们终于可以放飞自我，尽情玩耍了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>CHI-20260709-004</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>随缘</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>구어 / 동사 / 형용사</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>suí yuán</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>인연에 따르다, 운명에 맡기다, 될 대로 되라</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>另一种是彻底放飞，作息全凭“随缘”。</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>很多事情不必强求，随缘就好。</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>CHI-20260709-005</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>发愁</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>fā chóu</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>걱정하다, 근심하다, 한숨 쉬다</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>开学陡增焦虑。(개학이 다가와 걱정이 늘어나는 맥락과 관련)</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>孩子学习成绩不好，妈妈很发愁。</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>CHI-20260709-006</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>掉链子</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>구어 / 관용구</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>diào liànzi</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>(중요한 순간에) 실수하다, 망치다, 문제가 생기다, (일이) 틀어지다</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>중요한 순간에 예기치 않은 문제로 일이 틀어지는 상황</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>关键时刻他掉链子了，导致整个计划失败。</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>CHI-20260709-007</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>苦尽甘来</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>관용구 / 성어</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>kǔ jìn gān lái</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>고생 끝에 낙이 오다, 고진감래</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>그녀는 3년간의 고된 노력으로 꽃을 피웠다(换一场花开). (힘든 과정을 거쳐 좋은 결과를 얻는 맥락과 관련)</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>经历了这么多困难，我相信我们很快就能苦尽甘来了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>CHI-20260709-008</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>力挽狂澜</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>lì wǎn kuáng lán</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>급변하는 상황을 되돌리다, 위기에서 벗어나다</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>상하이 국유기업의 대규모 구조조정 및 새로운 물류 허브 구축 시도와 같이 어려운 상황을 반전시키는 맥락</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>在公司面临危机时，他临危受命，力挽狂澜，使公司转危为安。</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>CHI-20260709-009</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>按部就班</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>àn bù jiù bān</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>순서대로 하다, 절차에 따라 진행하다</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>여름방학을 세 단계로 나누어 계획하는 것처럼, 어떤 일을 계획에 따라 체계적으로 진행하는 맥락</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>新项目的启动需要我们按部就班，一步一个脚印地去完成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>CHI-20260709-010</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>事半功倍</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>shì bàn gōng bèi</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>적은 노력으로 큰 효과를 거두다</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>고품질 발전, 안정적인 투자 등의 목표 달성을 위해 효율적인 방법론을 찾는 맥락</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>掌握了正确的方法，学习就能事半功倍，效率大大提高。</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>CHI-20260709-011</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>任重道远</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>rèn zhòng dào yuǎn</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>책임이 막중하고 갈 길이 멀다</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>국가급 도시권 27개 구축, 빈곤 퇴치 이야기, 또는 주요 직책 임명과 같이 막중한 책임과 긴 여정을 암시하는 맥락</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>作为新上任的部门经理，他深知自己任重道远，需要付出更多努力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>CHI-20260709-012</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>举足轻重</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>jǔ zú qīng zhòng</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>아주 중요하여 결정적인 영향을 끼치다</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>국무원 부부장이나 연구회 회장직, 또는 국경 간 물류 허브와 같이 중요하고 영향력 있는 위치나 역할을 설명하는 맥락</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>在这个团队中，他的意见举足轻重，常常能影响最终的决策。</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>CHI-20260709-013</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>名副其实</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>míng fù qí shí</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>명실상부하다, 이름과 실제가 부합하다</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>친환경 건축 자재 브랜드 추천, '공화국의 장자'와 같은 호칭이 실제 내용과 부합함을 강조하는 맥락</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>他被誉为“厨艺大师”，今晚尝了他的菜，果然名副其实。</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>CHI-20260709-014</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>无微不至</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>wú wēi bù zhì</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>극진하다, 세심하게 돌보다</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>'가장 아름다운 이모'가 도움을 준 사례, 또는 청춘의 길을 지키기 위한 보호 노력처럼 매우 세심하고 극진하게 돌보는 맥락</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>父母对孩子的爱总是无微不至的，关心着他们成长的每一个细节。</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>CHI-20260709-015</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>当务之急</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>dāng wù zhī jí</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>당면한 급선무, 가장 시급한 일</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>하반기 투자 안정화 방안 모색, '두 가지 중대한 건설 프로젝트'의 전면 시행과 같이 가장 시급하고 중요한 과제를 설명하는 맥락</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>公司的资金链出现了问题，解决燃眉之急是我们的当务之急。</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>CHI-20260709-016</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>独树一帜</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>dú shù yī zhì</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>독자적인 경지를 개척하다, 독특한 스타일을 형성하다</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>친환경 보드 재료의 구조적 돌파구 마련, 고품질 발전 추구와 같이 자신만의 독특한 스타일이나 사상 체계를 형성하여 특별한 존재감을 드러내는 맥락</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>这位艺术家的作品风格独树一帜，深受年轻人的喜爱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>CHI-20260709-017</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>后顾之忧</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>hòu gù zhī yōu</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>뒷걱정, 미래나 가정에 대한 걱정거리</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>국유기업 직원들이 '철밥통'을 포기하는 상황, 고3 학부모의 ICU 입원과 같이 미래나 가정에 대한 걱정거리를 언급하는 맥락</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>只要解决了员工的后顾之忧，他们才能全身心地投入到工作中。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-10 | 538/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I524"/>
+  <dimension ref="A1:I539"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25044,6 +25044,711 @@
         </is>
       </c>
     </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>CHI-20260710-001</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>批复</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>pī fù</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>승인하다, 허가하다 (주로 정부나 상급기관에서 공식적으로)</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>黔江至吉首铁路项目可研报告获国家发改委批复。</t>
+        </is>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>我们的申请材料已经提交，正在等待上级批复。</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>CHI-20260710-002</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>迈入</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>mài rù</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>진입하다, (어떤 단계/시기로) 들어서다</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>高铁项目推进迈入全新阶段，对当地经济发展意义重大。</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>随着科技进步，人类社会正迈入一个全新的数字化时代。</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>CHI-20260710-003</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>性价比</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>xìng jià bǐ</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>가격 대비 성능, 가성비</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>乳胶漆哪个品牌性价比高还环保？这是消费者关心的问题。</t>
+        </is>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>这款手机配置高，价格合理，性价比非常不错。</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>CHI-20260710-004</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>两全其美</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>liǎng quán qí měi</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>두 가지를 모두 만족시키다, 양쪽 다 좋게 만들다</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>如何平衡工作与生活，做到两全其美，是现代人的课题。</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>我们想找到一个既能省钱又能环保的两全其美的方案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>CHI-20260710-005</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>大显身手</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>dà xiǎn shēn shǒu</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>실력을 유감없이 발휘하다, 솜씨를 마음껏 뽐내다</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>这次比赛为他提供了一个大显身手的机会。</t>
+        </is>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>新来的经理很有能力，相信他会在公司大显身手。</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>CHI-20260710-006</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>刻不容缓</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>kè bù róng huǎn</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>한시도 지체할 수 없다, 각박하다, 시급하다</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>灾后应急恢复工作刻不容缓，必须争分夺秒。</t>
+        </is>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>环境保护问题刻不容缓，我们必须立即采取行动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>CHI-20260710-007</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>胸有成竹</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>xiōng yǒu chéng zhú</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>미리 계획이 서 있거나 승산이 있어 자신감이 있다</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>이번 프레젠테이션은 팀원들과 철저히 준비했기 때문에, 발표자는 흉유성죽한 태도로 연단에 올랐다.</t>
+        </is>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>面对即将到来的谈判，他显得胸有成竹，因为他已经预料到了所有可能的问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>CHI-20260710-008</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>临阵磨枪</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>lín zhèn mó qiāng</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>싸움터에 나가서야 총칼을 갈다; 닥쳐서야 허둥지둥 준비하다 (벼락치기)</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>시험이 코앞인데 이제 와서 임진마창하는 건 소용없다. 평소에 꾸준히 공부했어야 했다.</t>
+        </is>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>他平时不努力，每次考试都临阵磨枪，结果总是差强人意。</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>CHI-20260710-009</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>提心吊胆</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>tí xīn diào dǎn</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>마음을 졸이다, 불안해하다, 노심초사하다</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>시험 결과 발표를 기다리는 동안, 학생들은 모두 제심조담하며 초조하게 기다렸다.</t>
+        </is>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>秘密任务执行期间，队员们都提心吊胆，生怕出现任何差错。</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>CHI-20260710-010</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>大局为重</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>dà jú wéi zhòng</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>큰 틀을 중시하다, 대의를 중요하게 여기다</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>개인적인 감정보다는 단체 전체의 이익을 고려하여, 다국위중하게 행동해야 한다.</t>
+        </is>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>在讨论薪资调整时，大家一致认为应以公司发展的大局为重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>CHI-20260710-011</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>集思广益</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>jí sī guǎng yì</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>여러 사람의 의견을 모아 이점을 취하다 (집단 지성을 발휘하다)</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>새로운 마케팅 전략을 세우기 위해, 우리는 팀 회의를 열어 집사광익하기로 했다.</t>
+        </is>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>为了解决这个技术难题，项目组决定集思广益，听取不同部门的建议。</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>CHI-20260710-012</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>加班加点</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>jiā bān jiā diǎn</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>야근하고 추가 근무하다</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>프로젝트 마감일이 임박하여, 모든 팀원들이 밤늦게까지 야근가점을 하며 노력하고 있다.</t>
+        </is>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>为了确保按时完成订单，工人们这几天都在加班加点地生产。</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>CHI-20260710-013</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>居安思危</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>jū ān sī wēi</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>편안할 때도 위험을 생각하다 (미리 대비하다)</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>지금은 비록 안정적이지만, 우리는 항상 주안사위하며 미래의 도전에 대비해야 한다.</t>
+        </is>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>一个成功的企业必须居安思危，不断创新才能在市场中立于不败之地。</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>CHI-20260710-014</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>百废待兴</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>bǎi fèi dài xīng</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>모든 폐허가 재건되기를 기다리다 (모든 일이 황폐해져서 다시 시작해야 할 때)</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>지진 피해 후 도시는 백폐대흥 상태였지만, 주민들은 용기를 잃지 않고 재건을 시작했다.</t>
+        </is>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>战后的城市一片狼藉，百废待兴，重建工作刻不容缓。</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>CHI-20260710-015</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>言行一致</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>yán xíng yī zhì</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>말과 행동이 일치하다</t>
+        </is>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>리더는 언제나 언행일치해야만 직원들의 신뢰를 얻을 수 있다.</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>他的优点是言行一致，说到做到，所以大家都非常信任他。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-13 | 562/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I539"/>
+  <dimension ref="A1:I563"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25749,6 +25749,1134 @@
         </is>
       </c>
     </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>CHI-20260713-001</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>绽放</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>zhànfàng</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>(꽃이) 만개하다, (재능/잠재력이) 활짝 피어나다</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>深耕美育润童心 潜心育人绽芳华.</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>经过多年的努力，她的设计才华终于在国际舞台上绽放。</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>CHI-20260713-002</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>标杆</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>biāogān</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>(업계/분야의) 기준, 모범이 되는 모델, 벤치마크</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>以先进为标杆、以榜样为力量！金沙双星社区表彰优秀高...</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>这家公司是行业内的标杆企业，值得我们学习。</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>CHI-20260713-003</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>规划</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>동사/명사</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>guīhuà</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>계획하다, 기획하다 (동사); 계획, 기획 (명사)</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>《美丽中国建设“十五五”规划》开出财金“药方”.</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>我们正在规划明年的市场推广方案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>CHI-20260713-004</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>捡起来</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>동사구</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>jiǎn qǐ lái</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>(중단했던 습관/취미 등을) 다시 시작하다, 다시 배우다</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>每天上午还会弹一个小时左右的琴——“把过去的爱好重新捡起来。”</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>工作忙了很久，终于有时间把荒废的英语重新捡起来了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>CHI-20260713-005</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>得心应手</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>déxīn yìngshǒu</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>마음먹은 대로 되다, 익숙해서 손쉽다, 능숙하다</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>童心巧手绘环保. ('巧手'에서 능숙함의 의미를 유추)</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>经过一段时间的练习，他现在操作这台机器已经得心应手了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>CHI-20260713-006</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>充充电</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>이합사/구어</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>chōng chōng diàn</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>(지식이나 에너지 등을) 재충전하다, 새로운 것을 배우다</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>暑假尝试“三段式”过法：孩子不累，开学不慌. (방학 중 재충전의 맥락)</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>忙碌了一周，周末我想好好在家充充电，看看书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>CHI-20260713-007</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>发表讲话</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>fābiǎo jiǎnghuà</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>연설/담화를 발표하다</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>国家主席习近平将出席大会开幕式并发表主旨讲话。</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>会议主席在开幕式上发表了热情洋溢的讲话。</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>CHI-20260713-008</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>整体情况</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>zhěngtǐ qíngkuàng</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>전반적인 상황, 전체적인 개요</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>外交部发言人林剑13日在例行记者会上介绍大会整体情况。</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>请你向大家介绍一下项目的整体情况和目前遇到的挑战。</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>CHI-20260713-009</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>表态</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>biǎo tài</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>태도를 표명하다, 입장을 밝히다</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>他多次表态。</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>对于公司的这项新政策，部门经理还没有明确表态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>CHI-20260713-010</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>留存</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>liú cún</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>보관하다, 남겨두다, 유지하다</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>劳动合同什么时候签？个人需要留存吗？人社部解答.</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>这些历史文献被妥善地留存在图书馆里。</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>CHI-20260713-011</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>凝心聚力</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>níngxīn jùlì</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>마음을 모으고 힘을 합치다, 단결하여 역량을 집중하다</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>深耕教研传薪火，凝心聚力备高考。</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>为了共同的目标，全体员工凝心聚力，努力奋斗。</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>CHI-20260713-012</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>省吃俭用</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>shěngchī jiǎnyòng</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>절약하며 아껴 쓰다, 검소하게 생활하다</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>张家界男孩省吃俭用高...</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>为了早日买房，小王夫妻俩一直省吃俭用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>CHI-20260713-013</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>陪读</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>péi dú</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>아이의 학업을 위해 함께 살며 돌보다 (주로 부모나 가족이)</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>小姨姨父一家主动提出高中陪读三年。</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>为了孩子的学习，许多家长选择在学校附近陪读。</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>CHI-20260713-014</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>立行立改</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>lìxíng lìgǎi</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>즉시 행동하고 즉시 개선하다, 바로 실행하고 바로 고치다</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>闻令速办解民忧 立行立改护校园。</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>对于顾客的反馈，我们公司承诺立行立改，绝不推诿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>CHI-20260713-015</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>高效处置</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>gāoxiào chǔzhì</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>효율적으로 처리하다, 신속하고 효과적으로 조치하다</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>宜城市高效处置南...</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>面对突发事件，指挥中心迅速高效处置，避免了更大损失。</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>CHI-20260713-016</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>陡增</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>dǒu zēng</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>갑자기 증가하다, 급증하다</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>后者可能让开学陡增焦虑。</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>受疫情影响，近期线上购物订单量陡增。</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>CHI-20260713-017</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>结构突破</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>jiégòu tūpò</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>구조적 돌파, 구조적 혁신</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>康森饰家FOSB欧松板：结构突破环保先行，赋能家居...</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>要实现行业领先，必须在核心技术和产品结构上取得突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>CHI-20260713-018</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>全速竞跑</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>quánsù jìngpǎo</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>전속력으로 질주하다, 치열하게 경쟁하다</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>氢能万亿级赛道全速竞跑.</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>在这个瞬息万变的时代，各行各业都在全速竞跑，寻求发展机遇。</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>CHI-20260713-019</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>恶劣言论</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>èliè yánlùn</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>악의적인 발언, 모욕적인 언사</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>外交部亚洲司负责人就日方涉“南海仲裁案裁决”恶劣言论...</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>公众人物应注意自己的言行，避免发表恶劣言论。</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>CHI-20260713-020</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>科学规划</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>kēxué guīhuà</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>과학적인 계획/기획</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>华兴教育高考复读，科学规划，让每一步都算数。</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>无论是学习还是工作，都需要有科学规划才能提高效率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>CHI-20260713-021</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>传薪火</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>chuán xīn huǒ</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>유산/전통을 이어받다, 정신을 계승하다</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>深耕教研传薪火，凝心聚力备高考——永州四中召开20...</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>我们青年一代有责任传承和弘扬中华优秀传统文化，传薪火。</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>CHI-20260713-022</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>作息</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>zuò xī</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>일과 휴식 (시간), 생활 리듬</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>另一种是彻底放飞，作息全凭“随缘”。</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>规律的作息对身体健康和学习效率都有很大帮助。</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>CHI-20260713-023</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>招募</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>zhāo mù</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>모집하다, 채용하다</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>海淀这20所中小幼学校招聘啦.</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>这家科技公司正在全球范围内招募顶尖的软件工程师。</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>CHI-20260713-024</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>解决民忧</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>jiějué mínyōu</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>국민들의 걱정/고민을 해결하다</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>闻令速办解民忧 立行立改护校园——宜城市高效处置南...</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>政府部门应该倾听民声，采取有效措施解决民忧。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-14 | 575/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I563"/>
+  <dimension ref="A1:I576"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26877,6 +26877,617 @@
         </is>
       </c>
     </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>CHI-20260714-001</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>喘口气</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>chuǎn kǒu qì</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>숨을 돌리다, 잠시 짬을 내어 쉬다</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>经历了一个多月高度紧张的高考，考完之后她终于可以慢下节奏，好好地喘口气了。</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>这几个月一直在连续加班，等这个项目做完了，我得好好喘口气。</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>CHI-20260714-002</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>翻身</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>fān shēn</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>어려운 처지에서 벗어나다, 전세를 뒤집어 재기하다</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>新力环保在六年时间里，从破产边缘一路走到营收过亿，实现了华丽的翻身。</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>他凭着一股不服输的劲头，终于在这个行业里打了个漂亮的翻身仗。</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>CHI-20260714-003</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>占便宜</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>zhàn pián yi</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>이득을 보다, 요행이나 꼼수로 공짜나 이익을 챙기다</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>那些所谓的低分保录陷阱，往往就是看准了家长和学生想要走捷径、占便宜的心理。</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>买东西不能总想着占便宜，一分钱一分货的道理大家都懂。</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>CHI-20260714-004</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>试水</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>shì shuǐ</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>새로운 환경이나 비즈니스에 시험적으로 뛰어들어 반응을 보다</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>新力环保在最初尝试转型的时候，也是抱着试水的心态开始做新型建材的。</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>我们公司决定先在华南市场试水，如果销售情况理想再向全国推广。</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>CHI-20260714-005</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>倒贴</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>dào tiē</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>이익을 보기는커녕 제 돈을 얹어 주다, 손해를 보며 보태다</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>公司刚成立那会儿效益差，老板不仅自己拿不到工资，甚至还要自己倒贴钱给员工发薪。</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>这份兼职工作太辛苦了，工资又低，扣除来回的车费自己还要倒贴。</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>CHI-20260714-006</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>走捷径</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>zǒu jié jìng</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>지름길을 가다, 편법을 쓰다</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>逆袭成功的学霸分享，学习没有捷径可走，脚踏实地积累才是最有效的记忆方法。</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>做学术研究需要耐得住寂寞，绝对不能想着走捷径，否则迟早要栽跟头。</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>CHI-20260714-007</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>玩儿命</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>wán r mìng</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>목숨을 걸다, 죽기 살기로 극단적인 노력을 쏟다</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>为了能在高考中实现逆袭，她高三那年简直是在玩儿命地刷题和记忆单词。</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>为了能在月底前按时交付项目方案，我们整个团队最近都在玩儿命加班。</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>CHI-20260714-008</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>重整旗鼓</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>chóng zhěng qí gǔ</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>실패한 후에 전열을 가다듬어 다시 시작하다, 재기하다</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>虽然高考志愿不幸滑档，但她没有气馁，决定重整旗鼓，重新出发，寻找新的学校。</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>创业失败后，他并没有放弃，而是吸取教训，准备重整旗鼓再次创业。</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>CHI-20260714-009</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>投机取巧</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>tóu jī qǔ qiǎo</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>기회를 틈타 요행을 바라다, 꼼수를 부리다, 부정한 방법으로 이득을 취하다</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>在学术研究中绝不能投机取巧，任何学术不端行为迟早都会被发现并受到严厉惩罚。</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>学习和工作是没有捷径的，只有脚踏实地，不能抱有投机取巧的心态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>CHI-20260714-010</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>防不胜防</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>fáng bù shèng fáng</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>끝도 없이 계속되어 미처 다 막아내기 어렵다, 대처하기가 매우 까다롭다</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>市场上充斥着各种‘低分保录海外名校’的虚假广告，家长们一不小心就会掉入陷阱，真是防不胜防。</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>现在的网络诈骗手段花样百出，真是让人防不胜防，大家一定要提高警惕。</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>CHI-20260714-011</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>避坑</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>bì kēng</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>시행착오나 사기, 잘못된 선택(지뢰)을 피하다</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>帮孩子选择复读学校时，家长一定要多方面考察，掌握这几点关键原则才能成功避坑。</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>买二手房有很多容易让人忽略的细节，这份攻略能帮你完美避坑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>CHI-20260714-012</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>硬着头皮</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>yìng zhe tóu pí</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>억지로, 울며 겨자 먹기로, 용기를 내어 마지못해 (어려운 일을) 하다</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>面对高考失利的残酷现实，很多决定复读的学生也只能硬着头皮再次面对堆积如山的试卷。</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>虽然心里对这次当众发言感到非常紧张，我还是硬着头皮走上了讲台。</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>CHI-20260714-013</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>背黑锅</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>bēi hēi guō</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>억울하게 남의 죄나 잘못을 뒤집어쓰다, 덤터기 쓰다</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>在职场上面对问题要敢于承担，但绝不能平白无故替别人的失误背黑锅。</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>那个宣传方案明明是小王弄错的，结果开会时却让整个小组替他背黑锅。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-15 | 601/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I576"/>
+  <dimension ref="A1:I602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27488,6 +27488,1228 @@
         </is>
       </c>
     </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>CHI-20260715-001</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>讲大道理</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>jiǎng dà dào lǐ</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>훈계하다, 잔소리하다, (거창한) 원론적인 이야기만 하다</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>고등학교 졸업 후 아버지를 따라 트럭을 몰았다는 기사를 봤어. 부모님이 아이들에게 '대단한 훈계'를 하지 않았다고 하더라.</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>我父母从来不爱给我讲大道理，他们更注重言传身教。</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>CHI-20260715-002</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>过暑假</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>guò shǔ jià</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>여름방학을 보내다</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>올해 여름방학은 '삼단식'으로 보내보세요. 아이는 피곤하지 않고, 개학 때도 당황하지 않을 거예요.</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>我们计划去海边过暑假，好好放松一下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>CHI-20260715-003</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>加分</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>jiā fēn</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>(점수 등을) 더하다, 가산점을 주다, (경쟁에서) 유리하게 작용하다</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>AI 시대에 문과생이 어떻게 효과적으로 자신에게 가산점을 줄 수 있을까? 그는 많은 자격증으로 자신의 경험을 증명했어.</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>在面试中表现出良好的沟通能力会为你的形象加分不少。</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>CHI-20260715-004</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>发脾气</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>fā pí qì</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>화를 내다, 짜증을 부리다</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>어제는 일 때문에 스트레스를 너무 많이 받아서 집에서 가족에게 화를 냈어. 정말 미안해.</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>他平时脾气很好，很少对人生气发脾气。</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>CHI-20260715-005</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>打酱油</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>dǎ jiàng yóu</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>방관하다, 무관심하다, 구경만 하다 (원래는 간장을 사러 가다)</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>그들의 논쟁이 격렬했지만, 나는 그저 옆에서 구경만 할 뿐이었어. 어떤 의견도 내지 않았지.</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>这事儿跟我没关系，我就是路过打酱油的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>CHI-20260715-006</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>带节奏</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>dài jié zòu</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>(여론 등을) 조종하다, 분위기를 주도하다, 선동하다</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>이 댓글들은 마치 누군가 고의적으로 부정적인 여론을 조종하려고 하는 것 같아.</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>网络上总有一些人在恶意带节奏，影响舆论走向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>CHI-20260715-007</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>面对面</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>miàn duì miàn</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>얼굴을 마주보고, 직접 대면하여</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>문제를 직접 대면하여 해결하세요! 창닝구 도시관리법 집행 시스템은 '대중 공개의 날' 행사를 통해 시민들에게 서비스를 제공하고 있습니다.</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>有些问题通过电话很难解释清楚，我们还是面对面谈吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>CHI-20260715-008</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>身心疲惫</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>shēn xīn pí bèi</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>몸과 마음이 지치다, 심신이 피로하다</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>개학이 되면 불안감이 급격히 커질 수 있어. 여름방학을 '삼단식'으로 보내면 아이가 몸과 마음이 지치는 것을 막을 수 있다고 해.</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>连续加班一个月，我感到身心疲惫，急需休息。</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>CHI-20260715-009</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>深表关切</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>구어/오피스</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>shēn biǎo guān qiè</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>깊은 우려를 표하다</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>外交部就当前海湾地区的紧张局势深表关切，呼吁各方保持克制。</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>国际社会对该地区不断升级的冲突深表关切。</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>CHI-20260715-010</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>现身说法</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>xiàn shēn shuō fǎ</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>실제 경험을 들어 설명하다, 직접 체험한 사람이 이야기하다</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>高考状元王桐现身说法，分享了他在文科求职中如何通过技能证书为自己加分的经历。</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>老师请一位考上名校的学长现身说法，给同学们传授学习经验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>CHI-20260715-011</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>彻底放飞</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>chè dǐ fàng fēi</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>완전히 자유를 만끽하다, (제약 없이) 마음껏 즐기다</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>有些家长选择让孩子在暑假彻底放飞，不安排任何学习任务。</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>考试结束后，学生们都想彻底放飞自我，好好放松一下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>CHI-20260715-012</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>真抓实干</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>zhēn zhuā shí gàn</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>성실하게 일하다, 실제적으로 행동하고 노력하다</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>长宁区城管执法系统以“真抓实干勇担当”为主题，强调要为民服务。</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>公司的发展离不开领导层的真抓实干和员工的共同努力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>CHI-20260715-013</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>勇于担当</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>구어/오피스</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>yǒng yú dān dāng</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>용기 있게 책임을 지다, 책임을 다하다</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>作为城市管理者，我们必须勇于担当，解决市民的实际难题。</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>新时代的年轻人要勇于担当社会责任，为国家建设贡献力量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>CHI-20260715-014</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>竞争激烈</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>구어/오피스</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>jìng zhēng jī liè</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>경쟁이 치열하다</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>国企招聘的岗位有限，每年都面临着非常激烈的竞争。</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>随着市场饱和，餐饮行业的竞争越来越激烈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>CHI-20260715-015</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>择优录取</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>오피스</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>zé yōu lù qǔ</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>우수한 사람을 선발하여 합격시키다</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>高考录取严格按照“公开、平等、竞争、择优”的原则进行。</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>这所大学的招生标准很高，每年都择优录取最优秀的学生。</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>CHI-20260715-016</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>产出成果</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>chǎn chū chéng guǒ</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>성과를 내다, 결과를 도출하다</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>北京怀柔科学城致力于科技创新，累计产出多项重大科技成果。</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>经过团队几个月的努力，我们终于产出了令人满意的研究成果。</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>CHI-20260715-017</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>取得突破</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>qǔ dé tū pò</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>돌파구를 마련하다, 큰 발전을 이루다</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>在环保技术领域，浙江的专家们不断努力，希望能取得新的突破。</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>科学家们在疫苗研发方面取得了突破性进展。</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>CHI-20260715-018</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>扭亏为盈</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>구어/오피스</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>niǔ kuī wéi yíng</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>적자에서 흑자로 전환하다</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>新力环保公司在短短六年内，从破产边缘扭亏为盈，营收过亿。</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>经过管理层改革，这家濒临倒闭的公司终于扭亏为盈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>CHI-20260715-019</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>付出代价</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>fù chū dài jià</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>대가를 치르다, 희생을 감수하다</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>人为搞“脱钩断链”，最终只会让各方付出更多代价。</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>为了实现梦想，他甘愿付出巨大的代价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>CHI-20260715-020</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>缓解焦虑</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>huǎn jiě jiāo lǜ</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>불안을 완화하다</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>暑假分成三阶段过，可以有效缓解孩子和家长的开学焦虑。</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>适当的运动可以帮助人们缓解工作压力和焦虑情绪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>CHI-20260715-021</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>调整心态</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>tiáo zhěng xīn tài</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>마음가짐을 조절하다, 태도를 바꾸다</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>面对高考后的选择，学生们需要及时调整心态，迎接新生活。</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>面对困难，我们首先要调整心态，积极应对。</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>CHI-20260715-022</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>积累经验</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>jī lěi jīng yàn</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>경험을 쌓다</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>王桐通过丰富的实习经历，为自己积累了宝贵的工作经验。</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>刚入职的新人应该多向同事请教，努力积累经验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>CHI-20260715-023</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>持之以恒</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>chí zhī yǐ héng</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>꾸준히 하다, 일관성 있게 지속하다</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>环保事业需要我们持之以恒地努力，才能看到成效。</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>学习任何一门语言，都需要持之以恒的毅力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>CHI-20260715-024</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>达成共识</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>dá chéng gòng shí</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>합의에 도달하다, 공감대를 형성하다</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>经过长时间的讨论，与会各方终于在关键问题上达成了共识。</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>团队成员必须先达成共识，才能有效地推进项目。</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>CHI-20260715-025</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>克服困难</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>kè fú kùn nan</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>어려움을 극복하다</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>新力环保公司在发展初期克服了重重困难，才有了今天的成就。</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>在人生的道路上，我们需要不断学习如何克服困难。</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>CHI-20260715-026</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>引起关注</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>yǐn qǐ guān zhù</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>주목을 끌다, 관심을 불러일으키다</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>APEC数字周的开幕引起了国内外媒体的广泛关注。</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>他的独特见解在会议上引起了与会者的强烈关注。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-16 | 626/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I602"/>
+  <dimension ref="A1:I627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28710,6 +28710,1181 @@
         </is>
       </c>
     </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>CHI-20260716-001</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>睦邻友好</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>mù lín yǒu hǎo</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>이웃나라와 친하게 지내다; 선린우호</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>中俄两国之间一直保持着睦邻友好关系。</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>我们希望与所有邻国保持睦邻友好的关系。</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>CHI-20260716-002</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>发展繁荣</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>fā zhǎn fán róng</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>발전하고 번영하다</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>技术进步最终是为了促进人类社会的发展繁荣。</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>我们期待城市经济能够持续发展繁荣。</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>CHI-20260716-003</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>促进</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>cù jìn</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>촉진하다, 증진시키다</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>我们应该共同努力，促进经济的可持续发展。</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>教育改革有助于促进社会公平和进步。</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>CHI-20260716-004</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>高质量</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>gāo zhì liàng</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>고품질의, 수준 높은</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>现在人们对生活质量的要求越来越高，都追求高质量的生活。</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>这家公司致力于提供高质量的产品和服务。</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>CHI-20260716-005</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>小车不倒只管推</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>xiǎo chē bù dǎo zhǐ guǎn tuī</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>오뚝이가 넘어지지 않는 한 계속 밀고 나간다; 포기하지 않고 꾸준히 나아가다</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>面对困难，袁熙坤大师总是抱着“小车不倒只管推”的精神坚持下去。</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>即使前方有挑战，我们也要“小车不倒只管推”，坚持到底。</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>CHI-20260716-006</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>干货</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>gān huò</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>핵심 내용, 알짜배기 정보, 실용적인 정보</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>这场讲座有很多干货，对我很有启发。</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>请你直接说干货，不要绕弯子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>CHI-20260716-007</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>履行</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>lǚ xíng</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>(의무, 약속 등을) 이행하다, 수행하다</t>
+        </is>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>作为一名员工，我们必须认真履行自己的职责。</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>公司将严格履行合同条款，确保项目顺利完成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>CHI-20260716-008</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>留住</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>liú zhù</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>붙잡아 두다, 보유하다, 놓치지 않다</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>企业要想长远发展，必须想办法留住核心人才。</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>我们要努力提升服务质量，留住更多的老客户。</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>CHI-20260716-009</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>求职</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>qiú zhí</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>구직하다, 일자리를 찾다</t>
+        </is>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>最近毕业生求职竞争非常激烈，找工作不容易。</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>他正在积极准备简历，希望能找到一份满意的工作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>CHI-20260716-010</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>圆梦</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>yuán mèng</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>꿈을 이루다, 소원을 성취하다</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>通过自己的努力，他终于圆了出国留学的梦。</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>帮助更多贫困儿童圆梦读书是我们的目标。</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>CHI-20260716-011</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>沦为</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>lún wéi</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>~로 전락하다, ~이 되다 (주로 좋지 않은 결과)</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>如果不提高警惕，公司很可能会沦为竞争对手的附庸。</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>他因为赌博，最终沦为了一无所有的流浪汉。</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>CHI-20260716-012</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>借助</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>jiè zhù</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>~의 힘을 빌리다, ~을 이용하다</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>现代社会，我们可以借助互联网获取各种信息。</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>借助大数据分析，我们能更精准地把握市场趋势。</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>CHI-20260716-013</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>倾斜</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>qīng xié</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>기울다, 기울어지다, (~쪽으로) 치우치다, (~을 우대하다)</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>公司的政策倾向于向基层员工倾斜，提高他们的待遇。</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>这次招聘政策向应届毕业生倾斜，提供了更多机会。</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>CHI-20260716-014</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>扎根</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>zhā gēn</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>뿌리내리다, 확고히 자리 잡다</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>这个理念已经在年轻一代心中深深扎根了。</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>他选择在这座小城市扎根，贡献自己的力量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>CHI-20260716-015</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>干涉</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>gān shè</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>간섭하다, 개입하다</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>我们不应该随意干涉别人的私人生活。</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>任何国家都无权干涉他国内政。</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>CHI-20260716-016</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>复读</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>fù dú</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>(재수를 위해) 재수하다, (유급하여) 같은 학년을 다시 다니다</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>他去年高考没考好，决定复读一年再考。</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>很多学生为了考上理想的大学而选择复读。</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>CHI-20260716-017</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>破产</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>pò chǎn</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>파산하다</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>由于经营不善，那家老牌企业最终宣告破产。</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>这家公司因为资金链断裂，很快就破产了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>CHI-20260716-018</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>实习</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>shí xí</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>실습하다, 인턴으로 일하다</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>很多大学生都会在暑假找机会去公司实习。</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>她正在一家跨国公司实习，学习了很多东西。</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>CHI-20260716-019</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>招标</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>zhāo biāo</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>입찰 공고를 내다, 입찰하다</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>这个工程项目正在进行公开招标。</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>我们正在为新项目进行国际招标。</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>CHI-20260716-020</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>取得进展</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>qǔ dé jìn zhǎn</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>진전을 이루다, 진척을 보이다</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>在项目初期阶段，我们已经在技术研发上取得了显著进展。</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>经过团队的不懈努力，销售额终于取得了突破性进展。</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>CHI-20260716-021</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>带火</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>dài huǒ</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>인기를 끌게 하다, 붐을 일으키다</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>这部电影的成功带火了一系列相关旅游景点。</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>短视频平台的挑战活动意外地带火了这家小店的特色美食。</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>CHI-20260716-022</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>筑牢</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>zhù láo</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>단단히 구축하다, 튼튼하게 다지다</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>我们必须筑牢城市安全防线，确保人民生命财产安全。</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>只有筑牢知识基础，才能在未来的学习中走得更远。</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>CHI-20260716-023</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>面向社会</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>miàn xiàng shè huì</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>사회를 대상으로 하다, 대외적으로 공개하다</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>本次招聘是面向社会公开选拔优秀人才。</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>新的政策出台后，将面向社会广泛征求意见。</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>CHI-20260716-024</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>逐梦</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>zhú mèng</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>꿈을 좇다, 꿈을 추구하다</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>青年们应该勇敢地逐梦，为理想而奋斗。</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>在这座城市，许多创业者都在为自己的理想逐梦。</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>CHI-20260716-025</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>升学</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>shēng xué</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>(상급 학교로) 진학하다</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>今年的升学竞争异常激烈，考生们都非常努力。</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>为了孩子的升学问题，家长们绞尽脑汁，费尽心思。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-17 | 648/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I627"/>
+  <dimension ref="A1:I649"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29885,6 +29885,1040 @@
         </is>
       </c>
     </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>CHI-20260717-001</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>落地</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>구어/동사</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>luòdì</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>계획, 프로젝트 등이 확정되거나 실제로 실행에 옮겨지는 것을 의미합니다. (literal: 땅에 내려앉다)</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>제시된 텍스트에서 '국단 밀가루 프로젝트 착수 및 계약 체결식' (国丹面粉项目落地签约仪式)이라는 표현이 보입니다. 여기서 '落地'는 프로젝트가 구체화되고 실행 단계에 들어서는 것을 의미합니다.</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>我们的新产品发布计划终于落地了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>CHI-20260717-002</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>二战</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>구어/동사</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>èrzhàn</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>(시험, 도전 등에서) 재수하다, 두 번째로 도전하다. (literal: 2차 대전이 아닌, '두 번째 싸움'이라는 의미로 쓰임)</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>텍스트에서 '항저우의 한 여학생이 '재수'를 선택했다' (杭州这位女生“二战”...)는 표현이 나옵니다. 이는 특히 '高考'(대입 시험) 등에서 재수를 의미할 때 자주 사용됩니다.</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>他决定再二战一年，考更好的大学。</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>CHI-20260717-003</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>涨知识</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>구어/이합사</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>zhǎng zhīshi</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>지식이 늘다, 새로운 것을 알게 되다, 상식 늘리기.</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>환경 보호 DIY 활동, 인공지능 컨퍼런스, 다양한 산업 보고서 발표 등 새로운 지식을 습득하고 시야를 넓히는 활동과 관련하여 사용될 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>看这部纪录片真的涨知识了，学到了很多新东西。</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>CHI-20260717-004</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>左右为难</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>zuǒyòu wéinán</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>이러지도 저러지도 못하다, 진퇴양난에 빠지다, 난처한 입장이다.</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>명문대 포기 후 재수를 선택하거나 ('985 명문대 포기'), 여러 부처가 협력해야 하는 복잡한 정책 결정('공공자원 거래 센터') 등 어려운 선택의 기로에 놓인 상황에 사용될 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>老板和客户意见不一致，我夹在中间左右为难。</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>CHI-20260717-005</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>身不由己</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>shēn bù yóu jǐ</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>마음대로 할 수 없다, 본의 아니게, 어쩔 수 없이.</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>입시 결과에 따라 원치 않는 선택을 하거나 ('합격 미달로 다시 출발'), 부모님의 상황('아버지를 따라 화물차를 몰았다')에 따라 개인의 의지와 상관없이 행동하게 되는 상황을 묘사할 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>很多时候，我们做一些决定都是身不由己的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>CHI-20260717-006</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>大饱眼福</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>dà bǎo yǎnfú</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>눈요기를 실컷 하다, 멋진 구경을 하다, 실컷 즐기다.</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>반핑산 문화 교류 및 민남어 음악 축제('闽南语音乐季活动')와 같은 문화 행사에서 다채로운 볼거리를 만끽할 때 사용될 수 있습니다.</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>这次旅行看到了很多美丽的风景，真是大饱眼福。</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>CHI-20260717-007</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>竣工投产</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>jùn gōng tóu chǎn</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>준공 및 생산 가동</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>亿膳馍道生产基地竣工投产暨国丹面粉项目落地签约仪式。</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>我们的新工厂预计明年上半年竣工投产。</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>CHI-20260717-008</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>大变身</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>dà biàn shēn</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>크게 변신하다, 대변신</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>闲置衣物大变身，公益环保双向暖心。</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>通过改造，这个老旧的社区终于实现了大变身，变得焕然一新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>CHI-20260717-009</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>双向暖心</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>shuāng xiàng nuǎn xīn</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>쌍방 모두에게 따뜻한 마음을 전하다/위로가 되다</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>闲置衣物大变身，公益环保双向暖心。</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>这次志愿者活动不仅帮助了他人，也让参与者感受到了双向暖心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>CHI-20260717-010</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>致力于</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>zhì lì yú</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>~에 전념하다, 헌신하다</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>致力于将闲置衣物转化为再生资源，助力环保与循环经济。</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>该公司一直致力于研发环保新材料。</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>CHI-20260717-011</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>跑货车</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>pǎo huò chē</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>화물차를 운전하다, 화물 운송업을 하다</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>暑假跟着父亲跑货车。</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>他辞掉白领工作，回乡跟着家人跑货车搞物流了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>CHI-20260717-012</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>履行职责</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>lǚ xíng zhí zé</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>직책을 수행하다, 직무를 이행하다</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>为规范和保障公共资源交易中心履行职责。</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>作为一名公务员，他始终认真履行职责。</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>CHI-20260717-013</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>维护秩序</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>wéi hù zhì xù</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>질서를 유지하다</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>维护招标投标交易秩序。</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>安保人员正在努力维护现场秩序，避免发生拥挤踩踏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>CHI-20260717-014</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>招人</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>zhāo rén</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>사람을 채용하다, 사람을 뽑다</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>金山这个国企招人！</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>我们公司最近业务扩张，正在大量招人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>CHI-20260717-015</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>引进</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>yǐn jìn</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>도입하다, 들여오다, (인재를) 영입하다</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>面向社会引进专业技术人才2名。</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>为了提高生产效率，工厂引进了一批先进设备。</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>CHI-20260717-016</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>营收</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>yíng shōu</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>매출, 영업 수입</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>从破产边缘到营收过亿。</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>尽管市场竞争激烈，但我们公司今年的营收仍保持了稳健增长。</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>CHI-20260717-017</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>书写答卷</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>shū xiě dá juàn</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>답안지를 작성하다 (비유적으로 성과를 내다, 업적을 남기다)</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>书写人大履职答卷。</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>经过多年的努力，中国在航天领域书写了令人瞩目的答卷。</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>CHI-20260717-018</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>履职</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>lǚ zhí</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>직무를 수행하다</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>书写人大履职答卷。</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>他作为新上任的市长，承诺将勤勉履职，服务市民。</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>CHI-20260717-019</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>志愿滑档</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>zhì yuàn huá dàng</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>지원 미달로 대학 합격 등수가 밀리다 (원하는 대학 학과에 떨어져 하위 선택지로 밀리는 상황)</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>志愿滑档后她重新出发。</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>他高考分数很高，没想到因为志愿填报失误导致滑档了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>CHI-20260717-020</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>重新出发</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>chóng xīn chū fā</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>다시 시작하다, 새롭게 출발하다</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>志愿滑档后她重新出发。</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>虽然这次失败了，但他决定重新出发，争取下次成功。</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>CHI-20260717-021</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>共和国长子</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>gòng hé guó cháng zǐ</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>공화국의 장남 (주로 건국 초기에 설립된 대형 국유기업을 지칭)</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>“共和国长子们”的风雨兼程。</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>那些被称为“共和国长子”的企业，为国家经济建设做出了巨大贡献。</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>CHI-20260717-022</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>圆梦启航</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>yuán mèng qǐ háng</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>꿈을 이루고 새로운 출발을 시작하다</t>
+        </is>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>又是一年圆梦启航的美好时节。</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>高考录取通知书的到来，标志着莘莘学子即将圆梦启航，迈向人生的新阶段。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-20 | 668/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I649"/>
+  <dimension ref="A1:I669"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30919,6 +30919,946 @@
         </is>
       </c>
     </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>CHI-20260720-001</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>招生</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>zhāo shēng</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>(학생을) 모집하다, 입학을 허가하다</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>今年我们学校扩大了招生规模，新开设了几个专业。</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>听说那家培训机构最近正在大量招生。</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>CHI-20260720-002</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>就业</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>jiù yè</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>취업하다</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>大批高校学子走出校园，开启人生全新旅程，毕业生就业问题是社会关注的焦点。</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>现在的大学生就业压力越来越大。</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>CHI-20260720-003</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>补齐短板</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>bǔ qí duǎn bǎn</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>(약점/부족한 점을) 보완하다, 메우다</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>为了提升边境地区教师队伍整体素质，教育部指导启动了一系列措施，着力补齐短板。</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>我们应该正视问题，努力补齐短板才能进步。</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>CHI-20260720-004</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>落实</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>luò shí</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>(정책, 계획 등을) 실행에 옮기다, 실현하다, 이행하다</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>国家发改委发布新政策后，各部门需要尽快落实相关规定。</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>这项政策必须尽快落实到位，才能看到效果。</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>CHI-20260720-005</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>报销</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>bào xiāo</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>(경비 등을) 청구하여 변제받다, 정산하다</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>一旦医保断缴超时，看病买药就得全额自费，无法报销。</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>出差的费用可以找财务部报销吗？</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>CHI-20260720-006</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>折腾</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>zhē teng</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>(사람을) 괴롭히다, 고생시키다; (일을) 번거롭게 하다; (몸을) 뒤척이다</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>他为了这个方案已经折腾了一整夜，都没怎么睡觉。</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>别再折腾了，赶紧休息吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>CHI-20260720-007</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>纠结</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>jiū jié</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>(마음이) 복잡하다, 갈등하다, 뒤얽히다</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>最近她一直在纠结要不要换工作，想来想去也拿不定主意。</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>我纠结了很久，最终还是决定买这件衣服。</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>CHI-20260720-008</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>心里没底</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>xīn lǐ méi dǐ</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>자신이 없다, 확신이 없다, 불안하다</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>虽然准备了很久，但明天要上台演讲，我心里还是有点没底。</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>对新的挑战，他心里总是有点没底。</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>CHI-20260720-009</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>一手包办</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>yī shǒu bāo bàn</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>(일을) 혼자서 도맡아 처리하다, 모든 것을 책임지다</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>她是一个特别能干的人，家里大大小小的事情几乎都是她一手包办的。</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>这个项目从头到尾都是他一手包办的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>CHI-20260720-010</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>紧随其后</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>jǐn suí qí hòu</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>뒤를 바싹 쫓다, 바로 이어서 발생하다</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>紧随其后的清华大学692分，北京大学690分。</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>他一说完，我就紧随其后发表了我的看法。</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>CHI-20260720-011</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>向内挖潜</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>오피스</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>xiàng nèi wā qián</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>내부 잠재력을 발굴하다, 내실을 다지다</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>向内挖潜、向外拓新！老牌国企解锁“进阶路”.</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>面对市场变化，我们首先要向内挖潜，提升自身竞争力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>CHI-20260720-012</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>向外拓新</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>오피스</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>xiàng wài tuò xīn</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>외부로 확장하고 혁신하다, 새로운 기회를 모색하다</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>向内挖潜、向外拓新！老牌国企解锁“进阶路”.</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>除了向内挖潜，我们还要向外拓新，寻找新的增长点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>CHI-20260720-013</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>明确红线</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>오피스</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>míng què hóng xiàn</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>(넘지 말아야 할) 한계선/최소 기준을 명확히 하다</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>明确红线补齐短板 加大执法追责力度.</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>公司管理层明确红线，要求所有员工严格遵守规章制度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>CHI-20260720-014</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>加大...力度</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>오피스</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>jiā dà... lì dù</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>...에 대한 노력을 강화하다, ...의 강도를 높이다</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>加大执法追责力度.</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>为了完成目标，我们必须加大投入力度，尽快完成项目。</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>CHI-20260720-015</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>断档</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>오피스</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>duàn dàng</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>단절되다, 공백이 생기다, (물품이) 품절되다</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>医保最怕断档，一旦断缴超时，看病买药就得全额.</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>这种热门商品总是供不应求，经常断档。</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>CHI-20260720-016</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>断缴</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>오피스</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>duàn jiǎo</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>(보험료, 세금 등을) 납부를 중단하다, 끊기다</t>
+        </is>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>一旦断缴超时，看病买药就得全额.</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>医保断缴会影响后续享受待遇，一定要及时补缴。</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>CHI-20260720-017</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>换书</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>huàn shū</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>책을 교환하다</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>废纸换书，别样的“环保人生”.</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>我们学校组织了换书活动，大家可以用旧书换新书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>CHI-20260720-018</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>发力</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>fā lì</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>힘을 내다, 노력하다, 주력하다</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>三方面发力把握海南...</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>团队成员都在为这个项目全力发力，希望能取得好成绩。</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>CHI-20260720-019</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>着力</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>zhuó lì</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>(어떤 일에) 힘을 쏟다, 주력하다</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>着力提升边境地区教师队伍整体素质.</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>政府着力解决民生问题，改善市民生活质量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>CHI-20260720-020</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>全面展开</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>오피스</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>quán miàn zhǎn kāi</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>전면적으로 시작하다/진행하다, 본격적으로 전개하다</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>南宁市区高中阶段学校招生工作全面展开.</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>项目准备工作已完成，下周将全面展开施工。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-21 | 690/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I669"/>
+  <dimension ref="A1:I691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31859,6 +31859,1040 @@
         </is>
       </c>
     </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>CHI-20260721-001</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>踩坑</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>구어/동사</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>cǎi kēng</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>(주로 부정적인 의미로) 실수하다, (경험 부족 등으로) 낭패를 보다, 바보 같은 짓을 하다.</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>2018届河北高考生齐羽曾考出684分，却因轻信高考志愿填报规划师，花3000元咨询费，报考了“双非”院校，成为学校录取最高分。这分明是花钱踩坑。</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>第一次创业，我犯了很多错误，算是踩坑了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>CHI-20260721-002</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>登顶</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>dēng dǐng</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>(산 정상에) 오르다; (최고 순위나 위치에) 오르다, 1위를 차지하다.</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>上海交大投档线695分登顶湖南，这位全省前50名的学子成为关注焦点。</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>经过多年的努力，这家公司终于在行业内登顶。</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>CHI-20260721-003</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>误导</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>wù dǎo</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>잘못 인도하다, 오도하다, 오해하게 하다.</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>悔！八年前684分考生，被“规划师”误导录进“双非”院校，真是令人扼腕叹息。</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>这条新闻报道内容有误导性，可能会引起公众误解。</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>CHI-20260721-004</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>滑档</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>구어/동사</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>huá dàng</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>(대학 입시에서) 지원한 학교의 합격선에 미달하여 떨어지다, 불합격하다.</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>提升6030名，总分637分！志愿滑档后她重新出发，最终考上了理想的大学。</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>因为填报志愿太冒险，他最终还是滑档了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>CHI-20260721-005</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>挖潜</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>이합사/동사</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>wā qián</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>잠재력을 발굴하다, 잠재력을 캐내다. (주로 내부 역량이나 자원 활용)</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>向内挖潜、向外拓新！老牌国企解锁“进阶路”，寻求新的增长点。</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>公司通过优化管理流程，充分挖潜内部资源，提高了效率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>CHI-20260721-006</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>拓新</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>tà xīn</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>새로운 것을 개척하다, 확장하다, 새로운 시장이나 영역을 넓히다.</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>向内挖潜、向外拓新！老牌国企解锁“进阶路”，展现出活力与创新。</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>为了应对市场变化，我们必须不断拓新业务领域。</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>CHI-20260721-007</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>进阶</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>jìn jiē</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>(단계적으로) 발전하다, 진보하다, 한 단계 나아가다.</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>向内挖潜、向外拓新！老牌国企解锁“进阶路”，实现了高质量发展。</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>通过这次培训，我的专业技能得到了显著进阶。</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>CHI-20260721-008</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>解读</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>jiě dú</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>해석하다, 풀이하다, 분석하다. (특히 정책, 상황, 데이터 등)</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>北京市发展和改革委员会举办上半年首都经济形势解读新闻发布会，吸引了众多媒体关注。</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>专家正在对最新的经济数据进行解读。</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>CHI-20260721-009</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>滋事</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>zī shì</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>소란을 피우다, 말썽을 일으키다, 시비를 걸다.</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>外交部：敦促菲方立即停止海上滋事挑衅和侵权行径，不要再误判形势。</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>他酒后喜欢滋事，所以大家都不太愿意和他一起出去。</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>CHI-20260721-010</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>明确</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>míng què</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>명확히 하다, 분명히 하다, 확실히 정하다.</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>明确红线补齐短板，加大执法追责力度，确保市场秩序公平公正。</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>会议上我们明确了下个季度的销售目标和策略。</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>CHI-20260721-011</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>结硕果</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>jié shuò guǒ</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>풍성한 결실을 맺다.</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>“航天铸魂”结硕果！燕山小学获评“山东省航空特色学校”，这是对他们努力的肯定。</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>经过团队成员的共同努力，我们的项目终于结硕果了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>CHI-20260721-012</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>传捷报</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>chuán jié bào</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>승전보를 전하다, 좋은 소식을 알리다. (주로 큰 성공이나 승리 후)</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>迭创新高！31名学子圆梦清华，盛夏传捷报，逐梦启新程。</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>公司新产品发布后市场反响热烈，营销部立即传捷报给高层。</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>CHI-20260721-013</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>创新高</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>이합사/동사</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>chuàng xīn gāo</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>신기록을 세우다, 최고 기록을 경신하다.</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>原标题：迭创新高！31名学子圆梦清华盛夏传捷报，逐梦启新程。</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>这个月的销售额再创新高，大家都很兴奋。</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>CHI-20260721-014</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>赶趟</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>구어/동사</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>gǎn tàng</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>(어떤 일에) 제때 맞추어 가다, 때를 맞추다, 뒤처지지 않다. (주로 부정문에 쓰여 때를 놓치지 않다, 제 시간에 하다)</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>提前完成年度目标，上半年北京中心城区新增超2万个停车位，各项工作都赶趟完成。</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>你快点走吧，再不走就赶不上趟了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>CHI-20260721-015</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>提前完成</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>tí qián wán chéng</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>예정보다 일찍 완료하다</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>提前完成年度目标，上半年北京中心城区新增超2万个停...</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>如果我们能提前完成任务，就能获得额外的奖金。</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>CHI-20260721-016</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>挑衅</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>tiǎo xìn</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>도발하다, 시비를 걸다</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>外交部：敦促菲方立即停止海上滋事挑衅。</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>他总是喜欢在会议上挑衅领导，结果搞得气氛很紧张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>CHI-20260721-017</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>很燃</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>hěn rán</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>열정적이다, 불타오르다, 멋지다 (긍정적인 감탄사)</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>“慢天使”不慢 “金牌宝宝”很燃！</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>看了这部电影，我感觉整个人都燃起来了，特别励志！</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>CHI-20260721-018</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>轻信</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>qīng xìn</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>경솔하게 믿다, 섣불리 믿다</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>八年前684分考生，被“规划师”误导，轻信他人。</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>我们不能轻信网上那些未经证实的消息。</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>CHI-20260721-019</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>应对</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>yìng duì</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>대응하다, 대처하다</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>中国基础教育以“本土经验”应对世界级难题。</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>我们需要制定一个周密的计划来应对市场变化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>CHI-20260721-020</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>择优</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>zé yōu</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>우수한 사람/것을 선발하다, 선별하다</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>按照“公开、平等、竞争、择优”的原则进行招聘。</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>这次招聘我们将择优录取，不拘一格。</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>CHI-20260721-021</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>收割</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>shōu gē</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>(비유적으로) 이익을 얻다, 이득을 취하다; (부정적으로) 이용하다, 갈취하다</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>各类收费咨询机构又大肆收割起考生和家长。</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>这些平台打着免费的旗号，实际上是在收割用户的个人信息。</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>CHI-20260721-022</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>来袭</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>lái xí</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>(불행, 재해, 좋지 않은 상황 등이) 닥쳐오다, 들이닥치다</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>重磅补贴来袭！最高省上万元！</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>一股寒流即将来袭，请大家注意保暖。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-22 | 707/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I691"/>
+  <dimension ref="A1:I708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32893,6 +32893,805 @@
         </is>
       </c>
     </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>CHI-20260722-001</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>得不偿失</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>débùchángshī</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>얻는 것보다 잃는 것이 많다, 득보다 실이 크다</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>단기적인 이익을 위해 장기적인 관계를 망치는 것은 결국 얻는 것보다 잃는 것이 많을 것입니다.</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>为了省一点小钱而浪费大量时间，真是得不偿失。</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>CHI-20260722-002</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>心里有数</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>xīnli yǒushù</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>잘 알고 있다, 속으로 헤아리고 있다, 짐작하고 있다</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>프로젝트 진행 상황에 대해 그는 이미 잘 알고 있을 것입니다.</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>虽然他没说，但我知道他心里有数，一切都在计划中。</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>CHI-20260722-003</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>一窍不通</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>yīqiàobùtōng</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>문외한이다, 전혀 알지 못하다</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>저는 경제학에 대해 전혀 알지 못해서 관련 기사를 읽어도 이해하기 어렵습니다.</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>我对电脑维修一窍不通，完全不知道该怎么办。</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>CHI-20260722-004</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>封顶</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>fēng dǐng</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>(건물 등) 골조 공사를 마치다, 상량하다; (수치 등이) 최고치에 달하다</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>副中心又一家国企总部大楼主体封顶！</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>经过两年的建设，新博物馆的主体工程终于顺利封顶了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>CHI-20260722-005</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>夯实</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>hāng shí</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>(기초를) 다지다, 튼튼히 하다, 공고히 하다</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>双权威绿标加持，大王椰持续夯实家居板材健康底色.</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>我们要持续夯实技术基础，才能在激烈的市场竞争中立于不败之地。</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>CHI-20260722-006</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>直面</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>zhí miàn</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>(문제 등을) 정면으로 마주하다, 직시하다</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>首期直面“家底”与“短...”</t>
+        </is>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>面对经济下行的压力，我们必须直面挑战，积极寻求解决方案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>CHI-20260722-007</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>增资</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>zēng zī</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>(회사, 기업 등이) 자본금을 늘리다, 증자하다</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>大连重工：全资子公司增资完成工商变更登记.</t>
+        </is>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>为了扩大生产规模，公司决定向股东募集资金进行增资。</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>CHI-20260722-008</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>引进人才</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>yǐn jìn rén cái</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>인재를 유치하다/영입하다</t>
+        </is>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>上海新金山投资控股集团有限公司面向社会引进专业技术人才2名.</t>
+        </is>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>为了提升科研实力，我们大学每年都致力于引进高水平人才。</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>CHI-20260722-009</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>滋事挑衅</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>zī shì tiǎo xìn</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>문제를 일으키고 도발하다</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>外交部：敦促菲方立即停止海上滋事挑衅和...</t>
+        </is>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>任何国家都无权在他国领土上滋事挑衅。</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>CHI-20260722-010</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>规划建设</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>guī huà jiàn shè</t>
+        </is>
+      </c>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>계획하고 건설하다</t>
+        </is>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>系统推进“六张网”规划建设，国常会再部署.</t>
+        </is>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>城市发展需要长远的规划建设，才能避免盲目扩张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>CHI-20260722-011</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>扩大投资</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>kuò dà tóu zī</t>
+        </is>
+      </c>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>투자를 확대하다</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>作为今年扩大有效投资的重要发力点，“六张网”规划建设正迎来密集的政策部署.</t>
+        </is>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>政府鼓励企业扩大投资，以促进经济增长和创造就业机会。</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>CHI-20260722-012</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>失控</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>shī kòng</t>
+        </is>
+      </c>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>통제 불능이 되다, 제어력을 상실하다</t>
+        </is>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>失控的监护“外包”：孩子被送特训机构之后.</t>
+        </is>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>如果不及时采取措施，疫情可能会彻底失控。</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>CHI-20260722-013</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>着手</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>zhuó shǒu</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>착수하다, 시작하다</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>(새로운 사업/프로젝트 시작 맥락에서 유추)</t>
+        </is>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>新项目马上要启动了，我们得尽快着手准备。</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>CHI-20260722-014</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>摆脱</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>bǎi tuō</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>벗어나다, 떨쳐버리다</t>
+        </is>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>(어려운 상황이나 제약에서 벗어나는 맥락에서 유추)</t>
+        </is>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>他努力工作，终于摆脱了贫困的生活。</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>CHI-20260722-015</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>达成协议</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>dá chéng xié yì</t>
+        </is>
+      </c>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>협의에 도달하다, 합의를 이루다</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>(기업 간 협력, 국제 관계 등의 맥락에서 유추)</t>
+        </is>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>经过多轮谈判，双方终于就贸易问题达成了协议。</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>CHI-20260722-016</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>拭目以待</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>shì mù yǐ dài</t>
+        </is>
+      </c>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>눈을 닦고 기다리다; (결과를) 기대하며 지켜보다</t>
+        </is>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>(발표된 정책이나 프로젝트의 결과를 기대하는 맥락에서 유추)</t>
+        </is>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>这部电影备受期待，观众们都拭目以待它的上映。</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>CHI-20260722-017</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>顺理成章</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>shùn lǐ chéng zhāng</t>
+        </is>
+      </c>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>이치에 맞아 당연하다, 순리대로 이루어지다</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>(특정 결과나 상황이 자연스러운 흐름에 따라 발생한다는 맥락에서 유추)</t>
+        </is>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>他的努力工作와 우수한 성과를 고려할 때, 승진은 순리성장한 일이다.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-22 | 725/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I708"/>
+  <dimension ref="A1:I726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33692,6 +33692,852 @@
         </is>
       </c>
     </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>CHI-20260722-018</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>心心念念</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>xīn xīn niàn niàn</t>
+        </is>
+      </c>
+      <c r="G709" t="inlineStr">
+        <is>
+          <t>간절히 바라다, 늘 마음속으로 염원하다</t>
+        </is>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>独立整洁的学习空间是很多困境青少年心心念念的心愿。</t>
+        </is>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>她终于拿到了心心念念的名企实习录取通知书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>CHI-20260722-019</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>不问青红皂白</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>bù wèn qīng hóng zào bái</t>
+        </is>
+      </c>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>사정이나 앞뒤 맥락을 따지지도 않고 무작정</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>海上一有风吹草动，有人就不问青红皂白地把责任推给别人。</t>
+        </is>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>你不能不问青红皂白就批评下属，先听听他的解释。</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>CHI-20260722-020</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>风吹草动</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>fēng chuī cǎo dòng</t>
+        </is>
+      </c>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>미세한 변화나 소문, 조그만 기척</t>
+        </is>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>哪怕海面上有一点风吹草动，某些媒体就会过度炒作。</t>
+        </is>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>行业内一有风吹草动，很多投资者就会变得非常敏感。</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>CHI-20260722-021</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>攀比</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>pān bǐ</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>남과 비교하며 과소비하거나 허세를 부리다</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>高考结束后，不少学生盲目攀比买高档电子产品，增加了家长的负担。</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>年轻人消费要理性，不要盲目和别人攀比。</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>CHI-20260722-022</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>掏腰包</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>tāo yāo bāo</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>자기 지갑을 열다, 사비를 들이다</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>为了给高考毕业的孩子的“成人礼”买单，许多父母不得不掏腰包。</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>这次部门聚会的费用全部由主管掏腰包了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>CHI-20260722-023</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>铺路</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>pū lù</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>미래를 위해 기반을 다지다, 길을 터주다</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>政府推进就业保障政策，就是为了给年轻人的未来发展铺路。</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>父母辛辛苦苦工作，就是为了给孩子的未来铺路。</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>CHI-20260722-024</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>摸底</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>mō dǐ</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>사전에 정황, 실태, 실력을 사전에 조사하거나 파악하다</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>相关部门在出台新政策前，对新就业形态劳动者的人数进行了摸底。</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>开会前，我们要对客户的需求做一个详细的摸底。</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>CHI-20260722-025</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>散心</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>sàn xīn</t>
+        </is>
+      </c>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>답답한 마음을 달래다, 머리를 식히다</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>高考结束后，很多考生选择出去旅游散心，缓解长期的压力。</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>工作太累了，周末我想去郊区散散心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>CHI-20260722-026</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>交心</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>jiāo xīn</t>
+        </is>
+      </c>
+      <c r="G717" t="inlineStr">
+        <is>
+          <t>솔직하게 속마음을 나누다</t>
+        </is>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>社区志愿者走访困境家庭，与青少年交心，了解他们的真实想法。</t>
+        </is>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>我和他认识多年了，是非常交心的朋友。</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>CHI-20260722-027</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>砸钱</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>zá qián</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>거침없이 많은 돈을 쏟아붓다</t>
+        </is>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>不少商家瞄准准考生市场，靠砸钱宣传来吸引消费者。</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>这个项目光靠砸钱是没用的，关键是要有好的产品设计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>CHI-20260722-028</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>买单</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>mǎi dān</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>계산하다, (결과나 실수에 대해) 책임지다</t>
+        </is>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>盲目消费的后果，最终还是要由学生和家长自己买单。</t>
+        </is>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>我们做出的每一个决策，都必须自己去买单。</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>CHI-20260722-029</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>打下手</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>dǎ xià shǒu</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>보조 역할을 하다, 옆에서 수발을 들다</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>新进公司的实习生一般先从打下手开始，慢慢熟悉业务。</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>今天做饭你主厨，我在旁边给你打下手。</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>CHI-20260722-030</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>推波助澜</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>tuī bō zhù lán</t>
+        </is>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>부추기다, (일의 상황을) 한층 더 부채질하다</t>
+        </is>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>部分商家为了增加销量，在社交平台上推波助澜，炒作过度消费的风气。</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>网络上的不实言论对这次公关危机起到了推波助澜的反效果。</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>CHI-20260722-031</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>兜底</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>dōu dǐ</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>최후의 보장을 하다, 끝까지 책임지고 처리해주다</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>政府出台了保障政策，为新就业形态劳动者的基本权益兜底。</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>你放手去干吧，万一出了什么问题由我们团队来兜底。</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>CHI-20260722-032</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>提上日程</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>tí shàng rì chéng</t>
+        </is>
+      </c>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>일정에 올리다, 본격적으로 추진을 시작하다</t>
+        </is>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>随着新一轮改革推行，个人养老金制度的细则落地已被提上日程。</t>
+        </is>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>公司决定将新产品的海外推广计划正式提上日程。</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>CHI-20260722-033</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>支招</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>zhī zhāo</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>아이디어를 주다, 해결책을 제시해 주다</t>
+        </is>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>针对困境学子的求职难题，多位行业专家现场为他们支招。</t>
+        </is>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>面对这么棘手的客户投诉，老同事给刚入职的我支了几招。</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>CHI-20260722-034</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>明眼人</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>míng yǎn rén</t>
+        </is>
+      </c>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>통찰력 있는 사람, 상황을 똑똑히 알아채는 사리 밝은 사람</t>
+        </is>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>明眼人都能看得出，这次策略调整是为了顺应未来的政策导向。</t>
+        </is>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>这明显是个商业陷阱，稍有经验的明眼人一扫就能看穿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>CHI-20260722-035</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>见缝插针</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>jiàn fèng chā zhēn</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>짬을 내다, 바쁜 와중에도 틈을 활용하다</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>很多职场年轻人见缝插针地利用日常碎片时间学习第二外语。</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>出差行程安排得非常紧，他只能见缝插针地在高铁上批改文件。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-23 | 739/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I726"/>
+  <dimension ref="A1:I740"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34538,6 +34538,664 @@
         </is>
       </c>
     </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>CHI-20260723-001</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>闹情绪</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>nào qíng xù</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>불만이 있어 감정적으로 굴다, 떼를 쓰다</t>
+        </is>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>职场新人遇到工作压力时，不能随便闹情绪，要学会理性沟通。</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>遇到问题时要冷静沟通，一味地闹情绪解决不了任何问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>CHI-20260723-002</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>踩点</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>cǎi diǎn</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>출근이나 약속 시간에 딱 맞게 겨우 도착하다</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>每天早上打卡上班，他总是踩点进办公室，一分不多一分不少。</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>为了不踩点上班，我今天特意比平时提前了二十分钟出门。</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>CHI-20260723-003</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>做功课</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>zuò gōng kè</t>
+        </is>
+      </c>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>사전에 철저히 대안이나 배경 정보를 조사/준비하다</t>
+        </is>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>去参加国企招聘面试之前，一定要提前做功课，了解企业的背景。</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>去买车之前我做足了功课，所以没被销售人员忽悠。</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>CHI-20260723-004</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>留后路</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>liú hòu lù</t>
+        </is>
+      </c>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>만약을 대비해 퇴로나 대안을 남겨두다</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>放弃名校选择二战高考需要极大的勇气，这等于不给自己留后路。</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>做商业投资时千万不能孤注一掷，一定要给自己留后路。</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>CHI-20260723-005</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>有数</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>yǒu shù</t>
+        </is>
+      </c>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>속으로 계산이 서다, 형편을 이미 잘 파악하고 있다</t>
+        </is>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>面对上半年的固定资产投资目标，负责人表示心里很有数。</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>关于项目的具体进展，你心里有数就行，别太紧张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>CHI-20260723-006</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>顶梁柱</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>dǐng liáng zhù</t>
+        </is>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>집안이나 조직을 떠받치는 핵심 기둥/대들보</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>那位货车司机父亲是全家的顶梁柱，靠勤劳供女儿考上了大学。</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>他是我们部门的技术顶梁柱，遇到难题大家都去请教他。</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>CHI-20260723-007</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>掉队</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>diào duì</t>
+        </is>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>경쟁이나 대열에서 뒤처지다, 낙오하다</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>在竞争激烈的市场环境里，企业如果不拓新就会面临掉队的风险。</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>学习如逆水行舟，稍有松懈就会在班里掉队。</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>CHI-20260723-008</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>立足</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>lì zú</t>
+        </is>
+      </c>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>사회나 시장에서 기반을 잡다, 발붙이다</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>老牌国企要想在当今市场上重新立足，就必须向内挖潜、向外拓新。</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>刚到新城市发展的年轻人，首先要脚踏实地立足下来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>CHI-20260723-009</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>把关</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>bǎ guān</t>
+        </is>
+      </c>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>엄격히 관리·검수하다, 품질을 책임지다</t>
+        </is>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>在高考招生录取现场，‘录检’工作人员严密把关，确保公平公正。</t>
+        </is>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>产品出厂前必须由专人把关，保证质量达标。</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>CHI-20260723-010</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>铆足劲</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>mǎo zú jìng</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>온 힘을 모으다, 각오를 다지다</t>
+        </is>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>为了圆梦理想的大学，她放弃了休闲时间，铆足劲拼搏。</t>
+        </is>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>下半年全队都铆足劲，争取一举突破今年的销售目标。</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>CHI-20260723-011</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>敲警钟</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>qiāo jǐng zhōng</t>
+        </is>
+      </c>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>경종을 울리다, 경각심을 주다</t>
+        </is>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>频发的安全事故给企业管理者敲响了警钟。</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>这次模拟考试成绩下滑，正好给骄傲的他敲响了警钟。</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>CHI-20260723-012</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>咬牙</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>yǎo yá</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>이를 악물다, 결단을 내리다, 고통을 참다</t>
+        </is>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>面对罕见病的折磨，她咬牙坚持完成了高考并考出好成绩。</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>创业初期资金非常紧缺，但他咬牙挺过了最困难的时期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>CHI-20260723-013</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>打硬仗</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>dǎ yìng zhàng</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>힘겨운 과제를 수행하다, 고난도 업무에 맞서다</t>
+        </is>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>这支研发团队敢打硬仗，在短时间内攻克了核心技术难题。</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>下季度的市场推广是一场硬仗，我们必须提前做好充分准备。</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>CHI-20260723-014</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>找路子</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F740" t="inlineStr">
+        <is>
+          <t>zhǎo lù zi</t>
+        </is>
+      </c>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>수단/방법을 강구하다, 돌파구를 찾다</t>
+        </is>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>面对传统市场饱和，企业开始积极找路子拓宽线上渠道。</t>
+        </is>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>遇到经营难题时，不能坐以待毙，得主动出去找路子。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-24 | 750/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I740"/>
+  <dimension ref="A1:I751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35196,6 +35196,523 @@
         </is>
       </c>
     </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>CHI-20260724-001</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>挂科</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F741" t="inlineStr">
+        <is>
+          <t>guà kē</t>
+        </is>
+      </c>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>낙제하다, 과목 낙제를 받다</t>
+        </is>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>수험생들과 대학생들이 치열한 경쟁 속에서 성적 관리에 각별한 노력을 기울이고 있다.</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>这次期末考试很难，不过幸好我没挂科。</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>CHI-20260724-002</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>减压</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>jiǎn yā</t>
+        </is>
+      </c>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>스트레스를 줄이다, 부담을 낮추다</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>수능 준비생들과 취준생들을 위한 다양한 힐링 문화 행사 및 쉼터 프로그램이 운영되고 있다.</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>工作累的时候，去跑跑步能帮你有效减压。</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>CHI-20260724-003</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>出彩</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>chū cǎi</t>
+        </is>
+      </c>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>두각을 나타내다, 눈부신 성과를 내다</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>지역 산업 발전과 환경 보호 활동에서 탁월한 성과를 거둔 인물의 이야기.</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>她在这次团队演讲中表现非常出彩，赢得了全场的掌声。</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>CHI-20260724-004</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>垫底</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>diàn dǐ</t>
+        </is>
+      </c>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>꼴찌를 하다, 하위권을 받쳐주다</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>치열한 경쟁률의 입시와 국기업체 채용 시험 결과를 둘러싼 이야기.</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>为了不给团队业绩垫底，他每天都加班加点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>CHI-20260724-005</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>默默无闻</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>mò mò wú wén</t>
+        </is>
+      </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>묵묵히 소문 없이 헌신하다, 세상에 알려지지 않다</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>국립공원과 생태 환경을 지키며 수십 년간 고생해 온 현장 관리자들.</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>正是许多默默无闻的护林员，守卫着我们的绿水青山。</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>CHI-20260724-006</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>循序渐进</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>xún xù jiàn jìn</t>
+        </is>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>차근차근 점진적으로 나아가다</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>사회보장 시범 사업 확대 및 신 직업 자격 제도의 안정적 정착 과정.</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>推进这项重大改革需要循序渐进，不能操之过急。</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>CHI-20260724-007</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>齐心协力</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>qí xīn xié lì</t>
+        </is>
+      </c>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>마음을 모아 한뜻으로 합심하다</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>지역 사회와 기관들이 힘을 합쳐 쓰레기 분리배출 및 환경 개선 운동을 벌인다.</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>只要大家齐心协力，就没有克服不了的困难。</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>CHI-20260724-008</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>满载而归</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>mǎn zài ér guī</t>
+        </is>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>풍성한 성과/결실을 얻고 돌아오다</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>해외 순방 및 경제 협상, 박람회 수주 활동에서 큰 성과를 거두고 귀국한 대표단.</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>代表团参加完这次国际能源论坛，可以说是满载而归。</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>CHI-20260724-009</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>厚积薄发</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>hòu jī bó fā</t>
+        </is>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>오랫동안 에너지를 충분히 축적한 뒤 성과를 발휘하다</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>凭借多年的技术积累，该公司终于实现了厚积薄发。</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>学习语言没有捷径，只有平时厚积薄发，考试时才能游刃有余。</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>CHI-20260724-010</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>扎堆</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>zhā duī</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>한데 몰리다, 떼 지어 집중되다</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>暑期来临，游客扎堆前往热门生态旅游景区。</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>下班高峰期大家扎堆打车，往往需要等待较长时间。</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>CHI-20260724-011</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>立竿见影</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>lì gān jiàn yǐng</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>즉각적인 효과를 거두다, 효력이 바로 나타나다</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>政府出台的这项就业扶持政策收到了立竿见影的效果。</t>
+        </is>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>调整了广告投放策略后，本月的销售额立刻收到了立竿见影的增长。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-27 | 763/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I751"/>
+  <dimension ref="A1:I764"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35713,6 +35713,617 @@
         </is>
       </c>
     </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>CHI-20260727-001</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>抓瞎</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>zhuā xiā</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>어찌할 바를 몰라 당황하다, 대책이 없이 막막해지다</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>如果事前不做好周密规划，一旦遇到突发状况就会彻底抓瞎。</t>
+        </is>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>电脑突然坏了，又没有备份文件，这下我彻底抓瞎了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>CHI-20260727-002</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>划算</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>huá suàn</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>가성비가 좋다, 이득이다, 계산이 맞다</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>参与环保旧物换图书活动，既能保护环境又能拿到新书，非常划算。</t>
+        </is>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>这款手机现在搞促销打折，买下来特别划算。</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>CHI-20260727-003</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>露马脚</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>lòu mǎ jiǎo</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>꼬리가 잡히다, 숨겨진 허점이나 정체가 드러나다</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>谎言说得再逼真，时间一长也难免会露马脚。</t>
+        </is>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>警方仔细排查细节，凶手很快就露出了马脚。</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>CHI-20260727-004</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>起跑线</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>qǐ pǎo xiàn</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>출발선, 경쟁의 시작점</t>
+        </is>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>许多家长为了不让孩子输在起跑线上，从小就报名各种补习班。</t>
+        </is>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>良好的家庭教育能给孩子提供一个更好的起跑线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>CHI-20260727-005</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>抢手</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>qiǎng shǒu</t>
+        </is>
+      </c>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>불티나게 팔리다, 매우 인기가 높다</t>
+        </is>
+      </c>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>这家市属国企发出的岗位招聘信息一经公布，就成为了求职市场上的抢手货。</t>
+        </is>
+      </c>
+      <c r="I756" t="inlineStr">
+        <is>
+          <t>暑期热门景点的门票非常抢手，需要提前预约。</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>CHI-20260727-006</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>吹牛</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>chuī niú</t>
+        </is>
+      </c>
+      <c r="G757" t="inlineStr">
+        <is>
+          <t>허풍을 떨다, 뻥치다</t>
+        </is>
+      </c>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>他这个人就喜欢说大话吹牛，你可千万别完全相信他。</t>
+        </is>
+      </c>
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>他总是爱在朋友面前吹牛，大家早已见怪不怪了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>CHI-20260727-007</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>避风港</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>bì fēng gǎng</t>
+        </is>
+      </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>안식처, 피난처</t>
+        </is>
+      </c>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>无论在外工作遇到多大的压力，温馨的家永远是疲惫心灵的避风港。</t>
+        </is>
+      </c>
+      <c r="I758" t="inlineStr">
+        <is>
+          <t>对我来说，图书馆就是避开喧嚣的避风港。</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>CHI-20260727-008</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>掉以轻心</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>diào yǐ qīng xīn</t>
+        </is>
+      </c>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>방심하다, 가볍게 여겨 주의를 소홀히 하다</t>
+        </is>
+      </c>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>尽管目前进展顺利，但我们依然不能掉以轻心。</t>
+        </is>
+      </c>
+      <c r="I759" t="inlineStr">
+        <is>
+          <t>面对重要考试，任何小细节都不能掉以轻心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>CHI-20260727-009</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>炒冷饭</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>chǎo lěng fàn</t>
+        </is>
+      </c>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>(새로운 내용 없이) 우려먹다, 재탕하다</t>
+        </is>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>这部电影的剧情毫无创新，完全是在炒冷饭。</t>
+        </is>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>每次开会他都重复老话题，大家都很讨厌他炒冷饭。</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>CHI-20260727-010</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>穿小鞋</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>chuān xiǎo xié</t>
+        </is>
+      </c>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>(남몰래) 괴롭히다, 골탕 먹이다</t>
+        </is>
+      </c>
+      <c r="H761" t="inlineStr">
+        <is>
+          <t>他因为顶撞了主管，担心以后会被穿小鞋。</t>
+        </is>
+      </c>
+      <c r="I761" t="inlineStr">
+        <is>
+          <t>职场中要学会沟通，避免因为误会而被别人穿小鞋。</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>CHI-20260727-011</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>占上风</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>zhàn shàng fēng</t>
+        </is>
+      </c>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>우세를 점하다, 주도권을 잡다</t>
+        </is>
+      </c>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>在昨晚的辩论赛中，反方观点明显占了上风。</t>
+        </is>
+      </c>
+      <c r="I762" t="inlineStr">
+        <is>
+          <t>凭借出色的产品质量，我们在市场竞争中占了上风。</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>CHI-20260727-012</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>见外</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F763" t="inlineStr">
+        <is>
+          <t>jiàn wài</t>
+        </is>
+      </c>
+      <c r="G763" t="inlineStr">
+        <is>
+          <t>서먹하게 굴다, 남으로 여기다</t>
+        </is>
+      </c>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>咱们都是多年的老朋友了，互相帮忙别太见外。</t>
+        </is>
+      </c>
+      <c r="I763" t="inlineStr">
+        <is>
+          <t>来我家吃饭就像在自己家一样，千万别见外。</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>CHI-20260727-013</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>顾此失彼</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F764" t="inlineStr">
+        <is>
+          <t>gù cǐ shī bǐ</t>
+        </is>
+      </c>
+      <c r="G764" t="inlineStr">
+        <is>
+          <t>이것저것 다 챙기지 못하다, 하나에 신경 쓰다 다른 것을 놓치다</t>
+        </is>
+      </c>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>同时处理太多任务，很容易出现顾此失彼的情况。</t>
+        </is>
+      </c>
+      <c r="I764" t="inlineStr">
+        <is>
+          <t>在追求速度的同时忽略了质量，往往会顾此失彼。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-28 | 774/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I764"/>
+  <dimension ref="A1:I775"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36324,6 +36324,523 @@
         </is>
       </c>
     </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>CHI-20260728-001</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>尘埃落定</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F765" t="inlineStr">
+        <is>
+          <t>chén āi luò dìng</t>
+        </is>
+      </c>
+      <c r="G765" t="inlineStr">
+        <is>
+          <t>마침내 결과가 매듭지어지다, 윤곽이 드러나다</t>
+        </is>
+      </c>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>高考和中考都已经结束了，等到一切尘埃落定，大家终于可以松一口气了。</t>
+        </is>
+      </c>
+      <c r="I765" t="inlineStr">
+        <is>
+          <t>等这次项目招标尘埃落定之后，我们再决定下一步的预算规划。</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>CHI-20260728-002</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>迫不及待</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F766" t="inlineStr">
+        <is>
+          <t>pò bù jí dài</t>
+        </is>
+      </c>
+      <c r="G766" t="inlineStr">
+        <is>
+          <t>더 이상 참지 못하다, 조바심 내며 서두르다</t>
+        </is>
+      </c>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>收到录取通知书后，许多新生都已经迫不及待地想要开启大学生活了。</t>
+        </is>
+      </c>
+      <c r="I766" t="inlineStr">
+        <is>
+          <t>一听到假期开始的消息，大家就迫不及待地收拾行李准备出发。</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>CHI-20260728-003</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>挂钩</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F767" t="inlineStr">
+        <is>
+          <t>guà gōu</t>
+        </is>
+      </c>
+      <c r="G767" t="inlineStr">
+        <is>
+          <t>연계하다, 연관 짓다</t>
+        </is>
+      </c>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>现在的业绩考核直接与终奖挂钩，大家的干劲一下子被提起来了。</t>
+        </is>
+      </c>
+      <c r="I767" t="inlineStr">
+        <is>
+          <t>员工的绩效奖金直接跟每月的销售业绩挂钩。</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>CHI-20260728-004</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>挂牌</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F768" t="inlineStr">
+        <is>
+          <t>guà pái</t>
+        </is>
+      </c>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>현판을 걸다, 개교/개업하다</t>
+        </is>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>新建的几所中学将在今年九月正式挂牌启用，有效缓解了入学压力。</t>
+        </is>
+      </c>
+      <c r="I768" t="inlineStr">
+        <is>
+          <t>我们新设立的分公司将于下周一举行挂牌仪式。</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>CHI-20260728-005</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>留神</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F769" t="inlineStr">
+        <is>
+          <t>liú shén</t>
+        </is>
+      </c>
+      <c r="G769" t="inlineStr">
+        <is>
+          <t>주의하다, 신경 쓰다</t>
+        </is>
+      </c>
+      <c r="H769" t="inlineStr">
+        <is>
+          <t>在人流量大的集市周边出行时，一定要留神脚下的道路安全。</t>
+        </is>
+      </c>
+      <c r="I769" t="inlineStr">
+        <is>
+          <t>路面刚下过雪有点滑，你走路的时候多留点神。</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>CHI-20260728-006</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>做手脚</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>zuò shǒu jiǎo</t>
+        </is>
+      </c>
+      <c r="G770" t="inlineStr">
+        <is>
+          <t>꼼수를 부리다, 몰래 조작하거나 손장난을 치다</t>
+        </is>
+      </c>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>严厉打击在产品质量检测报告中做手脚的违法行为。</t>
+        </is>
+      </c>
+      <c r="I770" t="inlineStr">
+        <is>
+          <t>做生意最讲究诚信，如果在合同条款里做手脚，早晚会失去客户。</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>CHI-20260728-007</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>留退路</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>liú tuì lù</t>
+        </is>
+      </c>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>플랜B를 준비하다, 만약의 사태에 대비해 도망칠 구멍을 남기다</t>
+        </is>
+      </c>
+      <c r="H771" t="inlineStr">
+        <is>
+          <t>做重大投资决策时，一定要给自己留退路，切忌孤注一掷。</t>
+        </is>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>即使谈判进展顺利，我们也得留一条退路，防止对方突然变卦。</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>CHI-20260728-008</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>倒计时</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>dào jì shí</t>
+        </is>
+      </c>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>카운트다운에 돌입하다, 시한이 임박하다</t>
+        </is>
+      </c>
+      <c r="H772" t="inlineStr">
+        <is>
+          <t>距离新学期开学已经进入倒计时，各项筹备工作正紧锣密鼓地进行。</t>
+        </is>
+      </c>
+      <c r="I772" t="inlineStr">
+        <is>
+          <t>新产品发布会已经进入倒计时，请公关团队做好最后的确认。</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>CHI-20260728-009</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>适得其反</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>shì dé qí fǎn</t>
+        </is>
+      </c>
+      <c r="G773" t="inlineStr">
+        <is>
+          <t>의도와 다르게 오히려 역효과가 나다</t>
+        </is>
+      </c>
+      <c r="H773" t="inlineStr">
+        <is>
+          <t>过度的教育焦虑反而会给孩子施加过大压力，结果适得其反。</t>
+        </is>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>如果盲目跟风做营销而忽视产品质量，后果可能会适得其反。</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>CHI-20260728-010</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>迎头赶上</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>yíng tóu gǎn shàng</t>
+        </is>
+      </c>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>전력을 다해 추격하다, 신속히 따라잡다</t>
+        </is>
+      </c>
+      <c r="H774" t="inlineStr">
+        <is>
+          <t>我国在新能源领域起步虽慢，但凭借政策支持已实现迎头赶上。</t>
+        </is>
+      </c>
+      <c r="I774" t="inlineStr">
+        <is>
+          <t>虽然我们在上半年的业绩暂时落后，但下半年依然有机会迎头赶上。</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>CHI-20260728-011</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>软硬兼施</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>ruǎn yìng jiān shī</t>
+        </is>
+      </c>
+      <c r="G775" t="inlineStr">
+        <is>
+          <t>회유와 압박을 병행하다, 강온 양면책을 쓰다</t>
+        </is>
+      </c>
+      <c r="H775" t="inlineStr">
+        <is>
+          <t>在解决复杂的拆迁搬迁问题时，工作组采取了软硬兼施的沟通策略。</t>
+        </is>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>面对油盐不进的谈判对手，我们有时需要软硬兼施才能逼对方妥协。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-29 | 791/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I775"/>
+  <dimension ref="A1:I792"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36841,6 +36841,805 @@
         </is>
       </c>
     </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>CHI-20260729-001</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>拼一把</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F776" t="inlineStr">
+        <is>
+          <t>pīn yī bǎ</t>
+        </is>
+      </c>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>한번 온 힘을 다해 도전해 보다</t>
+        </is>
+      </c>
+      <c r="H776" t="inlineStr">
+        <is>
+          <t>趁着年轻，不拼一把怎么知道自己能走多远？</t>
+        </is>
+      </c>
+      <c r="I776" t="inlineStr">
+        <is>
+          <t>虽然希望渺茫，但我还是决定拼一把。</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>CHI-20260729-002</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>占优势</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F777" t="inlineStr">
+        <is>
+          <t>zhàn yōushì</t>
+        </is>
+      </c>
+      <c r="G777" t="inlineStr">
+        <is>
+          <t>우위를 점하다, 유리하다</t>
+        </is>
+      </c>
+      <c r="H777" t="inlineStr">
+        <is>
+          <t>在就业市场上，有专业技能和实践经验的人更占优势。</t>
+        </is>
+      </c>
+      <c r="I777" t="inlineStr">
+        <is>
+          <t>他们在技术实力方面占绝对优势。</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>CHI-20260729-003</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>兑现</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F778" t="inlineStr">
+        <is>
+          <t>duìxiàn</t>
+        </is>
+      </c>
+      <c r="G778" t="inlineStr">
+        <is>
+          <t>약속이나 공약을 지키다, 이행하다</t>
+        </is>
+      </c>
+      <c r="H778" t="inlineStr">
+        <is>
+          <t>这位企业家赶到村里，兑现了自己发奖学金的承诺。</t>
+        </is>
+      </c>
+      <c r="I778" t="inlineStr">
+        <is>
+          <t>既然答应了客户，我们就必须按时兑现承诺。</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>CHI-20260729-004</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>拿得出手</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F779" t="inlineStr">
+        <is>
+          <t>ná de chū shǒu</t>
+        </is>
+      </c>
+      <c r="G779" t="inlineStr">
+        <is>
+          <t>남에게 자랑스럽게 내놓을 만하다</t>
+        </is>
+      </c>
+      <c r="H779" t="inlineStr">
+        <is>
+          <t>只有品质过硬的产品，才能在竞争激烈的市场上拿得出手。</t>
+        </is>
+      </c>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>我们公司终于做出来一套能拿得出的作品。</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>CHI-20260729-005</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>赶进度</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F780" t="inlineStr">
+        <is>
+          <t>gǎn jìndù</t>
+        </is>
+      </c>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>마감이나 정해진 일정을 맞추려 속도를 내다</t>
+        </is>
+      </c>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>工人们正在加班加点赶进度，确保工程按期完工。</t>
+        </is>
+      </c>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>为了赶进度，大家连续加班了好几天。</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>CHI-20260729-006</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>心里有底</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>xīnlǐ yǒu dǐ</t>
+        </is>
+      </c>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>속으로 자신감이 있다, 확신이나 대책이 서다</t>
+        </is>
+      </c>
+      <c r="H781" t="inlineStr">
+        <is>
+          <t>只要做足了准备，面对突发状况心里就有底。</t>
+        </is>
+      </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>查完资料以后，我对明天的面试心里有底了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>CHI-20260729-007</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>打铺垫</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>dǎ pūdiàn</t>
+        </is>
+      </c>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>밑바탕을 깔다, 사전 작업을 하다</t>
+        </is>
+      </c>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>高中三年的积累，为他考上名校打下了坚实的基础。</t>
+        </is>
+      </c>
+      <c r="I782" t="inlineStr">
+        <is>
+          <t>我先给领导打个铺垫，你过一会儿再去汇报。</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>CHI-20260729-008</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>抓紧</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>zhuājǐn</t>
+        </is>
+      </c>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>시간이나 기회를 놓치지 않고 바짝 서두르다</t>
+        </is>
+      </c>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>志愿填报即将截止，请考生抓紧时间提交。</t>
+        </is>
+      </c>
+      <c r="I783" t="inlineStr">
+        <is>
+          <t>时间不多了，大家抓紧收拾一下准备出发。</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>CHI-20260729-009</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>不计其数</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>bù jì qí shù</t>
+        </is>
+      </c>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>수없이 많다, 헤아릴 수 없다</t>
+        </is>
+      </c>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>这些年来，从这所学校走出的优秀毕业生不计其数。</t>
+        </is>
+      </c>
+      <c r="I784" t="inlineStr">
+        <is>
+          <t>网上关于这个话题的讨论不计其数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>CHI-20260729-010</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>止跌</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>zhǐ diē</t>
+        </is>
+      </c>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>(하락세나 저하를) 멈추다 / 반등의 계기를 마련하다</t>
+        </is>
+      </c>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>下一步将以更大力度激发投资内生动力，促进投资止跌回稳。</t>
+        </is>
+      </c>
+      <c r="I785" t="inlineStr">
+        <is>
+          <t>在相关政策的精准调控下，该地区的房价终于止跌企稳。</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>CHI-20260729-011</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>稳居</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F786" t="inlineStr">
+        <is>
+          <t>wěn jū</t>
+        </is>
+      </c>
+      <c r="G786" t="inlineStr">
+        <is>
+          <t>(순위나 자리를) 안정적으로 유지하다 / 확고히 지키다</t>
+        </is>
+      </c>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>用服务塑口碑！柘林城管满意度连续两年稳居全市前列。</t>
+        </is>
+      </c>
+      <c r="I786" t="inlineStr">
+        <is>
+          <t>这款智能手机的市场占有率已经连续三个季度稳居行业第一。</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>CHI-20260729-012</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>图文并茂</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>tú wén bìng mào</t>
+        </is>
+      </c>
+      <c r="G787" t="inlineStr">
+        <is>
+          <t>그림과 글이 잘 어우러지다 / 시각적으로 직관적이고 훌륭하다</t>
+        </is>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>通过图文并茂的形式，宣传本市生态环境执法工作的进展。</t>
+        </is>
+      </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>这份调研报告图文并茂，非常适合在企划会议上向客户展示。</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>CHI-20260729-013</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>抽空</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>chōu kòng</t>
+        </is>
+      </c>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>(바쁜 와중에) 짬을 내다 / 시간을 만들다</t>
+        </is>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>平时工作再忙，也要抽空多陪陪家人，注意劳逸结合。</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>这周末你能不能抽个空？我们一起讨论一下新项目的具体方案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>CHI-20260729-014</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>交底</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>jiāo dǐ</t>
+        </is>
+      </c>
+      <c r="G789" t="inlineStr">
+        <is>
+          <t>(상황·속내·속사정을) 솔직히 털어놓다 / 가감 없이 공유하다</t>
+        </is>
+      </c>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>项目正式开工之前，负责人必须要给全体团队人员交个底。</t>
+        </is>
+      </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>双方商务谈判前，经理先把我们公司的底线跟我交了底。</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>CHI-20260729-015</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>打包票</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>dǎ bāo piào</t>
+        </is>
+      </c>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>장담하다 / 확실하게 보증하다</t>
+        </is>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>在最终测试结果出来之前，谁也不敢跟客户打这个包票。</t>
+        </is>
+      </c>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>我敢跟你打包票，只要采用这个新流程，工作效率一定能提升。</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>CHI-20260729-016</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>拉一把</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>lā yī bǎ</t>
+        </is>
+      </c>
+      <c r="G791" t="inlineStr">
+        <is>
+          <t>(어려운 처지의 사람을) 도와주다 / 끌어주고 이끌다</t>
+        </is>
+      </c>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>在他创业最艰难的时候，正是几位老朋友伸手拉了他一把。</t>
+        </is>
+      </c>
+      <c r="I791" t="inlineStr">
+        <is>
+          <t>同事之间应该互相扶持，有人进度落后时大家要拉一把。</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>CHI-20260729-017</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>拖泥带水</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>tuō ní dài shuǐ</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>(일처리가) 매끄럽지 못하고 질질 끌다 / 우유부단하다</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>处理紧急突发事件一定要果断冷静，切忌拖泥带水。</t>
+        </is>
+      </c>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>他在做业务汇报时干脆利落、重点突出，一点也不拖泥带水。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-30 | 806/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I792"/>
+  <dimension ref="A1:I807"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37640,6 +37640,711 @@
         </is>
       </c>
     </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>CHI-20260730-001</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>熬夜</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>áo yè</t>
+        </is>
+      </c>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>밤을 새우며 일이나 공부를 하다</t>
+        </is>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>学霸分享经验时表示，与其每天熬夜刷题，不如提高课堂上的学习效率。</t>
+        </is>
+      </c>
+      <c r="I793" t="inlineStr">
+        <is>
+          <t>为了准备明天的方案汇报，我们整个团队昨晚又熬夜了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>CHI-20260730-002</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>添乱</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>tiān luàn</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>도움은커녕 귀찮게 하거나 문제를 더 벌리다</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>在开展环保整治行动时，希望部分违规企业不要给大局添乱，配合停产整改。</t>
+        </is>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>大家现在都在忙着准备活动，你就别在这里添乱了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>CHI-20260730-003</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>说话算话</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>shuō huà suàn huà</t>
+        </is>
+      </c>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>한 번 한 말을 반드시 책임지고 지키다</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>爱心企业家说话算话，将五万元现金重奖双手交到了考上清华的学子手中。</t>
+        </is>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>既然答应了这周末带孩子去游乐园，就要说话算话。</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>CHI-20260730-004</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>蒸蒸日上</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>zhēng zhēng rì shàng</t>
+        </is>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>사업이나 성과가 나날이 번창하고 좋아지다</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>受益于一系列利好政策，该开发区内上市公司的业务呈现出蒸蒸日上的良好态势。</t>
+        </is>
+      </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>祝贵公司在新的财年里事业蒸蒸日上，业绩再创高峰。</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>CHI-20260730-005</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>啃硬骨头</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>kěn yìng gǔ tou</t>
+        </is>
+      </c>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>어려운 난제를 끝까지 해결하려 들다</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>改革已经进入深水区，我们需要敢于啃硬骨头。</t>
+        </is>
+      </c>
+      <c r="I797" t="inlineStr">
+        <is>
+          <t>这个项目的技术难题很多，全靠研发部门敢啃硬骨头才顺利攻克。</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>CHI-20260730-006</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>拍胸脯</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>pāi xiōng pú</t>
+        </is>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>가슴을 두드리며 장담하다</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>他拍胸脯保证，月底之前一定完成工商变更登记。</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>别光顾着拍胸脯保证，到时候拿不出结果可就尴尬了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>CHI-20260730-007</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>划清界限</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>huà qīng jiè xiàn</t>
+        </is>
+      </c>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>선·경계를 확실히 긋다</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>外交部明确表示，中方与此类不实报道划清界限。</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>我们必须与违规违纪行为划清界限，坚守原则。</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>CHI-20260730-008</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>算总账</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>suàn zǒng zhàng</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>최종 결산을 하다, 총 책임을 물다</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>对长期破坏生态环境的行为，迟早是要算总账的。</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>年终绩效考核时，公司会对每个项目的收益算总账。</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>CHI-20260730-009</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>找突破口</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>zhǎo tū pò kǒu</t>
+        </is>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>돌파구를 찾다</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>为了促进投资止跌回稳，发改委积极寻找新的突破口。</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>在传统业务增长放缓时，公司决定在海外市场找突破口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>CHI-20260730-010</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>下苦功</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>xià kǔ gōng</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>뼈를 깎는 노력을 기울이다</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>高考能考出高分，离不开她在平时下的苦功。</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>要想在短时间内掌握一门外语，不下苦功是不行的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>CHI-20260730-011</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>抓落实</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>zhuā luò shí</t>
+        </is>
+      </c>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>(방침이나 정책을) 실천에 옮기다, 이행을 철저히 챙기다</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>下一步关键在于狠抓落实，推动各项政策落地见效。</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>好的规划如果不去抓落实，最终只会变成一纸空文。</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>CHI-20260730-012</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>搭便车</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>dā biàn chē</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>무임승차하다, 남의 성과나 편의에 얹혀가다</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>在合作推进项目中，有些地方只想搭便车而不愿付出。</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>做小组作业时不能只想着搭便车，每个人都要承担一部分任务。</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>CHI-20260730-013</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>抓眼球</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>zhuā yǎn qiú</t>
+        </is>
+      </c>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>시선을 사로잡다, 눈길을 끌다</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>媒体不能靠耸人听闻的假新闻来抓眼球。</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>这款产品在包装设计上非常抓眼球，上市后销量很好。</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>CHI-20260730-014</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>拉赞助</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>lā zàn zhù</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>후원을 유치하다, 협찬을 받다</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>为了举办这次社区环保活动，志愿者们到处拉赞助。</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>大学社团举办大型晚会前，外联部需要负责拉赞助。</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>CHI-20260730-015</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>扣帽子</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>kòu mào zi</t>
+        </is>
+      </c>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>낙인을 찍다, 억지 죄목·프레임을 씌우다</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>针对无端质问，外交部坚决反对随意给中方扣帽子。</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>在没有弄清事实真相之前，不要随便给别人扣帽子。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-07-31 | 817/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I807"/>
+  <dimension ref="A1:I818"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38345,6 +38345,523 @@
         </is>
       </c>
     </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>CHI-20260731-001</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>露馅</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>lòu xiàn</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>밑천이 드러나다, 거짓말이나 비밀이 들통나다</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>网传九寨沟湖水是用颜料染色的谣言，在专业辟谣后瞬间露馅了。</t>
+        </is>
+      </c>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>他装作听不懂中文，结果听到大家讲笑话忍不住笑出来，一下子露馅了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>CHI-20260731-002</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>翻盘</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>fān pán</t>
+        </is>
+      </c>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>판세를 뒤집다, 역전하다</t>
+        </is>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>高考前一个月数学成绩提升了40多分，他靠着坚韧不拔的毅力实现了逆风翻盘。</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>虽然前半场落后很多，但队员们配合默契，在最后三分钟实现了漂亮的大翻盘。</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>CHI-20260731-003</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>加把劲</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>jiā bǎ jìn</t>
+        </is>
+      </c>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>힘을 더 내다, 피치를 올리다</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>临考前最后一个月是关键冲刺期，老师不断鼓励大家再加把劲。</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>距离项目截止日期只剩三天了，大家再加把劲，争取提前完工。</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>CHI-20260731-004</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>跟风</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>gēn fēng</t>
+        </is>
+      </c>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>맹목적으로 따라 하다, 트렌드에 유행처럼 쏠리다</t>
+        </is>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>填报志愿是关乎人生规划的大事，考生应该结合自身兴趣，而不是盲目跟风。</t>
+        </is>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>做投资最忌讳盲目跟风，必须要有自己独立的分析和判断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>CHI-20260731-005</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>吃苦</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>chī kǔ</t>
+        </is>
+      </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>고생을 참다, 쓴맛을 감내하다</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>在高原极寒地区开展生态环境保护工作，没有吃苦耐劳的精神是坚持不下来的。</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>年轻人多吃点苦不是坏事，这能锻炼你的意志力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>CHI-20260731-006</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>抢风头</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>qiǎng fēng tou</t>
+        </is>
+      </c>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>시선을 사로잡다, 주객이 전도되다</t>
+        </is>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>深圳科学家用菌丝织出时尚裙子，在展览上一亮相就抢尽了风头。</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>她在发布会上穿的那件设计独特的礼服完全抢了现场其他人的风头。</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>CHI-20260731-007</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>硬核</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>yìng hé</t>
+        </is>
+      </c>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>확실한, 막강한, 진짜 실력이 뛰어난</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>高考考出691分并手写18本错题本，这样的学习方法可谓是非常硬核。</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>这家工厂展示的自动化生产线非常硬核，吸引了众多客户参观。</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>CHI-20260731-008</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>托关系</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>tuō guān xì</t>
+        </is>
+      </c>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>줄을 대다, 청탁하다</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>找工作要靠真本事，光靠托关系是长久不了的。</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>他为了把孩子送进名校，四处托关系找人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>CHI-20260731-009</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>撑腰</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>chēng yāo</t>
+        </is>
+      </c>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>든든한 버팀목이 되어주다, 뒤를 봐주다</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>有国家政策撑腰，企业发展绿色环保产业更有底气了。</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>别担心，有整个团队给你撑腰，你放手去做吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>CHI-20260731-010</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>讨公道</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>tǎo gōng dào</t>
+        </is>
+      </c>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>정당한 해명이나 사과를 요구하다, 공평함을 구하다</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>针对小区异味问题，业主们集体向相关部门讨公道。</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>消费者有权利为不合格产品的质量问题去向商家讨公道。</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>CHI-20260731-011</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>严丝合缝</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>yán sī hé fèng</t>
+        </is>
+      </c>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>빈틈없이 딱 맞물리다, 완벽하게 일치하다</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>这项新技术的对接流程设计得严丝合缝，没有任何漏洞。</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>两个部门在项目衔接上做得严丝合缝，大大提高了效率。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-03 | 826/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I818"/>
+  <dimension ref="A1:I827"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38862,6 +38862,429 @@
         </is>
       </c>
     </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>CHI-20260803-001</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>亮眼</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>liàng yǎn</t>
+        </is>
+      </c>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>실적이 뛰어난, 눈에 띄게 돋보이는</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>在今年上半年经济放缓的大环境下，该公司拿出了极其亮眼的成绩单。</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>他在这次新产品发布会上的表现非常亮眼，赢得了全场的掌声。</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>CHI-20260803-002</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>换汤不换药</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>huàn tāng bù huàn yào</t>
+        </is>
+      </c>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>겉모습만 바꾸고 본질은 그대로이다, 눈 가리고 아웅하다</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>虽然换了新的名字和包装，但教学模式依然是换汤不换药。</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>这次的新方案看起来很酷，本质上还是换汤不换药的旧东西。</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>CHI-20260803-003</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>起色</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>qǐ sè</t>
+        </is>
+      </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>호전, 실적이나 상태가 좋아지는 기미</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>经过几个月的调整，公司的销售业绩终于有了明显的起色。</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>吃了几天药之后，他的病情终于大有起色，精神好多了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>CHI-20260803-004</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>跑偏</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>pǎo piān</t>
+        </is>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>방향이 어긋나다, 삼천포로 빠지다</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>会议开到一半，大家讨论的主题渐渐跑偏了，偏离了原定议程。</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>写论文时一定要抓紧核心论点，千万别把方向给跑偏了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>CHI-20260803-005</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>紧巴巴</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>jǐn bā bā</t>
+        </is>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>여유 없이 빡빡하다, 아슬아슬하다</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>离考试只剩下两天时间了，复习进度安排得非常紧巴巴。</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>这个月买了新手机之后，我的日子过得相当紧巴巴。</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>CHI-20260803-006</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>抄近路</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>chāo jìn lù</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>지름길로 가다, 꼼수를 쓰거나 편법을 타다</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>做学术研究需要脚踏实地，想抄近路往往适得其反。</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>在基础技能训练上没有近路可抄，只能一遍遍练习。</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>CHI-20260803-007</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>知行合一</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>zhī xíng hé yī</t>
+        </is>
+      </c>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>지식과 행동이 하나로 일치함, 지행합일</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>只有做到知行合一，才能真正把环保理念落实到日常生活中。</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>学习职业技能最讲究知行合一，光懂理论不动手是不行的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>CHI-20260803-008</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>打抱不平</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>dǎ bào bù píng</t>
+        </is>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>억울하거나 불합리한 일을 보고 남을 두둔하고 도와주다</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>看到同事在工作中受了委屈，他总是第一个站出来打抱不平。</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>他性格直爽，经常为了下属的合理利益向领导打抱不平。</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>CHI-20260803-009</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>划等号</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>huà děng hào</t>
+        </is>
+      </c>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>동일시하다, 같다고 여기다</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>学历高并不等同于能力强，两者不能简单地划等号。</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>工作时间的长短不能和工作效率的高低直接划等号。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-04 | 833/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I827"/>
+  <dimension ref="A1:I834"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39285,6 +39285,335 @@
         </is>
       </c>
     </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>CHI-20260804-001</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>趁热打铁</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>chèn rè dǎ tiě</t>
+        </is>
+      </c>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>쇠뿔도 단김에 빼다, 기회를 놓치지 않다</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>趁着政策利好的东风，企业决定趁热打铁拓展市场。</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>既然大家想法一致，不如趁热打铁把合同签了吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>CHI-20260804-002</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>门槛</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>mén kǎn</t>
+        </is>
+      </c>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>진입 장벽, 자격 조건/기준</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>这项技能培训降低了学习门槛，让更多学生受益。</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr">
+        <is>
+          <t>这个岗位的入职门槛很高，必须具备五年以上相关经验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>CHI-20260804-003</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>打打闹闹</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>dǎ dǎ nào nào</t>
+        </is>
+      </c>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>장난치다, 시끌벅적하게 지내다</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>校园里的孩子们打打闹闹，充满了青春活力。</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>他们俩从小一起打打闹闹长大，感情非常好。</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>CHI-20260804-004</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>临场发挥</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>lín chǎng fā huī</t>
+        </is>
+      </c>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>현장 발휘, 즉흥적인 대응</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>在直播带货中，所谓的临场发挥不能成为违法的免责借口。</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>他在演讲中的临场发挥非常出色，赢得了全场的掌声。</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>CHI-20260804-005</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>追逐梦想</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>zhuī zhú mèng xiǎng</t>
+        </is>
+      </c>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>꿈을 좇다, 꿈을 향해 달려가다</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>毕业多年后再考入心仪的大学，追逐梦想何错之有。</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>无论年纪多大，都有追逐梦想的权利。</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>CHI-20260804-006</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>站住脚</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>zhàn zhù jiǎo</t>
+        </is>
+      </c>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>입지를 다지다, 자리를 잡다</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>企业只有靠过硬的产品质量，才能在市场上站住脚。</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>新人想要在职场上站住脚，能力和态度缺一不可。</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>CHI-20260804-007</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>实打实</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>shí dǎ shí</t>
+        </is>
+      </c>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>확실한, 과장 없는, 진짜의</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>出台五项帮扶举措，给毕业生提供实打实的支持。</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>我们提供的都是实打实的服务，没有任何虚假成分。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-05 | 842/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I834"/>
+  <dimension ref="A1:I843"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39614,6 +39614,429 @@
         </is>
       </c>
     </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>CHI-20260805-001</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>卷起来</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>juǎn qǐ lai</t>
+        </is>
+      </c>
+      <c r="G835" t="inlineStr">
+        <is>
+          <t>경쟁이 대단히 치열해지다, 림보/내부 경쟁에 몰리다</t>
+        </is>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>高考刚结束，各大高职院校和补录市场的招生竞争又开始卷起来了。</t>
+        </is>
+      </c>
+      <c r="I835" t="inlineStr">
+        <is>
+          <t>现在的职场环境太卷了，大家都在利用周末时间偷偷加班考证。</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>CHI-20260805-002</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>抢手货</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>qiǎng shǒu huò</t>
+        </is>
+      </c>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>인기 품목, 주가가 높아서 서로 데려가려는 인재/상품</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>掌握核心技术的复合型人才，在今年事业单位和国企招聘中成了抢手货。</t>
+        </is>
+      </c>
+      <c r="I836" t="inlineStr">
+        <is>
+          <t>这种具备跨界技能的新生代程序员在求职市场上绝对是抢手货。</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>CHI-20260805-003</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>铺后路</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>pū hòu lù</t>
+        </is>
+      </c>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>만약의 사태를 대비해 퇴로를 마련하다</t>
+        </is>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>不少考生在等待第一批录取结果的同时，也在关注补录志愿，为自己铺后路。</t>
+        </is>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>做任何创业投资都要留有余地，提前为自己铺好后路。</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>CHI-20260805-004</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>摸门道</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>mō mén dao</t>
+        </is>
+      </c>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>요령을 터득하다, 핵심 감을 잡다</t>
+        </is>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>刚接触业务时一头雾水，跟着老员工跑了几趟才慢慢摸出点门道来。</t>
+        </is>
+      </c>
+      <c r="I838" t="inlineStr">
+        <is>
+          <t>做自营账号不能瞎碰，得先摸清平台流量推荐的门道。</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>CHI-20260805-005</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>赶趟儿</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>gǎn tàng r</t>
+        </is>
+      </c>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>제때 맞추다, 시간에 늦지 않다</t>
+        </is>
+      </c>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>补录征集志愿8月13日才截止，现在准备材料完全赶趟儿。</t>
+        </is>
+      </c>
+      <c r="I839" t="inlineStr">
+        <is>
+          <t>别太着急，距离末班车发车还有半个小时，咱们绝对赶趟儿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>CHI-20260805-006</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>留后手</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>liú hòu shǒu</t>
+        </is>
+      </c>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>만약에 대비해 비장의 수/카드를 남겨두다</t>
+        </is>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>在复杂的商业谈判中，不能把底牌一次性全亮出来，得留后手。</t>
+        </is>
+      </c>
+      <c r="I840" t="inlineStr">
+        <is>
+          <t>做方案时最好准备一套备用计划，给自己留个后手。</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>CHI-20260805-007</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>下工夫</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>xià gōng fu</t>
+        </is>
+      </c>
+      <c r="G841" t="inlineStr">
+        <is>
+          <t>공을 들이다, 정성을 쏟다</t>
+        </is>
+      </c>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>要想把这个课题做深做透，必须在数据调研上下工夫。</t>
+        </is>
+      </c>
+      <c r="I841" t="inlineStr">
+        <is>
+          <t>他在口语练习上了不少工夫，所以发音非常地道。</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>CHI-20260805-008</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>见分晓</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>jiàn fēn xiǎo</t>
+        </is>
+      </c>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>결말이 나다, 승패/결과가 분명해지다</t>
+        </is>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>这场竞标非常激烈，谁能胜出明天就会见分晓。</t>
+        </is>
+      </c>
+      <c r="I842" t="inlineStr">
+        <is>
+          <t>等下个月的销售数据出来，新策略的效果自然见分晓。</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>CHI-20260805-009</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>咬紧牙关</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>yǎo jǐn yá guān</t>
+        </is>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>이를 악물다, 극복하려고 참다</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>创业初期资金非常紧张，大家咬紧牙关才挺了过来。</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>面对如此巨大的舆论压力，团队咬紧牙关按时完成了交期。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-06 | 847/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I843"/>
+  <dimension ref="A1:I848"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40037,6 +40037,241 @@
         </is>
       </c>
     </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>CHI-20260806-001</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>踩雷</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>cǎi léi</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>지뢰를 밟다, 실패사례나 안 좋은 것을 택하다</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>装修房子前一定要多做功课，避免买到不环保的材料踩雷。</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>买之前多看看买家评价，这样才不会踩雷。</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>CHI-20260806-002</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>买账</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>mǎi zhàng</t>
+        </is>
+      </c>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>(남의 정성·주장·물건 등을) 인정해 주다, 가치를 알아주다</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>如果产品本身不过硬，宣传得再好消费者也不买账。</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>你提出的这个解释根本没有说服力，大家不会买账的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>CHI-20260806-003</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>露脸</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>lù liǎn</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>얼굴을 비추다, 돋보이다</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>作为优秀的毕业生代表在台上发言，这次他真是露脸了。</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>明天的发布会上，你一定要好好表现，多露露脸。</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>CHI-20260806-004</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>踢皮球</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>tī pí qiú</t>
+        </is>
+      </c>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>책임을 이리저리 서로 전가하다</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>面对群众提出的诉求，有关部门绝不能互相踢皮球。</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>办理此项业务时，窗口工作人员相互踢皮球，引发了市民不满。</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>CHI-20260806-005</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>齐头并进</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>qí tóu bìng jìn</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>여러 분야나 일이 동시에 함께 발전해 나가다</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>公司不仅注重经济效益，还与生态环境保护齐头并进。</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>我们在推进新项目的同时，原有业务的质量提升也须齐头并进。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-07 | 859/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I848"/>
+  <dimension ref="A1:I860"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40272,6 +40272,570 @@
         </is>
       </c>
     </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>CHI-20260807-001</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>牵头</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>qiān tóu</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>주도하다, 앞장서서 이끌다</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>这次跨部门合作由我们研发部来牵头推进。</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>针对这次环境治理项目，政府决定由环保局牵头联合多部门共同办理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>CHI-20260807-002</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>揽活</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>lǎn huó</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>(일이나 책임을) 자청해서 맡다, 끌어안다</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>你自己手头的事情都没做完，怎么还跑去外面瞎揽活？</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>他在团队里总是主动揽活，大家都非常信任他的能力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>CHI-20260807-003</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>落榜</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>luò bǎng</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>시험에서 떨어지다, 낙방하다</t>
+        </is>
+      </c>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>虽然这次中考不幸落榜，但他没有放弃，准备继续复读。</t>
+        </is>
+      </c>
+      <c r="I851" t="inlineStr">
+        <is>
+          <t>即使一时落榜也不要灰心，人生还有很多重新开始的机会。</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>CHI-20260807-004</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>估分</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>gū fēn</t>
+        </is>
+      </c>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>(시험 후) 가채점하다</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>高考结束后，老师指导大家结合标准答案进行估分。</t>
+        </is>
+      </c>
+      <c r="I852" t="inlineStr">
+        <is>
+          <t>考完试别急着出去玩，先认真估分以便填报志愿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>CHI-20260807-005</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>纸上谈兵</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>zhǐ shàng tán bīng</t>
+        </is>
+      </c>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>탁상공론하다, 실전 경험 없이 말로만 이론을 늘어놓다</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>规划如果只停留在图纸上，不过是纸上谈兵罢了。</t>
+        </is>
+      </c>
+      <c r="I853" t="inlineStr">
+        <is>
+          <t>我们做方案不能纸上谈兵，必须去现场做实地调研。</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>CHI-20260807-006</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>抢眼</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>qiǎng yǎn</t>
+        </is>
+      </c>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>눈길을 사로잡다, 돋보이다</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>市属国企在今年上半年交出了一份十分抢眼的成绩单。</t>
+        </is>
+      </c>
+      <c r="I854" t="inlineStr">
+        <is>
+          <t>她在这次新品发布会上的表现非常抢眼，得到了各方好评。</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>CHI-20260807-007</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>打太极</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>dǎ tài jí</t>
+        </is>
+      </c>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>책임을 회피하다, 핑계를 대며 미루다</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>面对记者关于建设进度的追问，相关部门一直在打太极。</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr">
+        <is>
+          <t>遇事要直截了当解决，互相打太极只会降低工作效率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>CHI-20260807-008</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>抓耳挠腮</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>zhuā ěr náo sāi</t>
+        </is>
+      </c>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>어쩔 줄 몰라 안절부절못하다, 애가 타다</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>面对这道超纲的高考压轴题，不少考生急得抓耳挠腮。</t>
+        </is>
+      </c>
+      <c r="I856" t="inlineStr">
+        <is>
+          <t>遇到实在解决不了的难题，光抓耳挠腮也没用，赶紧请教老员工吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>CHI-20260807-009</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>攻关</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>gōng guān</t>
+        </is>
+      </c>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>난관을 극복하다, 핵심 기술을 단맥으로 연구개발하다</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>青年团队南下攻关环保变压器，成功打破了技术瓶颈。</t>
+        </is>
+      </c>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>为了攻下一个技术难关，研发小组连续加班熬夜了一个星期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>CHI-20260807-010</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>撬动</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>qiào dòng</t>
+        </is>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>지렛대 역할을 하여 이끌어내다, 파급 효과를 주다</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>高考后的考后经济有效地撬动了整个暑期消费市场。</t>
+        </is>
+      </c>
+      <c r="I858" t="inlineStr">
+        <is>
+          <t>政府希望通过少量引导资金，撬动更多的社会资本投入环保产业。</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>CHI-20260807-011</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>联动</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>lián dòng</t>
+        </is>
+      </c>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>연계하여 움직이다, 공조하다</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>大学多部门联动推进劳动育人，取得了显著效果。</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr">
+        <is>
+          <t>遇到突发自然灾害时，气象、交通和救援部门需要实时联动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>CHI-20260807-012</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>补录</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>bǔ lù</t>
+        </is>
+      </c>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>추가 모집하다, 결원을 보충하여 채용/입학시키다</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>海南中招补录征集志愿填报工作将于8月13日正式开始。</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr">
+        <is>
+          <t>如果你第一次志愿没被录取，还可以关注一下后续的补录机会。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-10 | 868/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I860"/>
+  <dimension ref="A1:I869"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40836,6 +40836,429 @@
         </is>
       </c>
     </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>CHI-20260810-001</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>翻车</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>fān chē</t>
+        </is>
+      </c>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>망하다, 큰 실수를 하다, 신뢰를 잃다</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>某品牌推出的AI女主角广告因为技术和审美问题遭遇网友吐槽，彻底翻车后被迫下架。</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>本来想在大家面前露一手，结果操作失误直接翻车了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>CHI-20260810-002</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>拼命</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>pīn mìng</t>
+        </is>
+      </c>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>목숨 걸고 노력하다, 죽기 살기로 하다</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>为了凑齐学费并补贴家用，这位18岁的高考高分学生暑假期间拼命跑外卖。</t>
+        </is>
+      </c>
+      <c r="I862" t="inlineStr">
+        <is>
+          <t>离考试只剩一周了，大家都在拼命复习。</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>CHI-20260810-003</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>坐地起价</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>zuò dì qǐ jià</t>
+        </is>
+      </c>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>터무니없이 가격을 올리다, 갑자기 바가지를 씌우다</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>部分培训机构趁着报名高峰期坐地起价，引起了许多消费者的强烈不满。</t>
+        </is>
+      </c>
+      <c r="I863" t="inlineStr">
+        <is>
+          <t>旅游旺季时，个别酒店坐地起价的行为受到了严格惩处。</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>CHI-20260810-004</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>捡漏</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>jiǎn lòu</t>
+        </is>
+      </c>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>뜻밖의 행운으로 득템하다, 싸게 가치 있는 것을 건지다</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>他在电商平台上打算捡漏买黄金，结果却遭遇了商家标错价格的纠纷。</t>
+        </is>
+      </c>
+      <c r="I864" t="inlineStr">
+        <is>
+          <t>我今天在二手市场捡漏买到了一本绝版图书。</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>CHI-20260810-005</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>赶时间</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>gǎn shí jiān</t>
+        </is>
+      </c>
+      <c r="G865" t="inlineStr">
+        <is>
+          <t>시간에 쫓기다, 바쁘게 서두르다</t>
+        </is>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>受台风天气影响列车停运，急着赶时间的旅客不得不重新规划路线。</t>
+        </is>
+      </c>
+      <c r="I865" t="inlineStr">
+        <is>
+          <t>我现在有点赶时间，咱们改天再聚吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>CHI-20260810-006</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>闹心</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>nào xīn</t>
+        </is>
+      </c>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>속상하고 짜증 나다, 답답하다</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>预订好的航班连续因为天气原因取消，让人感到特别闹心。</t>
+        </is>
+      </c>
+      <c r="I866" t="inlineStr">
+        <is>
+          <t>遇到这种说不清的事情，心里别提多闹心了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>CHI-20260810-007</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>擦亮眼睛</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>cā liàng yǎn jing</t>
+        </is>
+      </c>
+      <c r="G867" t="inlineStr">
+        <is>
+          <t>눈을 똑똑히 뜨다, 현혹되지 않고 주의하다</t>
+        </is>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>面对网络上的各种谣言和陷阱，大家要擦亮眼睛。</t>
+        </is>
+      </c>
+      <c r="I867" t="inlineStr">
+        <is>
+          <t>投资理财时必须擦亮眼睛，谨防高收益骗局。</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>CHI-20260810-008</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>挺身而出</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>tǐng shēn ér chū</t>
+        </is>
+      </c>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>위기 상황에서 용감하게 나서다</t>
+        </is>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>在危急时刻，总有许多志愿者挺身而出守护家园。</t>
+        </is>
+      </c>
+      <c r="I868" t="inlineStr">
+        <is>
+          <t>面对不公正的待遇，他毫不犹豫地挺身而出为其鸣不平。</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>CHI-20260810-009</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>发火</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>fā huǒ</t>
+        </is>
+      </c>
+      <c r="G869" t="inlineStr">
+        <is>
+          <t>화를 내다, 성질을 부리다</t>
+        </is>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>遇到突发状况要冷静沟通，盲目发火解决不了问题。</t>
+        </is>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>经理很少发火，但今天因为严重的质量问题大发雷霆。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-11 | 880/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I869"/>
+  <dimension ref="A1:I881"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41259,6 +41259,570 @@
         </is>
       </c>
     </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>CHI-20260811-001</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>焕然一新</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>huàn rán yì xīn</t>
+        </is>
+      </c>
+      <c r="G870" t="inlineStr">
+        <is>
+          <t>완전히 새로워지다, 몰라보게 싹 바뀌다</t>
+        </is>
+      </c>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>经过了几个月的精心改造，这所老学校在开学前终于焕然一新了。</t>
+        </is>
+      </c>
+      <c r="I870" t="inlineStr">
+        <is>
+          <t>重新装修后，办公室的环境让人感觉焕然一新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>CHI-20260811-002</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>多点开花</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>duō diǎn kāi huā</t>
+        </is>
+      </c>
+      <c r="G871" t="inlineStr">
+        <is>
+          <t>다방면에서 결실을 맺다, 성과가 신속히 퍼지다</t>
+        </is>
+      </c>
+      <c r="H871" t="inlineStr">
+        <is>
+          <t>学校不仅在文化课上成绩优异，在体育和艺术赛事中也是多点开花。</t>
+        </is>
+      </c>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>我们公司的新业务在各个城市多点开花，业绩大幅提升。</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>CHI-20260811-003</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>搞砸</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>gǎo zá</t>
+        </is>
+      </c>
+      <c r="G872" t="inlineStr">
+        <is>
+          <t>일을 망치다, 죽을 쑤다</t>
+        </is>
+      </c>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>因为一时粗心大意，他把好好的面试给搞砸了。</t>
+        </is>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>别太紧张，越紧张越容易把事情搞砸。</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>CHI-20260811-004</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>蹭</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>cèng</t>
+        </is>
+      </c>
+      <c r="G873" t="inlineStr">
+        <is>
+          <t>얹혀가다, 슬쩍 혜택을 얻다 (蹭热度 등)</t>
+        </is>
+      </c>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>不少品牌想借着这个热门话题蹭一下热度做推广。</t>
+        </is>
+      </c>
+      <c r="I873" t="inlineStr">
+        <is>
+          <t>今天车子坏了，我是蹭同事的车回家的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>CHI-20260811-005</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>站稳脚跟</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>zhàn wěn jiǎo gēn</t>
+        </is>
+      </c>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>확실하게 입지를 다지다, 자리잡다</t>
+        </is>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>经过几年的努力，这家新品牌终于在激烈的行业竞争中站稳了脚跟。</t>
+        </is>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>新手入职后的当务之急是在岗位上尽快站稳脚跟。</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>CHI-20260811-006</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>占先机</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>zhàn xiān jī</t>
+        </is>
+      </c>
+      <c r="G875" t="inlineStr">
+        <is>
+          <t>우위를 선점하다, 기선을 제압하다</t>
+        </is>
+      </c>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>企业只有抓住技术创新的机遇，才能在未来市场中占得先机。</t>
+        </is>
+      </c>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>早一步进入这个新兴领域，就能在竞争中占先机。</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>CHI-20260811-007</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>软实力</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>ruǎn shí lì</t>
+        </is>
+      </c>
+      <c r="G876" t="inlineStr">
+        <is>
+          <t>소프트 파워, 내실 있는 역량</t>
+        </is>
+      </c>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>提升教学质量不仅要改善硬件，更要注重提升学校的文化软实力。</t>
+        </is>
+      </c>
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>沟通能力和团队协作力是职场中非常重要的软实力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>CHI-20260811-008</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>铺路搭桥</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>pū lù dā qiáo</t>
+        </is>
+      </c>
+      <c r="G877" t="inlineStr">
+        <is>
+          <t>가교 역할을 하다, 발판과 기회를 마련해 주다</t>
+        </is>
+      </c>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>学校积极推动产学研结合，为毕业生的就业铺路搭桥。</t>
+        </is>
+      </c>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>政府出台了多项扶持政策，为青年创业者铺路搭桥。</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>CHI-20260811-009</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>睁一只眼闭一只眼</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>zhēng yì zhī yǎn bì yì zhī yǎn</t>
+        </is>
+      </c>
+      <c r="G878" t="inlineStr">
+        <is>
+          <t>못 본 척 눈감아주다, 대충 넘어가지다</t>
+        </is>
+      </c>
+      <c r="H878" t="inlineStr">
+        <is>
+          <t>对于破坏环境的违法行为，监管部门绝不能睁一只眼闭一只眼。</t>
+        </is>
+      </c>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>原则性的问题绝对不能睁一只眼闭一只眼，必须严格依规处理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>CHI-20260811-010</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>擦亮招牌</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>cā liàng zhāo pái</t>
+        </is>
+      </c>
+      <c r="G879" t="inlineStr">
+        <is>
+          <t>브랜드나 지역/기관의 명성과 간판을 더 빛내다</t>
+        </is>
+      </c>
+      <c r="H879" t="inlineStr">
+        <is>
+          <t>通过引入优质教育资源，该区进一步擦亮了优质教育的招牌。</t>
+        </is>
+      </c>
+      <c r="I879" t="inlineStr">
+        <is>
+          <t>我们应该不断提升服务品质，切实用口碑擦亮企业的招牌。</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>CHI-20260811-011</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>挑三拣四</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr">
+        <is>
+          <t>tiāo sān jiǎn sì</t>
+        </is>
+      </c>
+      <c r="G880" t="inlineStr">
+        <is>
+          <t>이것저것 지나치게 까다롭게 가리다</t>
+        </is>
+      </c>
+      <c r="H880" t="inlineStr">
+        <is>
+          <t>找工作时不能挑三拣四，先积累一线实战经验才是关键。</t>
+        </is>
+      </c>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>在就业压力大的背景下，踏实做事比挑三拣四重要得多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>CHI-20260811-012</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>甩手掌柜</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>shuǎi shǒu zhǎng guì</t>
+        </is>
+      </c>
+      <c r="G881" t="inlineStr">
+        <is>
+          <t>손 하나 까딱 않고 관망만 하는 책임자, 무책임하게 방관하는 사람</t>
+        </is>
+      </c>
+      <c r="H881" t="inlineStr">
+        <is>
+          <t>校长要做教育改革的领头羊，而不是只发号施令的甩手掌柜。</t>
+        </is>
+      </c>
+      <c r="I881" t="inlineStr">
+        <is>
+          <t>作为项目负责人，你必须亲力亲为，不能当甩手掌柜。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-12 | 892/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I881"/>
+  <dimension ref="A1:I893"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41823,6 +41823,570 @@
         </is>
       </c>
     </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>CHI-20260812-001</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>查漏补缺</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>chá lòu bǔ quē</t>
+        </is>
+      </c>
+      <c r="G882" t="inlineStr">
+        <is>
+          <t>부족한 부분을 찾아 보완하다</t>
+        </is>
+      </c>
+      <c r="H882" t="inlineStr">
+        <is>
+          <t>在平时地复习和自习中，最重要的就是精准查漏补缺，把没弄懂的知识点彻底搞懂。</t>
+        </is>
+      </c>
+      <c r="I882" t="inlineStr">
+        <is>
+          <t>这次期中考试结束后，我们要好好总结，争取查漏补缺。</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>CHI-20260812-002</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>摆烂</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>bǎi làn</t>
+        </is>
+      </c>
+      <c r="G883" t="inlineStr">
+        <is>
+          <t>자포자기하다, 막나가다</t>
+        </is>
+      </c>
+      <c r="H883" t="inlineStr">
+        <is>
+          <t>遇到困难绝不能选择直接摆烂，而是要想办法解决眼前的危机。</t>
+        </is>
+      </c>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>虽然这次成绩不理想，但你也不能就这样直接摆烂啊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>CHI-20260812-003</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>严阵以待</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>yán zhèn yǐ dài</t>
+        </is>
+      </c>
+      <c r="G884" t="inlineStr">
+        <is>
+          <t>만반의 태세를 갖추고 기다리다</t>
+        </is>
+      </c>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>面对台风的袭击，松江区教育系统各方力量迅速集结，严阵以待。</t>
+        </is>
+      </c>
+      <c r="I884" t="inlineStr">
+        <is>
+          <t>面对即将来临的行业大考，整个团队都已经严阵以待。</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>CHI-20260812-004</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>闻令而动</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>wén lìng ér dòng</t>
+        </is>
+      </c>
+      <c r="G885" t="inlineStr">
+        <is>
+          <t>명령을 받자마자 지체 없이 움직이다</t>
+        </is>
+      </c>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>在救援指令下达后，志愿服务团队闻令而动，第一时间赶赴现场。</t>
+        </is>
+      </c>
+      <c r="I885" t="inlineStr">
+        <is>
+          <t>接到防汛通知后，救援队伍闻令而动，迅速展开排查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>CHI-20260812-005</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>添砖加瓦</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>tiān zhuān jiā wǎ</t>
+        </is>
+      </c>
+      <c r="G886" t="inlineStr">
+        <is>
+          <t>힘을 보태다, 기여하다</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>大家都希望能为绿色低碳的环保事业添砖加瓦。</t>
+        </is>
+      </c>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>每一个人都能为建设美丽的家园添砖加瓦。</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>CHI-20260812-006</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>减负</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>jiǎn fù</t>
+        </is>
+      </c>
+      <c r="G887" t="inlineStr">
+        <is>
+          <t>(부담/짐을) 줄여주다</t>
+        </is>
+      </c>
+      <c r="H887" t="inlineStr">
+        <is>
+          <t>各地出台了多项切实举措，整治形式主义，真正为基层干部减负。</t>
+        </is>
+      </c>
+      <c r="I887" t="inlineStr">
+        <is>
+          <t>学校通过优化作业设计，有效减轻了学生的学业负担。</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>CHI-20260812-007</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>打头阵</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>dǎ tóu zhèn</t>
+        </is>
+      </c>
+      <c r="G888" t="inlineStr">
+        <is>
+          <t>선봉에 서다, 앞장서다</t>
+        </is>
+      </c>
+      <c r="H888" t="inlineStr">
+        <is>
+          <t>在这场抗击台风的守护战中，党员干部主动打头阵。</t>
+        </is>
+      </c>
+      <c r="I888" t="inlineStr">
+        <is>
+          <t>面对这个高难度的课题，经理决定亲自打头阵。</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>CHI-20260812-008</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>雨后春笋</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>yǔ hòu chūn sǔn</t>
+        </is>
+      </c>
+      <c r="G889" t="inlineStr">
+        <is>
+          <t>우후죽순 (새로운 사물이 급격히 쏟아져 나옴)</t>
+        </is>
+      </c>
+      <c r="H889" t="inlineStr">
+        <is>
+          <t>随着科创环境的改善，各类创客企业如雨后春笋般涌现出来。</t>
+        </is>
+      </c>
+      <c r="I889" t="inlineStr">
+        <is>
+          <t>近几年，智能新能源汽车品牌如雨后春笋般在市场上冒了出来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>CHI-20260812-009</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>井井有条</t>
+        </is>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>jǐng jǐng yǒu tiáo</t>
+        </is>
+      </c>
+      <c r="G890" t="inlineStr">
+        <is>
+          <t>질서정연하다, 차곡차곡 수순에 맞게 정리되다</t>
+        </is>
+      </c>
+      <c r="H890" t="inlineStr">
+        <is>
+          <t>虽然人员安置任务繁重，但现场指挥得当，一切安排得井井有条。</t>
+        </is>
+      </c>
+      <c r="I890" t="inlineStr">
+        <is>
+          <t>即使面对突发的紧急状况，她也能把各项工作安排得井井有条。</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>CHI-20260812-010</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>莫衷一是</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>mò zhōng yī shì</t>
+        </is>
+      </c>
+      <c r="G891" t="inlineStr">
+        <is>
+          <t>의견이 분분하여 매듭을 짓지 못하다</t>
+        </is>
+      </c>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>关于新学科的设立方案，大家讨论了很久，依然莫衷一是。</t>
+        </is>
+      </c>
+      <c r="I891" t="inlineStr">
+        <is>
+          <t>对于这个市场策略的调整，内部高层至今仍然莫衷一是。</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>CHI-20260812-011</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>锦上添花</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>jǐn shàng tiān huā</t>
+        </is>
+      </c>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>금상첨화, 좋은 것에 더 좋은 것을 더하다</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>顶尖名师的加入，为学校本就雄厚的师资力量锦上添花。</t>
+        </is>
+      </c>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>优质的售后服务能为优秀的产品质量锦上添花。</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>CHI-20260812-012</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>防患于未然</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>fáng huàn yú wèi rán</t>
+        </is>
+      </c>
+      <c r="G893" t="inlineStr">
+        <is>
+          <t>사고나 재앙을 미연에 방지하다</t>
+        </is>
+      </c>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>校园安全巡查制度的建立，目的就是防患于未然，杜绝隐患。</t>
+        </is>
+      </c>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>定期进行设备维护保养，才能有效降低故障率，防患于未然。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-13 | 902/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I893"/>
+  <dimension ref="A1:I903"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42387,6 +42387,476 @@
         </is>
       </c>
     </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>CHI-20260813-001</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>敲竹杠</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>qiāo zhú gàng</t>
+        </is>
+      </c>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>바가지를 씌우다, 부당하게 돈을 뜯어내다</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>旅游景区的整治工作必须到位，绝不允许有商家借机敲竹杠、乱收费。</t>
+        </is>
+      </c>
+      <c r="I894" t="inlineStr">
+        <is>
+          <t>这家餐馆明码标价，绝对不会敲竹杠。</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>CHI-20260813-002</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>打心眼儿里</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>dǎ xīn yǎn r lǐ</t>
+        </is>
+      </c>
+      <c r="G895" t="inlineStr">
+        <is>
+          <t>마음속 깊이, 진심으로</t>
+        </is>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>对于那些十年来默默清理长江垃圾的志愿人员，大家都打心眼儿里感到佩服。</t>
+        </is>
+      </c>
+      <c r="I895" t="inlineStr">
+        <is>
+          <t>看到你取得这么大的进步，我打心眼儿里为你高兴。</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>CHI-20260813-003</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>软磨硬泡</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>ruǎn mó yìng pào</t>
+        </is>
+      </c>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>끈질기게 졸라대다, 구안과 압박을 병행하여 설득하다</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>在推动基层建设和征地拆迁等工作中，工作人员耐心地软磨硬泡，终于做通了居民的思想工作。</t>
+        </is>
+      </c>
+      <c r="I896" t="inlineStr">
+        <is>
+          <t>经过我两天的软磨硬泡，老板终于同意了我的休假申请。</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>CHI-20260813-004</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>泼辣</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>pō la</t>
+        </is>
+      </c>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>과감하고 화끈하다, 야무지다</t>
+        </is>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>在基层一线开展工作的基层干部，办事情往往需要有一种敢打敢拼、泼辣果断的作风。</t>
+        </is>
+      </c>
+      <c r="I897" t="inlineStr">
+        <is>
+          <t>她工作作风非常泼辣，处理起突发事件干净利落。</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>CHI-20260813-005</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>杀手锏</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>shā shǒu jiǎn</t>
+        </is>
+      </c>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>필살기, 비장의 무기</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>自主研发的绿色环保黑科技，成为了施工企业在招投标竞争中拿项目的杀手锏。</t>
+        </is>
+      </c>
+      <c r="I898" t="inlineStr">
+        <is>
+          <t>核心自主技术才是我们企业打赢这场商业战的杀手锏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>CHI-20260813-006</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>出差错</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>chū chā cuò</t>
+        </is>
+      </c>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>착오가 생기다, 실수하다</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>高考考务工作要求极其严格，绝对不允许出现任何差错。</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>财务数据非常关键，核对时务必仔细，不能出一点儿差错。</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>CHI-20260813-007</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>做文章</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>zuò wén zhāng</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>문제를 삼다, 이슈화하다, 꼬투리를 잡다</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>有媒体就军备合作事宜做文章，外交部对此做出了客观回应。</t>
+        </is>
+      </c>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>我们要利用这次展览会好好做文章，宣传我们品牌的新形象。</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>CHI-20260813-008</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>拿手好戏</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>ná shǒu hǎo xì</t>
+        </is>
+      </c>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>가장 자신 있는 장기, 주특기</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>依靠绿色的“黑科技”实现高效环保施工，是该公司的拿手好戏。</t>
+        </is>
+      </c>
+      <c r="I901" t="inlineStr">
+        <is>
+          <t>制作传统手工艺品是她的拿手好戏，每次展示都能获得称赞。</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>CHI-20260813-009</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>走投无路</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>zǒu tóu wú lù</t>
+        </is>
+      </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>막다른 골목에 몰리다, 갈 곳이 없어 막막하다</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>欧洲工业运输因河道干涸面临重大挑战，仿佛到了走投无路的境地。</t>
+        </is>
+      </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>当你觉得走投无路的时候，不妨换个角度思考问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>CHI-20260813-010</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>挑刺儿</t>
+        </is>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>tiāo cì r</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>트집을 잡다, 꼬투리를 잡다</t>
+        </is>
+      </c>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>环保志愿者并不是故意去“找麻烦”或“挑刺儿”，而是协助监管。</t>
+        </is>
+      </c>
+      <c r="I903" t="inlineStr">
+        <is>
+          <t>他总是喜欢在别人的方案里挑刺儿，却提不出建设性的意见。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-14 | 920/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I903"/>
+  <dimension ref="A1:I921"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42857,6 +42857,852 @@
         </is>
       </c>
     </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>CHI-20260814-001</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>两张皮</t>
+        </is>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>liǎng zhāng pí</t>
+        </is>
+      </c>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>이론과 실무가 따로 놀다, 겉돌다</t>
+        </is>
+      </c>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>学校教育和企业需求严重脱节，存在着产教两张皮的现象。</t>
+        </is>
+      </c>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>我们的营销策略和客户的真实需求简直是两张皮。</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>CHI-20260814-002</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>先到先得</t>
+        </is>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>xiān dào xiān dé</t>
+        </is>
+      </c>
+      <c r="G905" t="inlineStr">
+        <is>
+          <t>선착순이다</t>
+        </is>
+      </c>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>本次招生活动的礼品数量有限，先到先得。</t>
+        </is>
+      </c>
+      <c r="I905" t="inlineStr">
+        <is>
+          <t>我们要去抢限量版门票，一定要快，先到先得！</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>CHI-20260814-003</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>脱钩</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>오피스 표현</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>tuō gōu</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>단절되다, 연관성이 끊기다</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>教学体系如果与市场需求脱钩，学生毕业就很难就业。</t>
+        </is>
+      </c>
+      <c r="I906" t="inlineStr">
+        <is>
+          <t>现在的教学内容和实际工作严重脱钩了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>CHI-20260814-004</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>想方设法</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>xiǎng fāng shè fǎ</t>
+        </is>
+      </c>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>온갖 방법을 다 쓰다, 궁리하다</t>
+        </is>
+      </c>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>相关部门正在想方设法化解堤坡渗水隐患。</t>
+        </is>
+      </c>
+      <c r="I907" t="inlineStr">
+        <is>
+          <t>为了赶上进度，我们正在想方设法提高效率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>CHI-20260814-005</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>没谱</t>
+        </is>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>méi pǔ</t>
+        </is>
+      </c>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>근거가 없다, 미덥지 못하다</t>
+        </is>
+      </c>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>这个计划听起来不太靠谱，感觉有点没谱。</t>
+        </is>
+      </c>
+      <c r="I908" t="inlineStr">
+        <is>
+          <t>这件事还没落实，你别随便乱说，太没谱了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>CHI-20260814-006</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>没门儿</t>
+        </is>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>méi ménr</t>
+        </is>
+      </c>
+      <c r="G909" t="inlineStr">
+        <is>
+          <t>말도 안 돼, 절대 안 돼</t>
+        </is>
+      </c>
+      <c r="H909" t="inlineStr">
+        <is>
+          <t>想要违规操作？没门儿！</t>
+        </is>
+      </c>
+      <c r="I909" t="inlineStr">
+        <is>
+          <t>这种不合理的要求，没门儿！</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>CHI-20260814-007</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>跑腿</t>
+        </is>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>pǎo tuǐ</t>
+        </is>
+      </c>
+      <c r="G910" t="inlineStr">
+        <is>
+          <t>심부름하다, 발품 팔다</t>
+        </is>
+      </c>
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>志愿者们每天四处跑腿，为社区解决环保小事。</t>
+        </is>
+      </c>
+      <c r="I910" t="inlineStr">
+        <is>
+          <t>这件事需要去现场协调，得找个人跑跑腿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>CHI-20260814-008</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>没商量</t>
+        </is>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>méi shāng liang</t>
+        </is>
+      </c>
+      <c r="G911" t="inlineStr">
+        <is>
+          <t>흥정의 여지가 없다, 단호하다</t>
+        </is>
+      </c>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>环保法规的执行力度，没商量！</t>
+        </is>
+      </c>
+      <c r="I911" t="inlineStr">
+        <is>
+          <t>明天必须完成任务，没商量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>CHI-20260814-009</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>兜圈子</t>
+        </is>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>dōu quān zi</t>
+        </is>
+      </c>
+      <c r="G912" t="inlineStr">
+        <is>
+          <t>빙빙 돌려 말하다</t>
+        </is>
+      </c>
+      <c r="H912" t="inlineStr">
+        <is>
+          <t>别跟我兜圈子，直接说你的条件吧。</t>
+        </is>
+      </c>
+      <c r="I912" t="inlineStr">
+        <is>
+          <t>他说话总喜欢兜圈子，听得人很着急。</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>CHI-20260814-010</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>没劲</t>
+        </is>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>méi jìn</t>
+        </is>
+      </c>
+      <c r="G913" t="inlineStr">
+        <is>
+          <t>재미없다, 시시하다</t>
+        </is>
+      </c>
+      <c r="H913" t="inlineStr">
+        <is>
+          <t>如果不参与社会公益，生活总觉得缺了点什么，挺没劲的。</t>
+        </is>
+      </c>
+      <c r="I913" t="inlineStr">
+        <is>
+          <t>这部电影情节太老套，看了一会儿觉得真没劲。</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>CHI-20260814-011</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>走形式</t>
+        </is>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F914" t="inlineStr">
+        <is>
+          <t>zǒu xíng shì</t>
+        </is>
+      </c>
+      <c r="G914" t="inlineStr">
+        <is>
+          <t>형식적으로 처리하다, 요식행위에 그치다</t>
+        </is>
+      </c>
+      <c r="H914" t="inlineStr">
+        <is>
+          <t>整治形式主义为基层减负，各地这样干。</t>
+        </is>
+      </c>
+      <c r="I914" t="inlineStr">
+        <is>
+          <t>我们做工作不能只走形式，必须切实解决实际问题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>CHI-20260814-012</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>搭把手</t>
+        </is>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F915" t="inlineStr">
+        <is>
+          <t>dā bǎ shǒu</t>
+        </is>
+      </c>
+      <c r="G915" t="inlineStr">
+        <is>
+          <t>거들어 주다, 도와주다</t>
+        </is>
+      </c>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>从“找麻烦”到“好帮手”——宁乡市环保志愿者协会的...</t>
+        </is>
+      </c>
+      <c r="I915" t="inlineStr">
+        <is>
+          <t>如果你忙不过来的话，我可以帮你搭把手。</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>CHI-20260814-013</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>敲定</t>
+        </is>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F916" t="inlineStr">
+        <is>
+          <t>qiāo dìng</t>
+        </is>
+      </c>
+      <c r="G916" t="inlineStr">
+        <is>
+          <t>확정하다, 결정하다</t>
+        </is>
+      </c>
+      <c r="H916" t="inlineStr">
+        <is>
+          <t>上汽集团计划在西班牙建厂...</t>
+        </is>
+      </c>
+      <c r="I916" t="inlineStr">
+        <is>
+          <t>会议时间已经敲定了，就在下周一。</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>CHI-20260814-014</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>大手笔</t>
+        </is>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>dà shǒu bǐ</t>
+        </is>
+      </c>
+      <c r="G917" t="inlineStr">
+        <is>
+          <t>큰 규모의 투자나 처리</t>
+        </is>
+      </c>
+      <c r="H917" t="inlineStr">
+        <is>
+          <t>绿色科技在身边 揭秘公发工程公司施工环保“黑科技”。</t>
+        </is>
+      </c>
+      <c r="I917" t="inlineStr">
+        <is>
+          <t>这家公司在研发上的投入真是大手笔。</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>CHI-20260814-015</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>拦路虎</t>
+        </is>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>lán lù hǔ</t>
+        </is>
+      </c>
+      <c r="G918" t="inlineStr">
+        <is>
+          <t>가로막는 장애물</t>
+        </is>
+      </c>
+      <c r="H918" t="inlineStr">
+        <is>
+          <t>欧洲工业运输大动脉受阻...</t>
+        </is>
+      </c>
+      <c r="I918" t="inlineStr">
+        <is>
+          <t>缺乏资金是项目推进过程中的最大拦路虎。</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>CHI-20260814-016</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>摆平</t>
+        </is>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>bǎi píng</t>
+        </is>
+      </c>
+      <c r="G919" t="inlineStr">
+        <is>
+          <t>문제를 해결하다, 원만히 처리하다</t>
+        </is>
+      </c>
+      <c r="H919" t="inlineStr">
+        <is>
+          <t>成功化解资江南岸堤坡渗水隐患。</t>
+        </is>
+      </c>
+      <c r="I919" t="inlineStr">
+        <is>
+          <t>这件事比较棘手，你有把握摆平吗？</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>CHI-20260814-017</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>不折不扣</t>
+        </is>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F920" t="inlineStr">
+        <is>
+          <t>bù zhé bù kòu</t>
+        </is>
+      </c>
+      <c r="G920" t="inlineStr">
+        <is>
+          <t>철저히, 조금도 다름없이</t>
+        </is>
+      </c>
+      <c r="H920" t="inlineStr">
+        <is>
+          <t>整治形式主义为基层减负，各地这样干。</t>
+        </is>
+      </c>
+      <c r="I920" t="inlineStr">
+        <is>
+          <t>我们要不折不扣地执行上级的规定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>CHI-20260814-018</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>大同小异</t>
+        </is>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F921" t="inlineStr">
+        <is>
+          <t>dà tóng xiǎo yì</t>
+        </is>
+      </c>
+      <c r="G921" t="inlineStr">
+        <is>
+          <t>대동소이하다</t>
+        </is>
+      </c>
+      <c r="H921" t="inlineStr">
+        <is>
+          <t>多所学校建设有新进展。</t>
+        </is>
+      </c>
+      <c r="I921" t="inlineStr">
+        <is>
+          <t>这两份方案大同小异，选哪一个都行。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-17 | 939/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I921"/>
+  <dimension ref="A1:I940"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43703,6 +43703,899 @@
         </is>
       </c>
     </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>CHI-20260817-001</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>和事佬</t>
+        </is>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F922" t="inlineStr">
+        <is>
+          <t>hé shì lǎo</t>
+        </is>
+      </c>
+      <c r="G922" t="inlineStr">
+        <is>
+          <t>중재자, 좋게 좋게 타협을 보려는 사람</t>
+        </is>
+      </c>
+      <c r="H922" t="inlineStr">
+        <is>
+          <t>他们两方为了利益争执不下，最后还是外交部出来当了个和事佬。</t>
+        </is>
+      </c>
+      <c r="I922" t="inlineStr">
+        <is>
+          <t>他们俩吵架的时候，我总是充当和事佬的角色。</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>CHI-20260817-002</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>道德绑架</t>
+        </is>
+      </c>
+      <c r="E923" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F923" t="inlineStr">
+        <is>
+          <t>dào dé bǎng jià</t>
+        </is>
+      </c>
+      <c r="G923" t="inlineStr">
+        <is>
+          <t>도덕적 강요, 프레임을 씌워 억지로 희생을 강요하는 행위</t>
+        </is>
+      </c>
+      <c r="H923" t="inlineStr">
+        <is>
+          <t>高校给校友捐款额排名，这简直就是道德绑架，让没捐钱的校友很难堪。</t>
+        </is>
+      </c>
+      <c r="I923" t="inlineStr">
+        <is>
+          <t>你不能用孝顺来道德绑架我，强迫我做不喜欢的事。</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>CHI-20260817-003</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>吃不消</t>
+        </is>
+      </c>
+      <c r="E924" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F924" t="inlineStr">
+        <is>
+          <t>chī bù xiāo</t>
+        </is>
+      </c>
+      <c r="G924" t="inlineStr">
+        <is>
+          <t>감당하기 힘들다, 버겁다</t>
+        </is>
+      </c>
+      <c r="H924" t="inlineStr">
+        <is>
+          <t>学校按照学院排名催促大家捐款，很多刚毕业的校友直呼吃不消。</t>
+        </is>
+      </c>
+      <c r="I924" t="inlineStr">
+        <is>
+          <t>每天加班到半夜，我的身体真的有点吃不消了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>CHI-20260817-004</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>面子工程</t>
+        </is>
+      </c>
+      <c r="E925" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F925" t="inlineStr">
+        <is>
+          <t>miàn zi gōng chéng</t>
+        </is>
+      </c>
+      <c r="G925" t="inlineStr">
+        <is>
+          <t>생색내기용 사업, 겉치레식 공사</t>
+        </is>
+      </c>
+      <c r="H925" t="inlineStr">
+        <is>
+          <t>所谓的绿色城市更新，如果只是做面子工程，根本解决不了居民的痛点。</t>
+        </is>
+      </c>
+      <c r="I925" t="inlineStr">
+        <is>
+          <t>很多市民抱怨这些景观改造只是面子工程，根本不实用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>CHI-20260817-005</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>说走就走</t>
+        </is>
+      </c>
+      <c r="E926" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F926" t="inlineStr">
+        <is>
+          <t>shuō zǒu jiù zǒu</t>
+        </is>
+      </c>
+      <c r="G926" t="inlineStr">
+        <is>
+          <t>(사전 계획 없이) 즉흥적으로 훌쩍 떠나다</t>
+        </is>
+      </c>
+      <c r="H926" t="inlineStr">
+        <is>
+          <t>这4个人没有办任何审批手续，来了一场说走就走的探险，结果被困在保护区了。</t>
+        </is>
+      </c>
+      <c r="I926" t="inlineStr">
+        <is>
+          <t>周末我来了一场说走就走的旅行，放松一下紧绷的神经。</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>CHI-20260817-006</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>不置可否</t>
+        </is>
+      </c>
+      <c r="E927" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F927" t="inlineStr">
+        <is>
+          <t>bù zhì kě fǒu</t>
+        </is>
+      </c>
+      <c r="G927" t="inlineStr">
+        <is>
+          <t>긍정도 부정도 하지 않다, 애매한 태도를 취하다</t>
+        </is>
+      </c>
+      <c r="H927" t="inlineStr">
+        <is>
+          <t>对于是否违反了保护区的规定，这几个人面对询问时却不置可否。</t>
+        </is>
+      </c>
+      <c r="I927" t="inlineStr">
+        <is>
+          <t>对于我提出的建议，经理不置可否，只是点了点头。</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>CHI-20260817-007</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>老天爷</t>
+        </is>
+      </c>
+      <c r="E928" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F928" t="inlineStr">
+        <is>
+          <t>lǎo tiān yé</t>
+        </is>
+      </c>
+      <c r="G928" t="inlineStr">
+        <is>
+          <t>하늘, 하느님 (원망이나 한탄 시 '하늘도 무심하시지'의 하늘)</t>
+        </is>
+      </c>
+      <c r="H928" t="inlineStr">
+        <is>
+          <t>莱茵河快被烤干了，老天爷再不下雨，欧洲的工业运输可就瘫痪了。</t>
+        </is>
+      </c>
+      <c r="I928" t="inlineStr">
+        <is>
+          <t>老天爷真是不作美，偏偏在我们举行户外活动时下起了暴雨。</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>CHI-20260817-008</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>燃眉之急</t>
+        </is>
+      </c>
+      <c r="E929" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F929" t="inlineStr">
+        <is>
+          <t>rán méi zhī jí</t>
+        </is>
+      </c>
+      <c r="G929" t="inlineStr">
+        <is>
+          <t>발등에 떨어진 불, 엄청나게 시급한 일</t>
+        </is>
+      </c>
+      <c r="H929" t="inlineStr">
+        <is>
+          <t>国家发改委下达的3000万元资金，及时解决了河南灾区重建的燃眉之急。</t>
+        </is>
+      </c>
+      <c r="I929" t="inlineStr">
+        <is>
+          <t>政府发放的这笔救灾款，切实解决了灾区群众的燃眉之急。</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>CHI-20260817-009</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>分一杯羹</t>
+        </is>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F930" t="inlineStr">
+        <is>
+          <t>fēn yī bēi gēng</t>
+        </is>
+      </c>
+      <c r="G930" t="inlineStr">
+        <is>
+          <t>남의 이득이나 시장 파이에서 한몫을 챙기다</t>
+        </is>
+      </c>
+      <c r="H930" t="inlineStr">
+        <is>
+          <t>全球经贸格局重塑，各国都想在这些新兴的绿色科技产业里分一杯羹。</t>
+        </is>
+      </c>
+      <c r="I930" t="inlineStr">
+        <is>
+          <t>眼看这个新兴行业利润丰厚，很多大企业都想来分一杯羹。</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>CHI-20260817-010</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>大打折扣</t>
+        </is>
+      </c>
+      <c r="E931" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>dǎ dǎ zhé kòu</t>
+        </is>
+      </c>
+      <c r="G931" t="inlineStr">
+        <is>
+          <t>(가치, 기대치, 만족도 등이) 크게 깎이다, 뚝 떨어지다</t>
+        </is>
+      </c>
+      <c r="H931" t="inlineStr">
+        <is>
+          <t>本来牛肉干的味道不错，但因为称重玩猫腻，品牌信誉大打折扣。</t>
+        </is>
+      </c>
+      <c r="I931" t="inlineStr">
+        <is>
+          <t>如果服务态度不好，再美味的菜肴也会让顾客的体验大打折扣。</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>CHI-20260817-011</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>摸着石头过河</t>
+        </is>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>mō zhe shí tou guò hé</t>
+        </is>
+      </c>
+      <c r="G932" t="inlineStr">
+        <is>
+          <t>돌다리도 두드려 보고 건너다, 신중하게 한 걸음씩 나아가다</t>
+        </is>
+      </c>
+      <c r="H932" t="inlineStr">
+        <is>
+          <t>对于全球重塑的大变局，中国在进行区域国别研究时，也需要摸着石头过河。</t>
+        </is>
+      </c>
+      <c r="I932" t="inlineStr">
+        <is>
+          <t>作为一个全新的探索领域，我们目前也只能摸着石头过河。</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>CHI-20260817-012</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>玩猫腻</t>
+        </is>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F933" t="inlineStr">
+        <is>
+          <t>wán māo nì</t>
+        </is>
+      </c>
+      <c r="G933" t="inlineStr">
+        <is>
+          <t>꼼수를 부리다, 잔머리를 써서 남을 속이다</t>
+        </is>
+      </c>
+      <c r="H933" t="inlineStr">
+        <is>
+          <t>64元的牛肉干重新称一下居然才17元，商家这明显是在重量上玩猫腻。</t>
+        </is>
+      </c>
+      <c r="I933" t="inlineStr">
+        <is>
+          <t>这家店在商品的重量上玩猫腻，结果被愤怒的顾客举报了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>CHI-20260817-013</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>口头禅</t>
+        </is>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F934" t="inlineStr">
+        <is>
+          <t>kǒu tóu chán</t>
+        </is>
+      </c>
+      <c r="G934" t="inlineStr">
+        <is>
+          <t>입버릇, 입에 달고 사는 말</t>
+        </is>
+      </c>
+      <c r="H934" t="inlineStr">
+        <is>
+          <t>“依法合规”不该只是挂在嘴边的口头禅，要真正落实在保护区管理上。</t>
+        </is>
+      </c>
+      <c r="I934" t="inlineStr">
+        <is>
+          <t>“没问题”是他的口头禅，每次找他帮忙他都这么说。</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>CHI-20260817-014</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>破烂不堪</t>
+        </is>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F935" t="inlineStr">
+        <is>
+          <t>pò làn bù kān</t>
+        </is>
+      </c>
+      <c r="G935" t="inlineStr">
+        <is>
+          <t>너덜너덜하다, 엉망진창으로 파손되다</t>
+        </is>
+      </c>
+      <c r="H935" t="inlineStr">
+        <is>
+          <t>暴雨过后，这条山区的铁路线受损严重，路基甚至变得破烂不堪。</t>
+        </is>
+      </c>
+      <c r="I935" t="inlineStr">
+        <is>
+          <t>这条老旧的小街由于年久失修，路面已经破烂不堪。</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>CHI-20260817-015</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>一气之下</t>
+        </is>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F936" t="inlineStr">
+        <is>
+          <t>yí qì zhī xià</t>
+        </is>
+      </c>
+      <c r="G936" t="inlineStr">
+        <is>
+          <t>홧김에, 너무 화가 난 나머지</t>
+        </is>
+      </c>
+      <c r="H936" t="inlineStr">
+        <is>
+          <t>顾客发现牛肉干的分量不足，一气之下把视频发到了网上，引起了广泛争议。</t>
+        </is>
+      </c>
+      <c r="I936" t="inlineStr">
+        <is>
+          <t>他一气之下辞去了工作，现在回想起来觉得有些冲动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>CHI-20260817-016</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>心无旁骛</t>
+        </is>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F937" t="inlineStr">
+        <is>
+          <t>xīn wú páng wù</t>
+        </is>
+      </c>
+      <c r="G937" t="inlineStr">
+        <is>
+          <t>딴 데 마음을 쓰지 않고 오직 한 가지 일에만 전념하다</t>
+        </is>
+      </c>
+      <c r="H937" t="inlineStr">
+        <is>
+          <t>高考状元在分享学习经验时提到，备考期间最重要的是做到心无旁骛。</t>
+        </is>
+      </c>
+      <c r="I937" t="inlineStr">
+        <is>
+          <t>既然决定了要考研，你就应该心无旁骛地准备，别再想着去旅游了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>CHI-20260817-017</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>和稀泥</t>
+        </is>
+      </c>
+      <c r="E938" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F938" t="inlineStr">
+        <is>
+          <t>hé xī ní</t>
+        </is>
+      </c>
+      <c r="G938" t="inlineStr">
+        <is>
+          <t>시시비비를 가리지 않고 적당히 얼버무려 타협하다</t>
+        </is>
+      </c>
+      <c r="H938" t="inlineStr">
+        <is>
+          <t>面对这起复杂的旅游纠纷，相关部门不能只想着和稀泥，得彻底解决村民和游客的矛盾。</t>
+        </is>
+      </c>
+      <c r="I938" t="inlineStr">
+        <is>
+          <t>团队里出现工作冲突应该正视并妥善解决，你作为组长一直和稀泥是不行的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>CHI-20260817-018</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>雪上加霜</t>
+        </is>
+      </c>
+      <c r="E939" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F939" t="inlineStr">
+        <is>
+          <t>xuě shàng jiā shuāng</t>
+        </is>
+      </c>
+      <c r="G939" t="inlineStr">
+        <is>
+          <t>설상가상으로, 엎친 데 덮친 격으로</t>
+        </is>
+      </c>
+      <c r="H939" t="inlineStr">
+        <is>
+          <t>莱茵河快被烤干了，这给本就面临能源危机的欧洲工业运输带来了雪上加霜的打击。</t>
+        </is>
+      </c>
+      <c r="I939" t="inlineStr">
+        <is>
+          <t>公司正处于资金紧张的困难时期，这时候核心技术人员突然辞职，真是雪上加霜。</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>CHI-20260817-019</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>有条不紊</t>
+        </is>
+      </c>
+      <c r="E940" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F940" t="inlineStr">
+        <is>
+          <t>yǒu tiáo bù wěn</t>
+        </is>
+      </c>
+      <c r="G940" t="inlineStr">
+        <is>
+          <t>질서정연하다, 차근차근 막힘없이 진행되다</t>
+        </is>
+      </c>
+      <c r="H940" t="inlineStr">
+        <is>
+          <t>即使面对复杂的地质条件，横断山脉这条超长隧道的建设工作依然有条不紊地推进。</t>
+        </is>
+      </c>
+      <c r="I940" t="inlineStr">
+        <is>
+          <t>面对突发的大量网络订单，工厂的物流部门依然有条不紊地配货，保证了按时发货。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-18 | 946/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I940"/>
+  <dimension ref="A1:I947"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44596,6 +44596,335 @@
         </is>
       </c>
     </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>CHI-20260818-001</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>请年假</t>
+        </is>
+      </c>
+      <c r="E941" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F941" t="inlineStr">
+        <is>
+          <t>qǐng nián jià</t>
+        </is>
+      </c>
+      <c r="G941" t="inlineStr">
+        <is>
+          <t>연차를 내다</t>
+        </is>
+      </c>
+      <c r="H941" t="inlineStr">
+        <is>
+          <t>招聘详情：人大附中石景山学校期待你的加入！转正后员工可享受带薪年假。</t>
+        </is>
+      </c>
+      <c r="I941" t="inlineStr">
+        <is>
+          <t>由于最近工作压力太大，我决定请年假出去旅游放松一下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>CHI-20260818-002</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>开夜车</t>
+        </is>
+      </c>
+      <c r="E942" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F942" t="inlineStr">
+        <is>
+          <t>kāi yè chē</t>
+        </is>
+      </c>
+      <c r="G942" t="inlineStr">
+        <is>
+          <t>밤샘 작업을 하다, 야근하다</t>
+        </is>
+      </c>
+      <c r="H942" t="inlineStr">
+        <is>
+          <t>为了准备2027届高三‘立人论坛’研讨会的发言材料，老师们连续开了几天夜车。</t>
+        </is>
+      </c>
+      <c r="I942" t="inlineStr">
+        <is>
+          <t>明天就要向客户交付最终的设计图了，今晚看来又得开夜车了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>CHI-20260818-003</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>顺风车</t>
+        </is>
+      </c>
+      <c r="E943" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F943" t="inlineStr">
+        <is>
+          <t>shùn fēng chē</t>
+        </is>
+      </c>
+      <c r="G943" t="inlineStr">
+        <is>
+          <t>무임승차, 남의 편의나 기회에 편승하다</t>
+        </is>
+      </c>
+      <c r="H943" t="inlineStr">
+        <is>
+          <t>中国实行的零关税举措，有力地支持了非洲国家搭上工业化发展的顺风车。</t>
+        </is>
+      </c>
+      <c r="I943" t="inlineStr">
+        <is>
+          <t>借助这次行业展会的机会，我们公司也顺便搭了一次数字化转型的顺风车。</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>CHI-20260818-004</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>大锅饭</t>
+        </is>
+      </c>
+      <c r="E944" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F944" t="inlineStr">
+        <is>
+          <t>dài guō fàn</t>
+        </is>
+      </c>
+      <c r="G944" t="inlineStr">
+        <is>
+          <t>성과와 무관한 균등 분배 (평등주의)</t>
+        </is>
+      </c>
+      <c r="H944" t="inlineStr">
+        <is>
+          <t>国企管理层岗位公开招贤纳士，旨在打破传统的‘大锅饭’制度，实行绩效激励。</t>
+        </is>
+      </c>
+      <c r="I944" t="inlineStr">
+        <is>
+          <t>为了激发员工的工作积极性，企业必须彻底打破大锅饭的分配体制。</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>CHI-20260818-005</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>因材施教</t>
+        </is>
+      </c>
+      <c r="E945" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F945" t="inlineStr">
+        <is>
+          <t>yīn cái shī jiào</t>
+        </is>
+      </c>
+      <c r="G945" t="inlineStr">
+        <is>
+          <t>소질에 따라 가르치다 (개별 맞춤 교육)</t>
+        </is>
+      </c>
+      <c r="H945" t="inlineStr">
+        <is>
+          <t>衡阳市田家炳实验中学注重因材施教，在有温度的土壤里灌溉每一个梦想。</t>
+        </is>
+      </c>
+      <c r="I945" t="inlineStr">
+        <is>
+          <t>每个学生的性格和兴趣都不同，好的教育应当因材施教，发掘他们的潜能。</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>CHI-20260818-006</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>不可或缺</t>
+        </is>
+      </c>
+      <c r="E946" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F946" t="inlineStr">
+        <is>
+          <t>bù kě huò quē</t>
+        </is>
+      </c>
+      <c r="G946" t="inlineStr">
+        <is>
+          <t>결코 없어서는 안 될, 필수적인</t>
+        </is>
+      </c>
+      <c r="H946" t="inlineStr">
+        <is>
+          <t>在法治护航下的生态蝶变过程中，健全的法律体系是环境保护不可或缺的基石。</t>
+        </is>
+      </c>
+      <c r="I946" t="inlineStr">
+        <is>
+          <t>现在，智能手机已经成为我们日常生活中不可或缺的工具了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>CHI-20260818-007</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>有的放矢</t>
+        </is>
+      </c>
+      <c r="E947" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F947" t="inlineStr">
+        <is>
+          <t>yǒu dì fàng shǐ</t>
+        </is>
+      </c>
+      <c r="G947" t="inlineStr">
+        <is>
+          <t>과녁을 보고 활을 쏘다, 목적이 명확하다 (대책이 확실하다)</t>
+        </is>
+      </c>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>面对莱茵河干涸对欧洲运输的冲击，相关企业需要有的放矢地调整供应链物流。</t>
+        </is>
+      </c>
+      <c r="I947" t="inlineStr">
+        <is>
+          <t>我们在制定营销计划时必须有的放矢，准确锁定核心客户的需求。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-19 | 960/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I947"/>
+  <dimension ref="A1:I961"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44925,6 +44925,664 @@
         </is>
       </c>
     </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>CHI-20260819-001</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>选边站队</t>
+        </is>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>xuǎn biān zhàn duì</t>
+        </is>
+      </c>
+      <c r="G948" t="inlineStr">
+        <is>
+          <t>한쪽 편을 들다, 눈치를 보며 줄을 서다</t>
+        </is>
+      </c>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>针对美方要求在人工智能领域限制与中方合作，中方发言人明确表示，反对在科技领域搞选边站队。</t>
+        </is>
+      </c>
+      <c r="I948" t="inlineStr">
+        <is>
+          <t>在这个商业竞争中，我们必须保持中立，千万不要盲目选边站队。</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>CHI-20260819-002</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>找茬</t>
+        </is>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>zhǎo chá</t>
+        </is>
+      </c>
+      <c r="G949" t="inlineStr">
+        <is>
+          <t>트집을 잡다, 시비를 걸다</t>
+        </is>
+      </c>
+      <c r="H949" t="inlineStr">
+        <is>
+          <t>帕劳方针对中方的火箭试验发表毫无根据的指责，中方指出这完全是恶意找茬。</t>
+        </is>
+      </c>
+      <c r="I949" t="inlineStr">
+        <is>
+          <t>我们的方案已经修改过好几遍了，他还是能挑出毛病，我觉得他纯粹是在找茬。</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>CHI-20260819-003</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>洗牌</t>
+        </is>
+      </c>
+      <c r="E950" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>xǐ pái</t>
+        </is>
+      </c>
+      <c r="G950" t="inlineStr">
+        <is>
+          <t>(판도가) 재조정되다, 대대적인 재편이 이루어지다</t>
+        </is>
+      </c>
+      <c r="H950" t="inlineStr">
+        <is>
+          <t>随着全球科技的快速更迭，世界经贸格局正在经历一轮加速大洗牌。</t>
+        </is>
+      </c>
+      <c r="I950" t="inlineStr">
+        <is>
+          <t>新能源汽车产业的异军突起，让整个传统汽车市场迎来了彻底的洗牌。</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>CHI-20260819-004</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>栽跟头</t>
+        </is>
+      </c>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>zāi gēn tou</t>
+        </is>
+      </c>
+      <c r="G951" t="inlineStr">
+        <is>
+          <t>큰코다치다, 호된 교훈을 얻다, 좌절하다</t>
+        </is>
+      </c>
+      <c r="H951" t="inlineStr">
+        <is>
+          <t>那些利用手中特权肆意谋取私利的官员，最终都会在反腐的铁拳下栽跟头。</t>
+        </is>
+      </c>
+      <c r="I951" t="inlineStr">
+        <is>
+          <t>做生意不能只图暴利，如果不讲诚信，迟早会在这上面栽跟头的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>CHI-20260819-005</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>脱胎换骨</t>
+        </is>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>tuō tāi huàn gǔ</t>
+        </is>
+      </c>
+      <c r="G952" t="inlineStr">
+        <is>
+          <t>환골탈태하다, 180도 완전히 새로워지다</t>
+        </is>
+      </c>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>长江苏州段以水为脉进行综合生态治理，让曾经污染严重的化工产区实现了脱胎换骨的蝶变。</t>
+        </is>
+      </c>
+      <c r="I952" t="inlineStr">
+        <is>
+          <t>经过一年的艰苦训练，他的精神面貌和体能都发生了脱胎换骨的变化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>CHI-20260819-006</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>捕风捉影</t>
+        </is>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>bǔ fēng zhuō yǐng</t>
+        </is>
+      </c>
+      <c r="G953" t="inlineStr">
+        <is>
+          <t>근거 없는 소문을 만들다, 뜬구름 잡는 소리를 하다</t>
+        </is>
+      </c>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>对于某些西方政客针对中方在人工智能安全问题上的指责，外交部坚决予以驳斥，认为纯属捕风捉影。</t>
+        </is>
+      </c>
+      <c r="I953" t="inlineStr">
+        <is>
+          <t>媒体在报道新闻时应当基于事实，而不是捕风捉影，制造不必要的社会恐慌。</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>CHI-20260819-007</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>大势所趋</t>
+        </is>
+      </c>
+      <c r="E954" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F954" t="inlineStr">
+        <is>
+          <t>dà shì suǒ qū</t>
+        </is>
+      </c>
+      <c r="G954" t="inlineStr">
+        <is>
+          <t>거스를 수 없는 시대적 대세이다</t>
+        </is>
+      </c>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>环保型超大型集装箱船的顺利交付，充分证明了全球航运业绿色低碳转型是大势所趋。</t>
+        </is>
+      </c>
+      <c r="I954" t="inlineStr">
+        <is>
+          <t>传统企业进行数字化转型是时代的大势所趋，任何企业都无法置身事外。</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>CHI-20260819-008</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>无从下手</t>
+        </is>
+      </c>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>wú cóng xià shǒu</t>
+        </is>
+      </c>
+      <c r="G955" t="inlineStr">
+        <is>
+          <t>어찌할 바를 모르다, 어디서부터 손을 대야 할지 모르다</t>
+        </is>
+      </c>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>国企党建工作无从下手？这份“党建十法”操作指南请收下。</t>
+        </is>
+      </c>
+      <c r="I955" t="inlineStr">
+        <is>
+          <t>面对这么庞大的历史遗留数据，技术团队也感到无从下手。</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>CHI-20260819-009</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>蓄势待发</t>
+        </is>
+      </c>
+      <c r="E956" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>xù shì dài fā</t>
+        </is>
+      </c>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>힘을 축적하며 때를 기다리다, 만반의 준비를 갖추다</t>
+        </is>
+      </c>
+      <c r="H956" t="inlineStr">
+        <is>
+          <t>稼轩未来学校蓄势待发，打造K12高品质教育新范式。</t>
+        </is>
+      </c>
+      <c r="I956" t="inlineStr">
+        <is>
+          <t>经过两年的技术研发，我们的新产品已经蓄势待发，准备推向全球市场。</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>CHI-20260819-010</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>另辟蹊径</t>
+        </is>
+      </c>
+      <c r="E957" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>lìng pì xī jìng</t>
+        </is>
+      </c>
+      <c r="G957" t="inlineStr">
+        <is>
+          <t>독자적인 새로운 길을 개척하다, 새로운 방법을 모색하다</t>
+        </is>
+      </c>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>面对日益激烈的传统经贸竞争，中国企业必须另辟蹊径，加速技术重塑。</t>
+        </is>
+      </c>
+      <c r="I957" t="inlineStr">
+        <is>
+          <t>如果传统营销方式效果不佳，我们不妨另辟蹊径，尝试一下短视频引流。</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>CHI-20260819-011</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>开门红</t>
+        </is>
+      </c>
+      <c r="E958" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>kāi mén hóng</t>
+        </is>
+      </c>
+      <c r="G958" t="inlineStr">
+        <is>
+          <t>첫출발이 좋다, 순조로운 첫 출발, 첫 성과</t>
+        </is>
+      </c>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>新学校即将开门迎新，期待迎来新学期教学质量的开门红。</t>
+        </is>
+      </c>
+      <c r="I958" t="inlineStr">
+        <is>
+          <t>销售部门在元旦假期实现了业绩的开门红，给全年开了个好头。</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>CHI-20260819-012</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>说大话</t>
+        </is>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>shuō dà huà</t>
+        </is>
+      </c>
+      <c r="G959" t="inlineStr">
+        <is>
+          <t>큰소리치다, 허풍을 떨다</t>
+        </is>
+      </c>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>外交部敦促有关国家多做实事，而不是在国际舞台上说大话、开空头支票。</t>
+        </is>
+      </c>
+      <c r="I959" t="inlineStr">
+        <is>
+          <t>他总是喜欢说大话，但真正遇到棘手问题时却总是躲得远远的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>CHI-20260819-013</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>看眼色</t>
+        </is>
+      </c>
+      <c r="E960" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F960" t="inlineStr">
+        <is>
+          <t>kàn yǎn sè</t>
+        </is>
+      </c>
+      <c r="G960" t="inlineStr">
+        <is>
+          <t>눈치를 살피다, 안색을 살피다</t>
+        </is>
+      </c>
+      <c r="H960" t="inlineStr">
+        <is>
+          <t>主权国家不应该看别国的眼色行事，而应坚持独立自主的外交政策。</t>
+        </is>
+      </c>
+      <c r="I960" t="inlineStr">
+        <is>
+          <t>自从公司换了新主管，大家每天上班都得看着他的眼色过日子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>CHI-20260819-014</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>阳奉阴违</t>
+        </is>
+      </c>
+      <c r="E961" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F961" t="inlineStr">
+        <is>
+          <t>yáng fèng yīn wéi</t>
+        </is>
+      </c>
+      <c r="G961" t="inlineStr">
+        <is>
+          <t>겉으로는 복종하는 척하면서 속으로는 배반하다</t>
+        </is>
+      </c>
+      <c r="H961" t="inlineStr">
+        <is>
+          <t>部分企业在环保政策上阳奉阴违，结果收到了几十万元的环保罚单。</t>
+        </is>
+      </c>
+      <c r="I961" t="inlineStr">
+        <is>
+          <t>在团队合作中，最忌讳的就是表面上答应得好好的，背后却阳奉阴违。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-20 | 976/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I961"/>
+  <dimension ref="A1:I977"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45583,6 +45583,758 @@
         </is>
       </c>
     </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>CHI-20260820-001</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>余额不足</t>
+        </is>
+      </c>
+      <c r="E962" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F962" t="inlineStr">
+        <is>
+          <t>yú'é bùzú</t>
+        </is>
+      </c>
+      <c r="G962" t="inlineStr">
+        <is>
+          <t>(시간, 체력, 자금 등이) 얼마 남지 않음, 고갈 직전임</t>
+        </is>
+      </c>
+      <c r="H962" t="inlineStr">
+        <is>
+          <t>听到学校公布了新的开学时间，孩子们纷纷哀叹自己的暑假余额已不足。</t>
+        </is>
+      </c>
+      <c r="I962" t="inlineStr">
+        <is>
+          <t>连续加班三天，我的精力余额已不足，今天必须早点睡。</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>CHI-20260820-002</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>黑科技</t>
+        </is>
+      </c>
+      <c r="E963" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F963" t="inlineStr">
+        <is>
+          <t>hēi kē jì</t>
+        </is>
+      </c>
+      <c r="G963" t="inlineStr">
+        <is>
+          <t>혁신적이고 신기한 첨단 기술 (마치 마법 같은 기술)</t>
+        </is>
+      </c>
+      <c r="H963" t="inlineStr">
+        <is>
+          <t>这款“会飞的救生圈”获得了外交部的点赞，真是让人大开眼界的黑科技。</t>
+        </is>
+      </c>
+      <c r="I963" t="inlineStr">
+        <is>
+          <t>这家公司新研发的黑科技产品，能通过眼神控制所有家电。</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>CHI-20260820-003</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>撸串</t>
+        </is>
+      </c>
+      <c r="E964" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F964" t="inlineStr">
+        <is>
+          <t>lū chuàn</t>
+        </is>
+      </c>
+      <c r="G964" t="inlineStr">
+        <is>
+          <t>꼬치구이(양꼬치 등)를 먹다, 소탈하게 술자리를 가지다</t>
+        </is>
+      </c>
+      <c r="H964" t="inlineStr">
+        <is>
+          <t>白天进行严格的军训，晚上在操场上开心地撸串，这所学校的生活太让人向往了。</t>
+        </is>
+      </c>
+      <c r="I964" t="inlineStr">
+        <is>
+          <t>今晚下班后别走，一起去路边摊撸串，我请客！</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>CHI-20260820-004</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>主心骨</t>
+        </is>
+      </c>
+      <c r="E965" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F965" t="inlineStr">
+        <is>
+          <t>zhǔ xīn gǔ</t>
+        </is>
+      </c>
+      <c r="G965" t="inlineStr">
+        <is>
+          <t>기둥, 중심이 되는 사람, 든든한 버팀목</t>
+        </is>
+      </c>
+      <c r="H965" t="inlineStr">
+        <is>
+          <t>在幸福苑社区的志愿服务中，优秀的党员骨干成了全体居民的主心骨。</t>
+        </is>
+      </c>
+      <c r="I965" t="inlineStr">
+        <is>
+          <t>老张是我们团队的主心骨，只要有他在，大家心里就踏实。</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>CHI-20260820-005</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>眼红</t>
+        </is>
+      </c>
+      <c r="E966" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F966" t="inlineStr">
+        <is>
+          <t>yǎn hóng</t>
+        </is>
+      </c>
+      <c r="G966" t="inlineStr">
+        <is>
+          <t>부러워하다, 시샘하다, 샘이 나다</t>
+        </is>
+      </c>
+      <c r="H966" t="inlineStr">
+        <is>
+          <t>看到别人家的学校晚上能撸串，其他学校的学生都羡慕得眼红了。</t>
+        </is>
+      </c>
+      <c r="I966" t="inlineStr">
+        <is>
+          <t>看到他年纪轻轻就买房买车，周围不少人心里都酸溜溜地眼红。</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>CHI-20260820-006</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>莫须有</t>
+        </is>
+      </c>
+      <c r="E967" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F967" t="inlineStr">
+        <is>
+          <t>mò xū yǒu</t>
+        </is>
+      </c>
+      <c r="G967" t="inlineStr">
+        <is>
+          <t>터무니없는, 막연히 지어낸, 근거가 없는</t>
+        </is>
+      </c>
+      <c r="H967" t="inlineStr">
+        <is>
+          <t>外交部发言人严厉驳斥了美方以莫须有的罪名对别国企业进行无理制裁的行为。</t>
+        </is>
+      </c>
+      <c r="I967" t="inlineStr">
+        <is>
+          <t>上司用莫须有的理由把我开除了，我一定要去申请劳动仲裁。</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>CHI-20260820-007</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>大洗牌</t>
+        </is>
+      </c>
+      <c r="E968" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F968" t="inlineStr">
+        <is>
+          <t>dà xǐ pái</t>
+        </is>
+      </c>
+      <c r="G968" t="inlineStr">
+        <is>
+          <t>대대적인 재편성, 판도 변화, 대규모 물갈이</t>
+        </is>
+      </c>
+      <c r="H968" t="inlineStr">
+        <is>
+          <t>随着环保科技的快速崛起，传统的重工业运输行业正迎来一轮大洗牌。</t>
+        </is>
+      </c>
+      <c r="I968" t="inlineStr">
+        <is>
+          <t>行业不景气导致许多竞争力差的公司倒闭，整个市场正在进行大洗牌。</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>CHI-20260820-008</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>吃红利</t>
+        </is>
+      </c>
+      <c r="E969" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F969" t="inlineStr">
+        <is>
+          <t>chī hóng lì</t>
+        </is>
+      </c>
+      <c r="G969" t="inlineStr">
+        <is>
+          <t>(특정 트렌드나 정책의) 혜택을 누리다, 단물을 빨다</t>
+        </is>
+      </c>
+      <c r="H969" t="inlineStr">
+        <is>
+          <t>中国向各国开放市场，世界各地的企业都希望能来到这里吃一波发展红利。</t>
+        </is>
+      </c>
+      <c r="I969" t="inlineStr">
+        <is>
+          <t>早期进入短视频领域的创业者们，几乎都吃到了流量的第一波红利。</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>CHI-20260820-009</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>香饽饽</t>
+        </is>
+      </c>
+      <c r="E970" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F970" t="inlineStr">
+        <is>
+          <t>xiāng bō bo</t>
+        </is>
+      </c>
+      <c r="G970" t="inlineStr">
+        <is>
+          <t>인기 있는 것, 아주 잘 나가는 사람이나 물건</t>
+        </is>
+      </c>
+      <c r="H970" t="inlineStr">
+        <is>
+          <t>格力技工学校报名系统刚开放就超3000人，现在技术人才成了香饽饽。</t>
+        </is>
+      </c>
+      <c r="I970" t="inlineStr">
+        <is>
+          <t>如今精通大数据和AI算法的研发人员，在就业市场上可是个香饽饽。</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>CHI-20260820-010</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>挤破头</t>
+        </is>
+      </c>
+      <c r="E971" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F971" t="inlineStr">
+        <is>
+          <t>jǐ pò tóu</t>
+        </is>
+      </c>
+      <c r="G971" t="inlineStr">
+        <is>
+          <t>기를 쓰고 몰려들다, 치열하게 경쟁하다</t>
+        </is>
+      </c>
+      <c r="H971" t="inlineStr">
+        <is>
+          <t>格力技工学校1天多时间报名超3000人，大家都挤破头想要进去学习一技之长。</t>
+        </is>
+      </c>
+      <c r="I971" t="inlineStr">
+        <is>
+          <t>这个国企岗位福利待遇极好，每年都有成千上万的毕业生挤破头去报考。</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>CHI-20260820-011</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>雪中送炭</t>
+        </is>
+      </c>
+      <c r="E972" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F972" t="inlineStr">
+        <is>
+          <t>xuě zhōng sòng tàn</t>
+        </is>
+      </c>
+      <c r="G972" t="inlineStr">
+        <is>
+          <t>눈 속에 있는 사람에게 숯을 보내다, 다른 사람이 가장 급할 때 실질적인 도움을 주다</t>
+        </is>
+      </c>
+      <c r="H972" t="inlineStr">
+        <is>
+          <t>民政部和财政部积极发展服务类社会救助，对困难群众来说真是雪中送炭。</t>
+        </is>
+      </c>
+      <c r="I972" t="inlineStr">
+        <is>
+          <t>在我创业资金周转最困难的时候，他的投资对我们来说无异于雪中送炭。</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>CHI-20260820-012</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>搭一把</t>
+        </is>
+      </c>
+      <c r="E973" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F973" t="inlineStr">
+        <is>
+          <t>dā yì bǎ</t>
+        </is>
+      </c>
+      <c r="G973" t="inlineStr">
+        <is>
+          <t>손을 보태다, 잠깐 돕다</t>
+        </is>
+      </c>
+      <c r="H973" t="inlineStr">
+        <is>
+          <t>发展服务类社会救助需要大家都来搭一把，共同帮扶社会弱势群体。</t>
+        </is>
+      </c>
+      <c r="I973" t="inlineStr">
+        <is>
+          <t>看你搬这么多资料挺吃力的，我来帮你搭一把手吧。</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>CHI-20260820-013</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>潜移默化</t>
+        </is>
+      </c>
+      <c r="E974" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F974" t="inlineStr">
+        <is>
+          <t>qián yí mò huà</t>
+        </is>
+      </c>
+      <c r="G974" t="inlineStr">
+        <is>
+          <t>보이지 않는 사이에 조금씩 동화되다, 자연스럽게 감화되다</t>
+        </is>
+      </c>
+      <c r="H974" t="inlineStr">
+        <is>
+          <t>重庆荣昌通过环保科普点亮“绿色之梦”，在潜移默化中提升市民环保意识。</t>
+        </is>
+      </c>
+      <c r="I974" t="inlineStr">
+        <is>
+          <t>父母的一言一行都会对孩子产生潜移默化的影响，因此必须注意言传身教。</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>CHI-20260820-014</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>打预防针</t>
+        </is>
+      </c>
+      <c r="E975" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F975" t="inlineStr">
+        <is>
+          <t>dǎ yù fáng zhēn</t>
+        </is>
+      </c>
+      <c r="G975" t="inlineStr">
+        <is>
+          <t>예방 주사를 놓다, (불미스러운 일에 대비해) 미리 경고하거나 마음의 준비를 시키다</t>
+        </is>
+      </c>
+      <c r="H975" t="inlineStr">
+        <is>
+          <t>外交部提醒中国公民谨慎赴帕劳旅游，提前给游客打预防针以确保安全。</t>
+        </is>
+      </c>
+      <c r="I975" t="inlineStr">
+        <is>
+          <t>经理提前给我们打了预防针，说这次的项目难度极大，大家要有心理准备。</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>CHI-20260820-015</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>不作评论</t>
+        </is>
+      </c>
+      <c r="E976" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F976" t="inlineStr">
+        <is>
+          <t>bù zuò píng lùn</t>
+        </is>
+      </c>
+      <c r="G976" t="inlineStr">
+        <is>
+          <t>논평하지 않다, 노코멘트하다</t>
+        </is>
+      </c>
+      <c r="H976" t="inlineStr">
+        <is>
+          <t>针对朝美领导人接触的传闻，外交部发言人表示对此不作评论。</t>
+        </is>
+      </c>
+      <c r="I976" t="inlineStr">
+        <is>
+          <t>对于网络上的不实传闻，我们公司将保持沉默，不作评论。</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>CHI-20260820-016</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>无济于事</t>
+        </is>
+      </c>
+      <c r="E977" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F977" t="inlineStr">
+        <is>
+          <t>wú jì yú shì</t>
+        </is>
+      </c>
+      <c r="G977" t="inlineStr">
+        <is>
+          <t>아무런 도움이 되지 않다, 소용없다</t>
+        </is>
+      </c>
+      <c r="H977" t="inlineStr">
+        <is>
+          <t>外交部指出，一味地采取制裁施压对解决国际争端来说是无济于事的。</t>
+        </is>
+      </c>
+      <c r="I977" t="inlineStr">
+        <is>
+          <t>事情已经发生了，你现在光感到后悔也无济于事，应该想想怎么补救。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-21 | 984/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I977"/>
+  <dimension ref="A1:I985"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46335,6 +46335,382 @@
         </is>
       </c>
     </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>CHI-20260821-001</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>打call</t>
+        </is>
+      </c>
+      <c r="E978" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F978" t="inlineStr">
+        <is>
+          <t>dǎ kōu</t>
+        </is>
+      </c>
+      <c r="G978" t="inlineStr">
+        <is>
+          <t>열렬히 응원하다, 지지하다</t>
+        </is>
+      </c>
+      <c r="H978" t="inlineStr">
+        <is>
+          <t>看到我们学校的环保志愿团队在社区做宣传，大家都忍不住为他们打call。</t>
+        </is>
+      </c>
+      <c r="I978" t="inlineStr">
+        <is>
+          <t>这家新开的餐厅味道太赞了，我要在朋友圈给它强烈打call！</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>CHI-20260821-002</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>雷声大雨点小</t>
+        </is>
+      </c>
+      <c r="E979" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F979" t="inlineStr">
+        <is>
+          <t>léi shēng dà yǔ diǎn xiǎo</t>
+        </is>
+      </c>
+      <c r="G979" t="inlineStr">
+        <is>
+          <t>말만 번지르르하고 실속이 없다, 소문난 잔치에 먹을 것이 없다</t>
+        </is>
+      </c>
+      <c r="H979" t="inlineStr">
+        <is>
+          <t>很多环保板材品牌广告打得响亮，检测起来却达不到标准，真是雷声大雨点小。</t>
+        </is>
+      </c>
+      <c r="I979" t="inlineStr">
+        <is>
+          <t>他们公司说要进军海外市场，结果大半年过去了，雷声大雨点小。</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>CHI-20260821-003</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>半桶水</t>
+        </is>
+      </c>
+      <c r="E980" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F980" t="inlineStr">
+        <is>
+          <t>bàn tǒng shuǐ</t>
+        </is>
+      </c>
+      <c r="G980" t="inlineStr">
+        <is>
+          <t>수박 겉핥기식 지식을 가진 사람, 어설픈 실력자</t>
+        </is>
+      </c>
+      <c r="H980" t="inlineStr">
+        <is>
+          <t>环保科普不能只靠“半桶水”的人去宣传，必须要邀请专业科研人员来讲。</t>
+        </is>
+      </c>
+      <c r="I980" t="inlineStr">
+        <is>
+          <t>他学了几天法语就觉得自己是专家，其实只是半桶水。</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>CHI-20260821-004</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>吃苦头</t>
+        </is>
+      </c>
+      <c r="E981" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F981" t="inlineStr">
+        <is>
+          <t>chī kǔ tou</t>
+        </is>
+      </c>
+      <c r="G981" t="inlineStr">
+        <is>
+          <t>고생을 톡톡히 하다, 호되게 당하다, 쓴맛을 보다</t>
+        </is>
+      </c>
+      <c r="H981" t="inlineStr">
+        <is>
+          <t>新生在炎热的夏天进行高强度的军训，虽然吃了不少苦头，但意志得到了磨砺。</t>
+        </is>
+      </c>
+      <c r="I981" t="inlineStr">
+        <is>
+          <t>要是不听医生的劝告继续疯狂熬夜，你的身体早晚要吃苦头。</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>CHI-20260821-005</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>生根发芽</t>
+        </is>
+      </c>
+      <c r="E982" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F982" t="inlineStr">
+        <is>
+          <t>shēng gēn fā yá</t>
+        </is>
+      </c>
+      <c r="G982" t="inlineStr">
+        <is>
+          <t>뿌리를 내리고 싹을 틔우다 (생각이나 이념이 정착하다)</t>
+        </is>
+      </c>
+      <c r="H982" t="inlineStr">
+        <is>
+          <t>环保魔法闯关营，绿色理念生根发芽。</t>
+        </is>
+      </c>
+      <c r="I982" t="inlineStr">
+        <is>
+          <t>经过一年的宣传，垃圾分类的意识已经在居民心中生根发芽。</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>CHI-20260821-006</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>说干就干</t>
+        </is>
+      </c>
+      <c r="E983" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F983" t="inlineStr">
+        <is>
+          <t>shuō gàn jiù gàn</t>
+        </is>
+      </c>
+      <c r="G983" t="inlineStr">
+        <is>
+          <t>말이 떨어지자마자 실행하다, 즉각 행동에 옮기다</t>
+        </is>
+      </c>
+      <c r="H983" t="inlineStr">
+        <is>
+          <t>说干就干！环保志愿者们立刻走上街头，开始清理社区垃圾。</t>
+        </is>
+      </c>
+      <c r="I983" t="inlineStr">
+        <is>
+          <t>他是个雷厉风行的人，说干就干，下午就去注册了新公司。</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>CHI-20260821-007</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>不遗余力</t>
+        </is>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F984" t="inlineStr">
+        <is>
+          <t>bù yí yú lì</t>
+        </is>
+      </c>
+      <c r="G984" t="inlineStr">
+        <is>
+          <t>힘을 아끼지 않고 온 힘을 다하다</t>
+        </is>
+      </c>
+      <c r="H984" t="inlineStr">
+        <is>
+          <t>相关部门不遗余力地推动民政与社会救助制度的改革。</t>
+        </is>
+      </c>
+      <c r="I984" t="inlineStr">
+        <is>
+          <t>为了支持孩子圆梦大学，父母总是不遗余力地默默付出。</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>CHI-20260821-008</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>咬牙坚持</t>
+        </is>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F985" t="inlineStr">
+        <is>
+          <t>yǎo yá jiān chí</t>
+        </is>
+      </c>
+      <c r="G985" t="inlineStr">
+        <is>
+          <t>이를 악물고 버티다, 끝까지 견뎌내다</t>
+        </is>
+      </c>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>尽管高考前突发气胸需要带管赴考，他依然咬牙坚持并圆梦清华。</t>
+        </is>
+      </c>
+      <c r="I985" t="inlineStr">
+        <is>
+          <t>最后两公里是最艰难的阶段，但只要咬牙坚持，就能到达终点。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-24 | 991/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I985"/>
+  <dimension ref="A1:I992"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46711,6 +46711,335 @@
         </is>
       </c>
     </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>CHI-20260824-001</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>说空话</t>
+        </is>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F986" t="inlineStr">
+        <is>
+          <t>shuō kōng huà</t>
+        </is>
+      </c>
+      <c r="G986" t="inlineStr">
+        <is>
+          <t>실천 없이 말만 앞서다, 빈말하다</t>
+        </is>
+      </c>
+      <c r="H986" t="inlineStr">
+        <is>
+          <t>学校口口声声说把学生放在心上，这就得拿出实际行动来，不能光说空话。</t>
+        </is>
+      </c>
+      <c r="I986" t="inlineStr">
+        <is>
+          <t>领导最讨厌只会说空话而拿不出实际行动的员工。</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>CHI-20260824-002</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>放在心上</t>
+        </is>
+      </c>
+      <c r="E987" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F987" t="inlineStr">
+        <is>
+          <t>fàng zài xīn shang</t>
+        </is>
+      </c>
+      <c r="G987" t="inlineStr">
+        <is>
+          <t>마음에 두다, 신경을 쓰다, 소중히 여기다</t>
+        </is>
+      </c>
+      <c r="H987" t="inlineStr">
+        <is>
+          <t>把学生“放心上”？这所高校，是认真的。</t>
+        </is>
+      </c>
+      <c r="I987" t="inlineStr">
+        <is>
+          <t>别把他的批评太放在心上，他只是对事不对人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>CHI-20260824-003</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>勤工俭学</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>qín gōng jiǎn xué</t>
+        </is>
+      </c>
+      <c r="G988" t="inlineStr">
+        <is>
+          <t>고학하다, 아르바이트를 하며 공부하다</t>
+        </is>
+      </c>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>“追梦女孩”曾紫轩提前半个月到学校勤工助学。</t>
+        </is>
+      </c>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>许多大学生通过勤工俭学来减轻家庭的经济负担。</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>CHI-20260824-004</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>眼界大开</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>yǎn jiè dà kāi</t>
+        </is>
+      </c>
+      <c r="G989" t="inlineStr">
+        <is>
+          <t>시야가 넓어지다, 크게 눈을 뜨다</t>
+        </is>
+      </c>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>这次“人工智能与人类发展”论坛展示的技术，真是让人眼界大开。</t>
+        </is>
+      </c>
+      <c r="I989" t="inlineStr">
+        <is>
+          <t>去国外留学一年的经历，让我眼界大开，想法也改变了很多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>CHI-20260824-005</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>干劲十足</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>gàn jìn shí zú</t>
+        </is>
+      </c>
+      <c r="G990" t="inlineStr">
+        <is>
+          <t>의욕이 넘치다, 열정이 가득하다</t>
+        </is>
+      </c>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>青年科创团队成员们干劲十足，加班加点也毫无怨言。</t>
+        </is>
+      </c>
+      <c r="I990" t="inlineStr">
+        <is>
+          <t>听到项目获得投资的消息，全体员工立刻干劲十足起来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>CHI-20260824-006</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>想得周到</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>xiǎng de zhōu dào</t>
+        </is>
+      </c>
+      <c r="G991" t="inlineStr">
+        <is>
+          <t>생각이 깊다, 사려 깊다, 빈틈이 없다</t>
+        </is>
+      </c>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>学校正建设一个专门放宠物的区域，这考虑得确实想得周到。</t>
+        </is>
+      </c>
+      <c r="I991" t="inlineStr">
+        <is>
+          <t>您连备用的雨伞都帮我准备了，真是想得太周到了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>CHI-20260824-007</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>有目共睹</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>yǒu mù gòng dǔ</t>
+        </is>
+      </c>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>모든 이의 눈에 분명히 보이다, 누구나 다 알고 인정하다</t>
+        </is>
+      </c>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>中印尼两国在南方国家合作中取得的成效，是有目共睹的。</t>
+        </is>
+      </c>
+      <c r="I992" t="inlineStr">
+        <is>
+          <t>他在公司这几年的辛苦付出和成就是大家有目共睹的。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-25 | 1006/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I992"/>
+  <dimension ref="A1:I1007"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47040,6 +47040,711 @@
         </is>
       </c>
     </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>CHI-20260825-001</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>失之交臂</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>shī zhī jiāo bì</t>
+        </is>
+      </c>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>아깝게 기회를 놓치다, 눈앞에서 놓치다</t>
+        </is>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>因为几分之差，他与理想的大学失之交臂，最后决定复读一年。</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>这次由于准备不充足，我们和那个大项目失之交臂了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>CHI-20260825-002</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>铲屎官</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>chǎn shǐ guān</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>반려동물 주인 (집사)</t>
+        </is>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>高校允许带宠物上学，这让许多年轻的铲屎官兴奋不已。</t>
+        </is>
+      </c>
+      <c r="I994" t="inlineStr">
+        <is>
+          <t>作为一名合格的铲屎官，每天下班后的第一件事就是给猫咪喂食。</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>CHI-20260825-003</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>客套话</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>명사</t>
+        </is>
+      </c>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>kè tào huà</t>
+        </is>
+      </c>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>의례적인 인사말, 격식 차리는 말</t>
+        </is>
+      </c>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>两国代表一见面，先说了几句客套话，随后便切入了正题。</t>
+        </is>
+      </c>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>大家都是自己人，那些客套话就免了吧，直接谈正事。</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>CHI-20260825-004</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>吃小灶</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>chī xiǎo zào</t>
+        </is>
+      </c>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>특별 대우를 받다, 특별 과외를 받다</t>
+        </is>
+      </c>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>作为重点培养的尖子生，老师每天放学后都会给他吃小灶。</t>
+        </is>
+      </c>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>为了快速提高口语水平，他给自己请了一位外教单独吃小灶。</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>CHI-20260825-005</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>高大上</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>gāo dà shàng</t>
+        </is>
+      </c>
+      <c r="G997" t="inlineStr">
+        <is>
+          <t>품격 있고 고급스럽다 (럭셔리하다)</t>
+        </is>
+      </c>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>新开办的AI体验教室装备了最新一代的交互大屏，看起来特别高大上。</t>
+        </is>
+      </c>
+      <c r="I997" t="inlineStr">
+        <is>
+          <t>这家公司的办公环境设计得非常高大上，让人羡慕。</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>CHI-20260825-006</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>张罗</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>zhāng luo</t>
+        </is>
+      </c>
+      <c r="G998" t="inlineStr">
+        <is>
+          <t>분주히 준비하다, 사람을 모으다, 챙기다</t>
+        </is>
+      </c>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>眼看下周就要开学了，父母正忙着帮孩子张罗书包和各种文具用品。</t>
+        </is>
+      </c>
+      <c r="I998" t="inlineStr">
+        <is>
+          <t>为了庆祝他的生日，朋友们这几天一直在张罗聚会的事。</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>CHI-20260825-007</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>铺张浪费</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>pū zhāng làng fěi</t>
+        </is>
+      </c>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>사치하고 낭비하다</t>
+        </is>
+      </c>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>学校食堂提倡勤俭节约，坚决反对铺张浪费。</t>
+        </is>
+      </c>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>举办婚礼虽然重要，但也没必要为了面子而铺张浪费。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>CHI-20260825-008</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>叹为观止</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>tàn wéi guān zhǐ</t>
+        </is>
+      </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>절정에 달해 탄성을 지르다, 감탄을 금치 못하다</t>
+        </is>
+      </c>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>看到这次AI中考系统的精准度，所有在场的校长都叹为观止。</t>
+        </is>
+      </c>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>这部科幻电影的特效和视觉画面简直令人叹为观止。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>CHI-20260825-009</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>告状</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1001" t="inlineStr">
+        <is>
+          <t>gào zhuàng</t>
+        </is>
+      </c>
+      <c r="G1001" t="inlineStr">
+        <is>
+          <t>(윗사람에게 일러바치기 위해) 고자질하다, 고발하다</t>
+        </is>
+      </c>
+      <c r="H1001" t="inlineStr">
+        <is>
+          <t>这两个小朋友在体验活动中一吵架就跑去跟班主任告状。</t>
+        </is>
+      </c>
+      <c r="I1001" t="inlineStr">
+        <is>
+          <t>他在工作中遇到一点小矛盾就去向老板告状，让同事们很不满。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>CHI-20260825-010</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>执着</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1002" t="inlineStr">
+        <is>
+          <t>zhí zhuó</t>
+        </is>
+      </c>
+      <c r="G1002" t="inlineStr">
+        <is>
+          <t>집착하다, 고집하다, 끝까지 고수하다</t>
+        </is>
+      </c>
+      <c r="H1002" t="inlineStr">
+        <is>
+          <t>哪怕高考失利，这位姑娘依然对军校梦想非常执着，复读一年终于成功。</t>
+        </is>
+      </c>
+      <c r="I1002" t="inlineStr">
+        <is>
+          <t>他对科研工作的执着和追求，赢得了所有同事的尊重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>CHI-20260825-011</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>塞车</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1003" t="inlineStr">
+        <is>
+          <t>sāi chē</t>
+        </is>
+      </c>
+      <c r="G1003" t="inlineStr">
+        <is>
+          <t>교통 체증이 발생하다, 차가 막히다</t>
+        </is>
+      </c>
+      <c r="H1003" t="inlineStr">
+        <is>
+          <t>今天开学第一天，校门口严重塞车，交警都在现场疏导。</t>
+        </is>
+      </c>
+      <c r="I1003" t="inlineStr">
+        <is>
+          <t>为了避免上班塞车，我每天早上都提早半小时出门。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>CHI-20260825-012</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>顺路</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1004" t="inlineStr">
+        <is>
+          <t>shùn lù</t>
+        </is>
+      </c>
+      <c r="G1004" t="inlineStr">
+        <is>
+          <t>가는 길이다, 동선이 겹치다</t>
+        </is>
+      </c>
+      <c r="H1004" t="inlineStr">
+        <is>
+          <t>既然我们都去市北实验学校，那我顺路开车带你一起去吧。</t>
+        </is>
+      </c>
+      <c r="I1004" t="inlineStr">
+        <is>
+          <t>没关系，我正好顺路去一趟超市，可以帮你把快递顺便拿回来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>CHI-20260825-013</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>见利忘义</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1005" t="inlineStr">
+        <is>
+          <t>jiàn lì wàng yì</t>
+        </is>
+      </c>
+      <c r="G1005" t="inlineStr">
+        <is>
+          <t>눈앞의 이익을 보고 신의를 저버리다</t>
+        </is>
+      </c>
+      <c r="H1005" t="inlineStr">
+        <is>
+          <t>在商业谈判中，最害怕遇到那些见利忘义、临时变卦的合作伙伴。</t>
+        </is>
+      </c>
+      <c r="I1005" t="inlineStr">
+        <is>
+          <t>做人一定要讲信用，绝不能做出见利忘义的事来伤害朋友。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>CHI-20260825-014</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>见多识广</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1006" t="inlineStr">
+        <is>
+          <t>jiàn duō shí guǎng</t>
+        </is>
+      </c>
+      <c r="G1006" t="inlineStr">
+        <is>
+          <t>보고 들은 것이 많아 식견이 넓다</t>
+        </is>
+      </c>
+      <c r="H1006" t="inlineStr">
+        <is>
+          <t>这位走访过多个国家的校长见多识广，办学理念也非常先进。</t>
+        </is>
+      </c>
+      <c r="I1006" t="inlineStr">
+        <is>
+          <t>张教授是一位见多识广的学者，在多个学术领域都非常有发言权。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>CHI-20260825-015</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>树立</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1007" t="inlineStr">
+        <is>
+          <t>shù lì</t>
+        </is>
+      </c>
+      <c r="G1007" t="inlineStr">
+        <is>
+          <t>(관념, 모범, 믿음 등을) 올바르게 세우다, 확립하다</t>
+        </is>
+      </c>
+      <c r="H1007" t="inlineStr">
+        <is>
+          <t>班主任要在学生面前树立良好的榜样，引导他们健康成长。</t>
+        </is>
+      </c>
+      <c r="I1007" t="inlineStr">
+        <is>
+          <t>学校教育的重要目标之一，就是帮助学生树立正确的人生观和价值观。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-26 | 1016/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1007"/>
+  <dimension ref="A1:I1017"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47745,6 +47745,476 @@
         </is>
       </c>
     </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>CHI-20260826-001</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>死记硬背</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1008" t="inlineStr">
+        <is>
+          <t>sǐ jì yìng bèi</t>
+        </is>
+      </c>
+      <c r="G1008" t="inlineStr">
+        <is>
+          <t>이해 없이 무작정 외우다, 주입식으로 암기하다</t>
+        </is>
+      </c>
+      <c r="H1008" t="inlineStr">
+        <is>
+          <t>虽然快开学了，但学习不能只靠死记硬背，得掌握方法。</t>
+        </is>
+      </c>
+      <c r="I1008" t="inlineStr">
+        <is>
+          <t>学习语言不能靠死记硬背，要多在实际场景中运用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>CHI-20260826-002</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>死磕</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1009" t="inlineStr">
+        <is>
+          <t>sǐ kē</t>
+        </is>
+      </c>
+      <c r="G1009" t="inlineStr">
+        <is>
+          <t>끝까지 매달리다, 악바리처럼 버티다, 끝장을 보다</t>
+        </is>
+      </c>
+      <c r="H1009" t="inlineStr">
+        <is>
+          <t>那个患有视觉障碍的孩子，凭着一股和命运死磕的劲头，硬是考了721的高分。</t>
+        </is>
+      </c>
+      <c r="I1009" t="inlineStr">
+        <is>
+          <t>遇到技术难题不要轻易放弃，多跟它死磕几次总能找到解决方案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>CHI-20260826-003</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>不甘示弱</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1010" t="inlineStr">
+        <is>
+          <t>bù gān shì ruò</t>
+        </is>
+      </c>
+      <c r="G1010" t="inlineStr">
+        <is>
+          <t>지기 싫어하다, 뒤처지기 싫어 맞서다</t>
+        </is>
+      </c>
+      <c r="H1010" t="inlineStr">
+        <is>
+          <t>别的学校都升级了校服，我们学校也不甘示弱，决定给全体学生免费发校服。</t>
+        </is>
+      </c>
+      <c r="I1010" t="inlineStr">
+        <is>
+          <t>看到竞争对手推出了新功能，我们研发部门也不甘示弱，立刻开始了产品升级。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>CHI-20260826-004</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>磨洋工</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1011" t="inlineStr">
+        <is>
+          <t>mó yáng gōng</t>
+        </is>
+      </c>
+      <c r="G1011" t="inlineStr">
+        <is>
+          <t>시간을 때우다, 빈둥거리며 늑장 부리다</t>
+        </is>
+      </c>
+      <c r="H1011" t="inlineStr">
+        <is>
+          <t>施工单位必须抓紧时间推进环保工程，绝不能在工地上磨洋工。</t>
+        </is>
+      </c>
+      <c r="I1011" t="inlineStr">
+        <is>
+          <t>如果你总是磨洋工，不仅会拖慢整个团队的进度，还会影响考核。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>CHI-20260826-005</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>有分寸</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>yǒu fēn cun</t>
+        </is>
+      </c>
+      <c r="G1012" t="inlineStr">
+        <is>
+          <t>선을 잘 지키다, 말과 행동이 적절하다, 분별력이 있다</t>
+        </is>
+      </c>
+      <c r="H1012" t="inlineStr">
+        <is>
+          <t>虽然高校允许带宠物，但“铲屎官”们也要有分寸，不能影响正常的教学秩序。</t>
+        </is>
+      </c>
+      <c r="I1012" t="inlineStr">
+        <is>
+          <t>他说话很有分寸，既表达了自己的态度，又没有让对方感到尴尬。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>CHI-20260826-006</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>乱套</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>luàn tào</t>
+        </is>
+      </c>
+      <c r="G1013" t="inlineStr">
+        <is>
+          <t>뒤죽박죽이 되다, 엉망진창이 되다, 질서가 깨지다</t>
+        </is>
+      </c>
+      <c r="H1013" t="inlineStr">
+        <is>
+          <t>开学季如果不提前做好交通规划，校门口的路肯定会乱套。</t>
+        </is>
+      </c>
+      <c r="I1013" t="inlineStr">
+        <is>
+          <t>主管请假了三天，结果部门的工作没人协调，全乱套了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>CHI-20260826-007</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>有眼光</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1014" t="inlineStr">
+        <is>
+          <t>yǒu yǎn guāng</t>
+        </is>
+      </c>
+      <c r="G1014" t="inlineStr">
+        <is>
+          <t>안목이 있다, 보는 눈이 있다</t>
+        </is>
+      </c>
+      <c r="H1014" t="inlineStr">
+        <is>
+          <t>千年舟能够把普通的板材做成奢侈品，不得不说他们的设计师很有眼光。</t>
+        </is>
+      </c>
+      <c r="I1014" t="inlineStr">
+        <is>
+          <t>经理一眼就挑中了这个创意，真是太有眼光了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>CHI-20260826-008</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>使绊子</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1015" t="inlineStr">
+        <is>
+          <t>shǐ bàn zi</t>
+        </is>
+      </c>
+      <c r="G1015" t="inlineStr">
+        <is>
+          <t>딴지를 걸다, 훼방을 놓다, 발을 걸어 넘어뜨리다</t>
+        </is>
+      </c>
+      <c r="H1015" t="inlineStr">
+        <is>
+          <t>同行竞争应该光明正大，绝不能在背后给竞争对手使绊子。</t>
+        </is>
+      </c>
+      <c r="I1015" t="inlineStr">
+        <is>
+          <t>他总担心别人超越自己，经常在工作中暗地里给同事使绊子。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>CHI-20260826-009</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>交学费</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1016" t="inlineStr">
+        <is>
+          <t>jiāo xué fèi</t>
+        </is>
+      </c>
+      <c r="G1016" t="inlineStr">
+        <is>
+          <t>(실패나 실수를 통해) 경험치를 쌓다, 쓴맛을 보며 배우다</t>
+        </is>
+      </c>
+      <c r="H1016" t="inlineStr">
+        <is>
+          <t>刚开始搞高原生态环保实践时，由于经验不足，确实交了不少学费。</t>
+        </is>
+      </c>
+      <c r="I1016" t="inlineStr">
+        <is>
+          <t>刚入行的人免不了要交点学费，跌倒了再爬起来就是。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>CHI-20260826-010</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>下不为例</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1017" t="inlineStr">
+        <is>
+          <t>xià bù wéi lì</t>
+        </is>
+      </c>
+      <c r="G1017" t="inlineStr">
+        <is>
+          <t>이번 한 번만 봐주다, 다음에는 예외가 없다</t>
+        </is>
+      </c>
+      <c r="H1017" t="inlineStr">
+        <is>
+          <t>这次允许你带宠物来学校是特殊情况，但下不为例，以后必须按规章办。</t>
+        </is>
+      </c>
+      <c r="I1017" t="inlineStr">
+        <is>
+          <t>鉴于你是初犯，这次迟到就先口头警告，下不为例。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-27 | 1025/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1017"/>
+  <dimension ref="A1:I1026"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48215,6 +48215,429 @@
         </is>
       </c>
     </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>CHI-20260827-001</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>没门</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>méi mén</t>
+        </is>
+      </c>
+      <c r="G1018" t="inlineStr">
+        <is>
+          <t>절대 안 된다, 가망 없다</t>
+        </is>
+      </c>
+      <c r="H1018" t="inlineStr">
+        <is>
+          <t>상대방의 무리한 부탁을 단호하게 거절할 때</t>
+        </is>
+      </c>
+      <c r="I1018" t="inlineStr">
+        <is>
+          <t>想让我帮你作弊？没门！</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>CHI-20260827-002</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>钻牛角尖</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1019" t="inlineStr">
+        <is>
+          <t>zuān niú jiǎo jiān</t>
+        </is>
+      </c>
+      <c r="G1019" t="inlineStr">
+        <is>
+          <t>고집스럽게 한우물만 파다, 융통성 없이 생각하다</t>
+        </is>
+      </c>
+      <c r="H1019" t="inlineStr">
+        <is>
+          <t>이미 해결하기 어려운 문제에 지나치게 매달리거나 시야가 좁아졌을 때</t>
+        </is>
+      </c>
+      <c r="I1019" t="inlineStr">
+        <is>
+          <t>别总是钻牛角尖，换个角度想问题可能就简单多了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>CHI-20260827-003</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>看走眼</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1020" t="inlineStr">
+        <is>
+          <t>kàn zǒu yǎn</t>
+        </is>
+      </c>
+      <c r="G1020" t="inlineStr">
+        <is>
+          <t>사람이나 물건을 잘못 보다(판단하다)</t>
+        </is>
+      </c>
+      <c r="H1020" t="inlineStr">
+        <is>
+          <t>상대의 본질을 잘못 파악했거나 가짜를 진짜로 착각했을 때</t>
+        </is>
+      </c>
+      <c r="I1020" t="inlineStr">
+        <is>
+          <t>哎呀，这次是我看走眼了，没想到他竟然是这种人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>CHI-20260827-004</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>摆架子</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1021" t="inlineStr">
+        <is>
+          <t>bǎi jià zi</t>
+        </is>
+      </c>
+      <c r="G1021" t="inlineStr">
+        <is>
+          <t>거드름 피우다, 폼 잡다</t>
+        </is>
+      </c>
+      <c r="H1021" t="inlineStr">
+        <is>
+          <t>지위가 높은 사람이 권위적인 태도를 보이거나 우쭐댈 때</t>
+        </is>
+      </c>
+      <c r="I1021" t="inlineStr">
+        <is>
+          <t>大家都是平等的同事，你在这儿摆什么架子啊？</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>CHI-20260827-005</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>没头没脑</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1022" t="inlineStr">
+        <is>
+          <t>méi tóu méi nǎo</t>
+        </is>
+      </c>
+      <c r="G1022" t="inlineStr">
+        <is>
+          <t>앞뒤 없이, 무턱대고, 영문 모르고</t>
+        </is>
+      </c>
+      <c r="H1022" t="inlineStr">
+        <is>
+          <t>상대방의 행동이나 말이 맥락 없이 갑자기 튀어나올 때</t>
+        </is>
+      </c>
+      <c r="I1022" t="inlineStr">
+        <is>
+          <t>他没头没脑地冲进来，大声喊了一句就跑了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>CHI-20260827-006</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>冒尖</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1023" t="inlineStr">
+        <is>
+          <t>mào jiān</t>
+        </is>
+      </c>
+      <c r="G1023" t="inlineStr">
+        <is>
+          <t>두드러지다, 뛰어나다</t>
+        </is>
+      </c>
+      <c r="H1023" t="inlineStr">
+        <is>
+          <t>在全行业的竞争中，这家企业开始逐渐冒尖。</t>
+        </is>
+      </c>
+      <c r="I1023" t="inlineStr">
+        <is>
+          <t>小王在这一批新人里很冒尖，非常有潜力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>CHI-20260827-007</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>开小灶</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1024" t="inlineStr">
+        <is>
+          <t>kāi xiǎo zào</t>
+        </is>
+      </c>
+      <c r="G1024" t="inlineStr">
+        <is>
+          <t>별도로 특별 교육/배려를 해주다</t>
+        </is>
+      </c>
+      <c r="H1024" t="inlineStr">
+        <is>
+          <t>老师决定给基础薄弱的学生开小灶。</t>
+        </is>
+      </c>
+      <c r="I1024" t="inlineStr">
+        <is>
+          <t>组长说今晚留下来给我开小灶，指导项目代码。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>CHI-20260827-008</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>吹毛求疵</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1025" t="inlineStr">
+        <is>
+          <t>chuī máo qiú cī</t>
+        </is>
+      </c>
+      <c r="G1025" t="inlineStr">
+        <is>
+          <t>결점을 찾아내려 애쓰다, 지나치게 까다롭게 굴다</t>
+        </is>
+      </c>
+      <c r="H1025" t="inlineStr">
+        <is>
+          <t>工作上认真可以，但不能总是吹毛求疵。</t>
+        </is>
+      </c>
+      <c r="I1025" t="inlineStr">
+        <is>
+          <t>他总是喜欢在这些细枝末节上吹毛求疵。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>CHI-20260827-009</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>大换血</t>
+        </is>
+      </c>
+      <c r="E1026" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1026" t="inlineStr">
+        <is>
+          <t>dà huàn xuè</t>
+        </is>
+      </c>
+      <c r="G1026" t="inlineStr">
+        <is>
+          <t>대대적인 인적 쇄신(물갈이)</t>
+        </is>
+      </c>
+      <c r="H1026" t="inlineStr">
+        <is>
+          <t>公司管理层进行了大换血，引进了许多人才。</t>
+        </is>
+      </c>
+      <c r="I1026" t="inlineStr">
+        <is>
+          <t>部门业绩太差，领导决定进行大换血。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-28 | 1036/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1026"/>
+  <dimension ref="A1:I1037"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48638,6 +48638,523 @@
         </is>
       </c>
     </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>CHI-20260828-001</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>智商税</t>
+        </is>
+      </c>
+      <c r="E1027" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1027" t="inlineStr">
+        <is>
+          <t>zhì shāng shuì</t>
+        </is>
+      </c>
+      <c r="G1027" t="inlineStr">
+        <is>
+          <t>호갱 행위로 인한 낭비 (어리석은 소비)</t>
+        </is>
+      </c>
+      <c r="H1027" t="inlineStr">
+        <is>
+          <t>开学经济太火爆，大家买装备时要理性，不要交了‘智商税’。</t>
+        </is>
+      </c>
+      <c r="I1027" t="inlineStr">
+        <is>
+          <t>这牌子的护肤品根本没效果，纯粹是交智商税。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>CHI-20260828-002</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>擦边球</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1028" t="inlineStr">
+        <is>
+          <t>cā biān qiú</t>
+        </is>
+      </c>
+      <c r="G1028" t="inlineStr">
+        <is>
+          <t>법이나 규제의 사각지대를 이용하다, 아슬아슬하게 통과하다</t>
+        </is>
+      </c>
+      <c r="H1028" t="inlineStr">
+        <is>
+          <t>两姐妹的高考分数仅差3分，刚好擦边球考上了同一所大学。</t>
+        </is>
+      </c>
+      <c r="I1028" t="inlineStr">
+        <is>
+          <t>有些小广告一直在打法律的擦边球，必须严厉打击。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>CHI-20260828-003</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>起作用</t>
+        </is>
+      </c>
+      <c r="E1029" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1029" t="inlineStr">
+        <is>
+          <t>qǐ zuò yòng</t>
+        </is>
+      </c>
+      <c r="G1029" t="inlineStr">
+        <is>
+          <t>효과가 나타나다, 역할을 하다</t>
+        </is>
+      </c>
+      <c r="H1029" t="inlineStr">
+        <is>
+          <t>发改委一连串稳投资的政策终于起作用了，市场正在逐步回暖。</t>
+        </is>
+      </c>
+      <c r="I1029" t="inlineStr">
+        <is>
+          <t>感冒药开始起作用了，我觉得好多了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>CHI-20260828-004</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>丢三落四</t>
+        </is>
+      </c>
+      <c r="E1030" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1030" t="inlineStr">
+        <is>
+          <t>diū sān là sì</t>
+        </is>
+      </c>
+      <c r="G1030" t="inlineStr">
+        <is>
+          <t>덤벙대다, 물건을 잘 잃어버리거나 잘 흘리고 다니다</t>
+        </is>
+      </c>
+      <c r="H1030" t="inlineStr">
+        <is>
+          <t>开学前一晚，别丢三落四的，把文具和书本都准备齐。</t>
+        </is>
+      </c>
+      <c r="I1030" t="inlineStr">
+        <is>
+          <t>你总是丢三落四的，出门前再检查一下钱包和钥匙。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>CHI-20260828-005</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>吃力</t>
+        </is>
+      </c>
+      <c r="E1031" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1031" t="inlineStr">
+        <is>
+          <t>chī lì</t>
+        </is>
+      </c>
+      <c r="G1031" t="inlineStr">
+        <is>
+          <t>힘에 부치다, 힘겹다, 고전하다</t>
+        </is>
+      </c>
+      <c r="H1031" t="inlineStr">
+        <is>
+          <t>如果高考调整不提前适应，有些考生在考场上可能会觉得吃力。</t>
+        </is>
+      </c>
+      <c r="I1031" t="inlineStr">
+        <is>
+          <t>我的英语底子薄，学起专业课来有些吃力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>CHI-20260828-006</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>劳逸结合</t>
+        </is>
+      </c>
+      <c r="E1032" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1032" t="inlineStr">
+        <is>
+          <t>láo yì jié hé</t>
+        </is>
+      </c>
+      <c r="G1032" t="inlineStr">
+        <is>
+          <t>일과 휴식을 적절히 병행하다</t>
+        </is>
+      </c>
+      <c r="H1032" t="inlineStr">
+        <is>
+          <t>面对开学后的繁重学业，学生们应该学会劳逸结合，科学调适身心。</t>
+        </is>
+      </c>
+      <c r="I1032" t="inlineStr">
+        <is>
+          <t>在准备高考的过程中，一定要注意劳逸结合，保持良好的心态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>CHI-20260828-007</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>人云亦云</t>
+        </is>
+      </c>
+      <c r="E1033" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1033" t="inlineStr">
+        <is>
+          <t>rén yún yì yún</t>
+        </is>
+      </c>
+      <c r="G1033" t="inlineStr">
+        <is>
+          <t>줏대 없이 남의 말을 맹목적으로 따르다</t>
+        </is>
+      </c>
+      <c r="H1033" t="inlineStr">
+        <is>
+          <t>面对所谓的“开学经济”热潮，家长要保持理性，不能人云亦云。</t>
+        </is>
+      </c>
+      <c r="I1033" t="inlineStr">
+        <is>
+          <t>选大学专业时要根据自己的兴趣，不要人云亦云地去报热门专业。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>CHI-20260828-008</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>三分钟热度</t>
+        </is>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1034" t="inlineStr">
+        <is>
+          <t>sān fēn zhōng rè dù</t>
+        </is>
+      </c>
+      <c r="G1034" t="inlineStr">
+        <is>
+          <t>작심삼일, 쉽게 끓고 쉽게 식는 열정</t>
+        </is>
+      </c>
+      <c r="H1034" t="inlineStr">
+        <is>
+          <t>很多人为了应对“开学综合征”而制定计划，但往往只是三分钟热度。</t>
+        </is>
+      </c>
+      <c r="I1034" t="inlineStr">
+        <is>
+          <t>学习乐器需要持之以恒，如果只有三分钟热度是学不好的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>CHI-20260828-009</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>说到底</t>
+        </is>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>shuō dào dǐ</t>
+        </is>
+      </c>
+      <c r="G1035" t="inlineStr">
+        <is>
+          <t>결국은, 근본적으로 말하자면</t>
+        </is>
+      </c>
+      <c r="H1035" t="inlineStr">
+        <is>
+          <t>环保实践说到底是为了人与自然的和谐相处，不能只做表面文章。</t>
+        </is>
+      </c>
+      <c r="I1035" t="inlineStr">
+        <is>
+          <t>产品的包装设计得再好看，说到底还是要看它的质量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>CHI-20260828-010</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>不相上下</t>
+        </is>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>bù xiāng shàng xià</t>
+        </is>
+      </c>
+      <c r="G1036" t="inlineStr">
+        <is>
+          <t>우열을 가릴 수 없다, 막상막하이다</t>
+        </is>
+      </c>
+      <c r="H1036" t="inlineStr">
+        <is>
+          <t>这对双胞胎姐妹的高考成绩不相上下，最终同时被同一所大学录取。</t>
+        </is>
+      </c>
+      <c r="I1036" t="inlineStr">
+        <is>
+          <t>这两家全屋定制品牌的产品质量不相上下，很难做出选择。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>CHI-20260828-011</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>当耳边风</t>
+        </is>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>dāng ěr biān fēng</t>
+        </is>
+      </c>
+      <c r="G1037" t="inlineStr">
+        <is>
+          <t>한 귀로 듣고 한 귀로 흘리다, 귓등으로 듣다</t>
+        </is>
+      </c>
+      <c r="H1037" t="inlineStr">
+        <is>
+          <t>家长反复强调开学要理性消费，但他总是当耳边风，买了许多无用的装备。</t>
+        </is>
+      </c>
+      <c r="I1037" t="inlineStr">
+        <is>
+          <t>老师叮嘱过很多次考试注意事项，你可别当耳边风。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-08-31 | 1041/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1037"/>
+  <dimension ref="A1:I1042"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49155,6 +49155,241 @@
         </is>
       </c>
     </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>CHI-20260831-001</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>下海</t>
+        </is>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>xià hǎi</t>
+        </is>
+      </c>
+      <c r="G1038" t="inlineStr">
+        <is>
+          <t>상업/사업에 뛰어들다 (안정된 공직이나 직장을 그만두고 자영업이나 비즈니스를 시작하다)</t>
+        </is>
+      </c>
+      <c r="H1038" t="inlineStr">
+        <is>
+          <t>정부 기관인 발개위(发改委)나 지자체 공무원들이 안정적인 철밥통을 내려놓고 민간 인공지능(AI) 스타트업이나 기업으로 이직하는 추세를 뜻합니다.</t>
+        </is>
+      </c>
+      <c r="I1038" t="inlineStr">
+        <is>
+          <t>九十年代初，很多体制内的干部选择下海经商。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>CHI-20260831-002</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>打官腔</t>
+        </is>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>dǎ guān qiāng</t>
+        </is>
+      </c>
+      <c r="G1039" t="inlineStr">
+        <is>
+          <t>원론적인 답변만 하다, 관료적인 말투로 책임을 회피하다</t>
+        </is>
+      </c>
+      <c r="H1039" t="inlineStr">
+        <is>
+          <t>정부 부처 대변인이나 관공서 담당자가 민원인의 구체적이고 곤란한 질문에 대해 원론적이고 형식적인 답변만 늘어놓는 답답한 행동을 비판할 때 씁니다.</t>
+        </is>
+      </c>
+      <c r="I1039" t="inlineStr">
+        <is>
+          <t>请直接回答我的问题，不要总是和我们打官腔。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>CHI-20260831-003</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>收心</t>
+        </is>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>shōu xīn</t>
+        </is>
+      </c>
+      <c r="G1040" t="inlineStr">
+        <is>
+          <t>휴가나 방학 후 들뜬 마음을 가다듬고 일이나 공부에 다시 집중하다</t>
+        </is>
+      </c>
+      <c r="H1040" t="inlineStr">
+        <is>
+          <t>开学了，大家应该把注意力放回学习上。</t>
+        </is>
+      </c>
+      <c r="I1040" t="inlineStr">
+        <is>
+          <t>暑假已经结束了，你得赶紧收心，准备迎接新学期的挑战。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>CHI-20260831-004</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>破天荒</t>
+        </is>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>pò tiān huāng</t>
+        </is>
+      </c>
+      <c r="G1041" t="inlineStr">
+        <is>
+          <t>난생처음으로, 전대미문으로 (이전에는 없었던 놀라운 일이 발생하다)</t>
+        </is>
+      </c>
+      <c r="H1041" t="inlineStr">
+        <is>
+          <t>这个从不迟到的人今天竟然迟到了。</t>
+        </is>
+      </c>
+      <c r="I1041" t="inlineStr">
+        <is>
+          <t>那个平时不爱说话的学霸，今天竟然破天荒地在台上演讲了一个小时。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>CHI-20260831-005</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>心服口服</t>
+        </is>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>xīn fú kǒu fú</t>
+        </is>
+      </c>
+      <c r="G1042" t="inlineStr">
+        <is>
+          <t>마음으로나 말로 모두 진정으로 굴복하여 승복하다</t>
+        </is>
+      </c>
+      <c r="H1042" t="inlineStr">
+        <is>
+          <t>他的专业水平确实让人佩服。</t>
+        </is>
+      </c>
+      <c r="I1042" t="inlineStr">
+        <is>
+          <t>他用无可辩驳的数据和极其专业的分析，让在场的专家们心服口服。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-01 | 1049/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1042"/>
+  <dimension ref="A1:I1050"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49390,6 +49390,382 @@
         </is>
       </c>
     </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>CHI-20260901-001</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>说白了</t>
+        </is>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>shuō bái le</t>
+        </is>
+      </c>
+      <c r="G1043" t="inlineStr">
+        <is>
+          <t>솔직히 말해서, 쉽게 말해, 요컨대</t>
+        </is>
+      </c>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>예능 촬영팀이 해변에 쓰레기를 이틀이나 방치한 사건은, 솔직히 말해서 업계의 환경 보호 의식 결여가 원인입니다.</t>
+        </is>
+      </c>
+      <c r="I1043" t="inlineStr">
+        <is>
+          <t>这件事说白了，就是由于双方沟通不畅造成的误会。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>CHI-20260901-002</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>撂挑子</t>
+        </is>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>liào tiāo zi</t>
+        </is>
+      </c>
+      <c r="G1044" t="inlineStr">
+        <is>
+          <t>책임을 내팽개치다, 도중에 일을 그만두다</t>
+        </is>
+      </c>
+      <c r="H1044" t="inlineStr">
+        <is>
+          <t>환경 훼손에 대해 끝까지 엄중한 책임을 묻겠다고 압박하자, 해당 사업 책임자가 부담감을 견디지 못하고 도중에 일을 팽개쳐 버릴지 우려됩니다.</t>
+        </is>
+      </c>
+      <c r="I1044" t="inlineStr">
+        <is>
+          <t>遇到一点挫折就撂挑子不干，怎么能成大事呢？</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>CHI-20260901-003</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>不走寻常路</t>
+        </is>
+      </c>
+      <c r="E1045" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1045" t="inlineStr">
+        <is>
+          <t>bù zǒu xún cháng lù</t>
+        </is>
+      </c>
+      <c r="G1045" t="inlineStr">
+        <is>
+          <t>독창적인 길을 걷다, 뻔한 형식을 탈피하다</t>
+        </is>
+      </c>
+      <c r="H1045" t="inlineStr">
+        <is>
+          <t>이 학교는 지루한 개학식 대신 경찰차 에스코트와 로봇 시연회 등 뻔한 형식을 탈피한 행사로 큰 찬사를 받았습니다.</t>
+        </is>
+      </c>
+      <c r="I1045" t="inlineStr">
+        <is>
+          <t>现在的年轻创业者都喜欢不走寻常路，勇于挑战传统行业。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>CHI-20260901-004</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>唱独角戏</t>
+        </is>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1046" t="inlineStr">
+        <is>
+          <t>chàng dú jiǎo xì</t>
+        </is>
+      </c>
+      <c r="G1046" t="inlineStr">
+        <is>
+          <t>혼자 북 치고 장구 치다, 혼자 힘겹게 일을 처리하다</t>
+        </is>
+      </c>
+      <c r="H1046" t="inlineStr">
+        <is>
+          <t>학생들의 안전한 건강 환경 조성은 교육지원청 혼자서 원맨쇼를 하듯 해결할 수 없으며, 유관 부처 모두의 긴밀한 공조가 필수적입니다.</t>
+        </is>
+      </c>
+      <c r="I1046" t="inlineStr">
+        <is>
+          <t>跨部门的合作方案需要大家齐心协力，单靠我们部门唱独角戏是完成不了的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>CHI-20260901-005</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>缩水</t>
+        </is>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1047" t="inlineStr">
+        <is>
+          <t>suō shuǐ</t>
+        </is>
+      </c>
+      <c r="G1047" t="inlineStr">
+        <is>
+          <t>규모가 줄어들다, 가치나 혜택이 대폭 축소되다</t>
+        </is>
+      </c>
+      <c r="H1047" t="inlineStr">
+        <is>
+          <t>연속 4년 동안 신입생 학부모들에게 무료 숙박을 제공하던 대학 복지 혜택이 학교 예산 삭감으로 인해 크게 축소되었습니다.</t>
+        </is>
+      </c>
+      <c r="I1047" t="inlineStr">
+        <is>
+          <t>随着通货膨胀，老百姓手里现金的实际购买力也在无形中缩水。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>CHI-20260901-006</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>见微知著</t>
+        </is>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1048" t="inlineStr">
+        <is>
+          <t>jiàn wēi zhī zhù</t>
+        </is>
+      </c>
+      <c r="G1048" t="inlineStr">
+        <is>
+          <t>작은 징조를 보고 전체를 알다</t>
+        </is>
+      </c>
+      <c r="H1048" t="inlineStr">
+        <is>
+          <t>优秀的管理者能够见微知著，在小毛病扩大前就将其解决。</t>
+        </is>
+      </c>
+      <c r="I1048" t="inlineStr">
+        <is>
+          <t>从一个人的细节表现中，往往能见微知著，看出他的真实素养。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>CHI-20260901-007</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>门外汉</t>
+        </is>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1049" t="inlineStr">
+        <is>
+          <t>mén wài hàn</t>
+        </is>
+      </c>
+      <c r="G1049" t="inlineStr">
+        <is>
+          <t>비전문가, 아웃사이더</t>
+        </is>
+      </c>
+      <c r="H1049" t="inlineStr">
+        <is>
+          <t>对于人工智能和编程技术，我完全是一个门外汉，得从零学起。</t>
+        </is>
+      </c>
+      <c r="I1049" t="inlineStr">
+        <is>
+          <t>在医学这个高度专业的领域里，普通老百姓大多都是门外汉。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>CHI-20260901-008</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>侃侃而谈</t>
+        </is>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1050" t="inlineStr">
+        <is>
+          <t>kǎn kǎn ér tán</t>
+        </is>
+      </c>
+      <c r="G1050" t="inlineStr">
+        <is>
+          <t>당당하고 거침없이 이야기하다</t>
+        </is>
+      </c>
+      <c r="H1050" t="inlineStr">
+        <is>
+          <t>在开学第一课的讲台上，这位人工智能专家面对台下的学生侃侃而谈。</t>
+        </is>
+      </c>
+      <c r="I1050" t="inlineStr">
+        <is>
+          <t>平时不爱说话的他，只要一提到足球，就能跟人侃侃而谈好几个小时。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-02 | 1056/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1050"/>
+  <dimension ref="A1:I1057"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49766,6 +49766,335 @@
         </is>
       </c>
     </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>CHI-20260902-001</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>走俏</t>
+        </is>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1051" t="inlineStr">
+        <is>
+          <t>zǒu qiào</t>
+        </is>
+      </c>
+      <c r="G1051" t="inlineStr">
+        <is>
+          <t>날개 돋친 듯 팔리다, 시장에서 큰 인기를 끌다</t>
+        </is>
+      </c>
+      <c r="H1051" t="inlineStr">
+        <is>
+          <t>今年开学季，兼具智能和环保概念的文具在市场上非常走俏。</t>
+        </is>
+      </c>
+      <c r="I1051" t="inlineStr">
+        <is>
+          <t>这款主打便携和低卡的新款咖啡，一上市就在年轻白领中迅速走俏。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>CHI-20260902-002</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>唱高调</t>
+        </is>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1052" t="inlineStr">
+        <is>
+          <t>chàng gāo diào</t>
+        </is>
+      </c>
+      <c r="G1052" t="inlineStr">
+        <is>
+          <t>실천 없이 번지르르한 소리만 늘어놓다</t>
+        </is>
+      </c>
+      <c r="H1052" t="inlineStr">
+        <is>
+          <t>解决气候危机需要各国拿出真金白银的行动，光在会议上唱高调根本没用。</t>
+        </is>
+      </c>
+      <c r="I1052" t="inlineStr">
+        <is>
+          <t>管理团队不能只坐在办公室里唱高调，得真正深入一线了解基层员工的痛点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>CHI-20260902-003</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>压轴</t>
+        </is>
+      </c>
+      <c r="E1053" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1053" t="inlineStr">
+        <is>
+          <t>yā zhòu</t>
+        </is>
+      </c>
+      <c r="G1053" t="inlineStr">
+        <is>
+          <t>대미를 장식하다, 마지막 하이라이트로 등장하다</t>
+        </is>
+      </c>
+      <c r="H1053" t="inlineStr">
+        <is>
+          <t>在开学典礼的最后环节，优秀毕业生的励学演讲成了全场的压轴戏。</t>
+        </is>
+      </c>
+      <c r="I1053" t="inlineStr">
+        <is>
+          <t>今晚的文创新品发布会上，那款耗时三年研发的智能旗舰款压轴登场。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>CHI-20260902-004</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>打底</t>
+        </is>
+      </c>
+      <c r="E1054" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1054" t="inlineStr">
+        <is>
+          <t>dǎ dǐ</t>
+        </is>
+      </c>
+      <c r="G1054" t="inlineStr">
+        <is>
+          <t>기본기를 탄탄히 다져두다, 최소한의 안전판을 깔아두다</t>
+        </is>
+      </c>
+      <c r="H1054" t="inlineStr">
+        <is>
+          <t>备考各种专业证书，最关键的还是把基础理论知识彻底打好底。</t>
+        </is>
+      </c>
+      <c r="I1054" t="inlineStr">
+        <is>
+          <t>先拿下一个保底的常规客户打底，我们接下来就可以放手去搏高利润大单了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>CHI-20260902-005</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>请教</t>
+        </is>
+      </c>
+      <c r="E1055" t="inlineStr">
+        <is>
+          <t>동사</t>
+        </is>
+      </c>
+      <c r="F1055" t="inlineStr">
+        <is>
+          <t>qǐng jiào</t>
+        </is>
+      </c>
+      <c r="G1055" t="inlineStr">
+        <is>
+          <t>(예의를 갖추어 전문가나 윗사람에게) 자문하다, 조언을 구하다</t>
+        </is>
+      </c>
+      <c r="H1055" t="inlineStr">
+        <is>
+          <t>青年干部要经常深入一线，虚心向实践经验丰富的老前辈请教。</t>
+        </is>
+      </c>
+      <c r="I1055" t="inlineStr">
+        <is>
+          <t>关于跨境税务合规的具体细节，我们需要尽快向专业的涉外律师请教。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>CHI-20260902-006</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>打圆场</t>
+        </is>
+      </c>
+      <c r="E1056" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1056" t="inlineStr">
+        <is>
+          <t>dǎ yuán chǎng</t>
+        </is>
+      </c>
+      <c r="G1056" t="inlineStr">
+        <is>
+          <t>분위기를 누그러뜨리다, 중재하여 싸움을 말리다</t>
+        </is>
+      </c>
+      <c r="H1056" t="inlineStr">
+        <is>
+          <t>看到会议室气氛有点僵，李主管赶紧站出来打了个圆场。</t>
+        </is>
+      </c>
+      <c r="I1056" t="inlineStr">
+        <is>
+          <t>他们两个争得面红耳赤，幸好有同事在旁边打圆场才没吵起来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>CHI-20260902-007</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>开后门</t>
+        </is>
+      </c>
+      <c r="E1057" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1057" t="inlineStr">
+        <is>
+          <t>kāi hòu mén</t>
+        </is>
+      </c>
+      <c r="G1057" t="inlineStr">
+        <is>
+          <t>뒷구멍을 봐주다, 부정한 방법으로 편의나 특혜를 제공하다</t>
+        </is>
+      </c>
+      <c r="H1057" t="inlineStr">
+        <is>
+          <t>这次招考全程公开透明，绝不允许任何人托关系开后门。</t>
+        </is>
+      </c>
+      <c r="I1057" t="inlineStr">
+        <is>
+          <t>公司招聘有严格的面试流程，谁也不可能靠开后门进来。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-03 | 1065/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1057"/>
+  <dimension ref="A1:I1066"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50095,6 +50095,429 @@
         </is>
       </c>
     </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>CHI-20260903-001</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>擦屁股</t>
+        </is>
+      </c>
+      <c r="E1058" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1058" t="inlineStr">
+        <is>
+          <t>cā pì gu</t>
+        </is>
+      </c>
+      <c r="G1058" t="inlineStr">
+        <is>
+          <t>남이 저지른 잘못을 뒤치다꺼리하다, 뒷감당을 하다</t>
+        </is>
+      </c>
+      <c r="H1058" t="inlineStr">
+        <is>
+          <t>촬영 팀이 어지럽히고 떠난 촬영장을 다른 실무진이 긴급 투입되어 밤새 치우며 불평하는 상황</t>
+        </is>
+      </c>
+      <c r="I1058" t="inlineStr">
+        <is>
+          <t>他每次做事情都丢三落四的，最后总要别人跟在后面帮他擦屁股。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>CHI-20260903-002</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>唱对台戏</t>
+        </is>
+      </c>
+      <c r="E1059" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1059" t="inlineStr">
+        <is>
+          <t>chàng duì tái xì</t>
+        </is>
+      </c>
+      <c r="G1059" t="inlineStr">
+        <is>
+          <t>상대방과 대립 구도를 세워 맞서 싸우다</t>
+        </is>
+      </c>
+      <c r="H1059" t="inlineStr">
+        <is>
+          <t>해외 경쟁 브랜드가 내놓은 친환경 기준에 맞불을 놓아 자신들만의 독자적인 표준을 제시하며 갈등하는 글로벌 시장 상황</t>
+        </is>
+      </c>
+      <c r="I1059" t="inlineStr">
+        <is>
+          <t>不管我提出什么样的改革建议，他总要跟我唱对台戏，真是不可理喻。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>CHI-20260903-003</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>吃瓜群众</t>
+        </is>
+      </c>
+      <c r="E1060" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1060" t="inlineStr">
+        <is>
+          <t>chī guā qún zhòng</t>
+        </is>
+      </c>
+      <c r="G1060" t="inlineStr">
+        <is>
+          <t>사건의 제3자 구경꾼, 관심 있게 관전하는 대중</t>
+        </is>
+      </c>
+      <c r="H1060" t="inlineStr">
+        <is>
+          <t>온라인상에서 프로그램 제작사와 지역 주민 간의 쓰레기 배출 책임 공방전이 벌어지자, 관전 중인 네티즌들을 지칭하는 상황</t>
+        </is>
+      </c>
+      <c r="I1060" t="inlineStr">
+        <is>
+          <t>这起明星绯闻案的真相还没水落石出，我们吃瓜群众还是先别急着站队。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>CHI-20260903-004</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>说了算</t>
+        </is>
+      </c>
+      <c r="E1061" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1061" t="inlineStr">
+        <is>
+          <t>shuō le suàn</t>
+        </is>
+      </c>
+      <c r="G1061" t="inlineStr">
+        <is>
+          <t>최종 결정권이 있다, 마음대로 좌지우지할 수 있다</t>
+        </is>
+      </c>
+      <c r="H1061" t="inlineStr">
+        <is>
+          <t>협상 테이블에서 실무진의 의견보다는 결국 최종 결재권자인 팀장의 한마디가 상황을 결정짓는 직장 현실</t>
+        </is>
+      </c>
+      <c r="I1061" t="inlineStr">
+        <is>
+          <t>在技术架构的选择上，应该让总工程师说了算，其他人不要瞎指挥。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>CHI-20260903-005</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>有底气</t>
+        </is>
+      </c>
+      <c r="E1062" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1062" t="inlineStr">
+        <is>
+          <t>yǒu dǐ qì</t>
+        </is>
+      </c>
+      <c r="G1062" t="inlineStr">
+        <is>
+          <t>자신감이 있다, (배경이나 실력이 든든하여) 당당하다</t>
+        </is>
+      </c>
+      <c r="H1062" t="inlineStr">
+        <is>
+          <t>拥有技术积累和资金支持，让我们在面对激烈的市场竞争时更有底气。</t>
+        </is>
+      </c>
+      <c r="I1062" t="inlineStr">
+        <is>
+          <t>只有做足了功课，上台发言时才会非常有底气。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>CHI-20260903-006</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>组合拳</t>
+        </is>
+      </c>
+      <c r="E1063" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1063" t="inlineStr">
+        <is>
+          <t>zǔ hé quán</t>
+        </is>
+      </c>
+      <c r="G1063" t="inlineStr">
+        <is>
+          <t>(정책이나 비즈니스 등에서) 다각적인 연쇄 조치, 종합적인 해결책</t>
+        </is>
+      </c>
+      <c r="H1063" t="inlineStr">
+        <is>
+          <t>政府出台了一套支持小微企业的“组合拳”，帮助企业渡过难关。</t>
+        </is>
+      </c>
+      <c r="I1063" t="inlineStr">
+        <is>
+          <t>面对这次公关危机，公司必须打出一套“组合拳”来挽回声誉。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>CHI-20260903-007</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>拉家常</t>
+        </is>
+      </c>
+      <c r="E1064" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1064" t="inlineStr">
+        <is>
+          <t>lā jiā cháng</t>
+        </is>
+      </c>
+      <c r="G1064" t="inlineStr">
+        <is>
+          <t>사소한 일상 이야기를 나누다, 잡담을 하다</t>
+        </is>
+      </c>
+      <c r="H1064" t="inlineStr">
+        <is>
+          <t>社区工作人员深入居民家中拉家常，了解大家面临的实际困难。</t>
+        </is>
+      </c>
+      <c r="I1064" t="inlineStr">
+        <is>
+          <t>领导在茶歇时间主动跟我们拉家常，气氛一下子变得轻松了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>CHI-20260903-008</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>干巴巴</t>
+        </is>
+      </c>
+      <c r="E1065" t="inlineStr">
+        <is>
+          <t>구어</t>
+        </is>
+      </c>
+      <c r="F1065" t="inlineStr">
+        <is>
+          <t>gān bā bā</t>
+        </is>
+      </c>
+      <c r="G1065" t="inlineStr">
+        <is>
+          <t>(내용, 글, 말이) 메마르고 딱딱하다, 영양가가 없다, 지루하다</t>
+        </is>
+      </c>
+      <c r="H1065" t="inlineStr">
+        <is>
+          <t>如果文物展览只是干巴巴的文字介绍，很难吸引年轻人的关注。</t>
+        </is>
+      </c>
+      <c r="I1065" t="inlineStr">
+        <is>
+          <t>你的汇报太干巴巴了，应该多加一些图表和具体案例来丰富内容。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>CHI-20260903-009</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>不声不响</t>
+        </is>
+      </c>
+      <c r="E1066" t="inlineStr">
+        <is>
+          <t>성어</t>
+        </is>
+      </c>
+      <c r="F1066" t="inlineStr">
+        <is>
+          <t>bù shēng bù xiǎng</t>
+        </is>
+      </c>
+      <c r="G1066" t="inlineStr">
+        <is>
+          <t>아무 소리도 내지 않다, 말없이 조용히 (행동)하다</t>
+        </is>
+      </c>
+      <c r="H1066" t="inlineStr">
+        <is>
+          <t>他平时话不多，却在这次高考中不声不响地考了全校第一名。</t>
+        </is>
+      </c>
+      <c r="I1066" t="inlineStr">
+        <is>
+          <t>谁也没想到，他竟然不声不响地把这么大的环保项目谈下来了。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Daily Chinese DB update: 2026-09-04 | 1072/2000 expressions
</commit_message>
<xml_diff>
--- a/data/01_Database/chinese_expressions_db.xlsx
+++ b/data/01_Database/chinese_expressions_db.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1066"/>
+  <dimension ref="A1:I1073"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50518,6 +50518,335 @@
         </is>
       </c>
     </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>CHI-20260904-001</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>一哄而上</t>
+        </is>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1067" t="inlineStr">
+        <is>
+          <t>yī hòng ér shàng</t>
+        </is>
+      </c>
+      <c r="G1067" t="inlineStr">
+        <is>
+          <t>한꺼번에 우르르 몰려들다, 졸속으로 덤벼들다</t>
+        </is>
+      </c>
+      <c r="H1067" t="inlineStr">
+        <is>
+          <t>친환경 트렌드에 맞춰 준비 없이 뛰어드는 패션 업계들의 실태.</t>
+        </is>
+      </c>
+      <c r="I1067" t="inlineStr">
+        <is>
+          <t>大家都一哄而上去做新能源，结果造成了产能过剩。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>CHI-20260904-002</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>人情世故</t>
+        </is>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1068" t="inlineStr">
+        <is>
+          <t>rén qíng shì gù</t>
+        </is>
+      </c>
+      <c r="G1068" t="inlineStr">
+        <is>
+          <t>세상 살아가는 이치, 처세술, 대인관계 도리</t>
+        </is>
+      </c>
+      <c r="H1068" t="inlineStr">
+        <is>
+          <t>직장 초년생이 국유기업이나 공직 사회에 들어와 배우게 되는 처세술.</t>
+        </is>
+      </c>
+      <c r="I1068" t="inlineStr">
+        <is>
+          <t>在职场上，除了工作能力，懂点人情世故也很重要。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>CHI-20260904-003</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>临门一脚</t>
+        </is>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1069" t="inlineStr">
+        <is>
+          <t>lín mén yī jiǎo</t>
+        </is>
+      </c>
+      <c r="G1069" t="inlineStr">
+        <is>
+          <t>마지막 결정적인 한 방, 화룡점정</t>
+        </is>
+      </c>
+      <c r="H1069" t="inlineStr">
+        <is>
+          <t>가오카오 합격 발표 직전이나 대규모 환경 정화 사업 완공 직전의 마지막 단계.</t>
+        </is>
+      </c>
+      <c r="I1069" t="inlineStr">
+        <is>
+          <t>项目策划得很完美，现在就差临门一脚的资金支持了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>CHI-20260904-004</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>说闲话</t>
+        </is>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>이합사</t>
+        </is>
+      </c>
+      <c r="F1070" t="inlineStr">
+        <is>
+          <t>shuō xiánhuà</t>
+        </is>
+      </c>
+      <c r="G1070" t="inlineStr">
+        <is>
+          <t>뒷공론을 하다, 쓸데없는 소리를 하다</t>
+        </is>
+      </c>
+      <c r="H1070" t="inlineStr">
+        <is>
+          <t>我们与其他国家的正常合作，不应受到第三方的无端干涉和说闲话。</t>
+        </is>
+      </c>
+      <c r="I1070" t="inlineStr">
+        <is>
+          <t>只要我们行得正、做得端，就不怕别人在背后说闲话。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>CHI-20260904-005</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>见风使舵</t>
+        </is>
+      </c>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1071" t="inlineStr">
+        <is>
+          <t>jiàn fēng shǐ duò</t>
+        </is>
+      </c>
+      <c r="G1071" t="inlineStr">
+        <is>
+          <t>상황에 따라 이리저리 태도를 바꾸다, 기회주의적으로 처신하다</t>
+        </is>
+      </c>
+      <c r="H1071" t="inlineStr">
+        <is>
+          <t>有些快时尚品牌见风使舵，打着环保的旗号制定有利于自己的标准。</t>
+        </is>
+      </c>
+      <c r="I1071" t="inlineStr">
+        <is>
+          <t>他这个人总是见风使舵，谁有权势他就往谁那边靠。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>CHI-20260904-006</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>急功近利</t>
+        </is>
+      </c>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1072" t="inlineStr">
+        <is>
+          <t>jí gōng jìn lì</t>
+        </is>
+      </c>
+      <c r="G1072" t="inlineStr">
+        <is>
+          <t>눈앞의 이익과 성과에만 급급하다</t>
+        </is>
+      </c>
+      <c r="H1072" t="inlineStr">
+        <is>
+          <t>城市规划和环保建设需要长远目光，绝不能急功近利。</t>
+        </is>
+      </c>
+      <c r="I1072" t="inlineStr">
+        <is>
+          <t>教育孩子要慢慢引导，急功近利往往会适得其反。</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>CHI-20260904-007</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Scraped_News</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>各抒己见</t>
+        </is>
+      </c>
+      <c r="E1073" t="inlineStr">
+        <is>
+          <t>관용구</t>
+        </is>
+      </c>
+      <c r="F1073" t="inlineStr">
+        <is>
+          <t>gè shū jǐ jiàn</t>
+        </is>
+      </c>
+      <c r="G1073" t="inlineStr">
+        <is>
+          <t>각자의 의견을 마음껏 개진하다</t>
+        </is>
+      </c>
+      <c r="H1073" t="inlineStr">
+        <is>
+          <t>在人大代表建议征集会上，大家就如何提升绿化环境各抒己见。</t>
+        </is>
+      </c>
+      <c r="I1073" t="inlineStr">
+        <is>
+          <t>在今天的研讨会上，中外专家们就环保技术合作各抒己见。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>